<commit_message>
fix(classeurs): réparer la feuille « Résultats détaillés »
La feuille contenait 127 cellules fantômes rangées dans une autre ligne,
restes d'une ancienne mise en page (K37 = E34*10+F34, L38 = OR(K35=31)…),
qui portaient les formules partagées maîtresses de plusieurs colonnes.
OnlyOffice résolvait les formules depuis ces fantômes : #VALEUR! dans la
synthèse (ligne Management, urgentes, priorités avec action).

- 70 fantômes en double supprimés, 57 replacés dans leur ligne
- formules partagées remplacées par des formules simples, cellules triées
- toutes les lignes de données suivent la formule canonique (0 écart)

Effets : 0 erreur au recalcul (contre 2 : K37, K38), 32/32 cibles comptées
quand la grille est remplie (31 avant), priorités des cibles 5.1 à 5.5
correctes. Synthèse de l'exemple inchangée. Variantes régénérées.

Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/INR_GPC_ONR Exemple.xlsx
+++ b/INR_GPC_ONR Exemple.xlsx
@@ -31230,8 +31230,7 @@
         <v>Intervention urgente</v>
       </c>
       <c r="K5" s="227" t="n">
-        <f t="shared" ref="K5:K9" si="1">IF(ISBLANK('ONR 1'!K7),"",'ONR 1'!K7)</f>
-        <v>31</v>
+        <f>IF(ISBLANK('ONR 1'!K7),"",'ONR 1'!K7)</f>
       </c>
       <c r="L5" s="227" t="b">
         <f>IF(ISBLANK('ONR 1'!L7),"",'ONR 1'!L7)</f>
@@ -31262,20 +31261,16 @@
         <v>0</v>
       </c>
       <c r="S5" s="228" t="str">
-        <f t="shared" ref="S5:S9" si="2">IF(ISBLANK('ONR 1'!S7),"",'ONR 1'!S7)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!S7),"",'ONR 1'!S7)</f>
       </c>
       <c r="T5" s="226" t="n">
-        <f t="shared" ref="T5:T9" si="3">IF(ISBLANK('ONR 1'!T7),"",'ONR 1'!T7)</f>
-        <v>6</v>
+        <f>IF(ISBLANK('ONR 1'!T7),"",'ONR 1'!T7)</f>
       </c>
       <c r="U5" s="227" t="n">
-        <f t="shared" ref="U5:U9" si="4">IF(ISBLANK('ONR 1'!U7),"",'ONR 1'!U7)</f>
-        <v>63</v>
+        <f>IF(ISBLANK('ONR 1'!U7),"",'ONR 1'!U7)</f>
       </c>
       <c r="V5" s="229" t="str">
-        <f t="shared" ref="V5:V11" si="5">IF(ISBLANK('ONR 1'!G7),"",'ONR 1'!G7)</f>
-        <v>L’équipe Achats retient le prix d’achat comme seul critère de choix. Elle ne demande pas d’analyse du cycle de vie (ACV) aux fournisseurs dans les appels d’offres.</v>
+        <f>IF(ISBLANK('ONR 1'!G7),"",'ONR 1'!G7)</f>
       </c>
       <c r="W5" s="203" t="str">
         <f>IF(ISBLANK('ONR 1'!V7),"",'ONR 1'!V7)</f>
@@ -31285,46 +31280,34 @@
         <f>IF(ISBLANK('ONR 1'!W7),"",'ONR 1'!W7)</f>
       </c>
       <c r="Y5" s="230" t="str">
-        <f t="shared" ref="Y5:Y11" si="6">IF(ISBLANK('ONR 1'!I7),"",'ONR 1'!I7)</f>
-        <v>Point fort : la direction des achats souhaite adopter des pratiques plus durables.
-Point faible : l’équipe connaît peu les labels environnementaux des équipements informatiques.</v>
+        <f>IF(ISBLANK('ONR 1'!I7),"",'ONR 1'!I7)</f>
       </c>
       <c r="Z5" s="230" t="str">
-        <f t="shared" ref="Z5:Z11" si="7">IF(ISBLANK('ONR 1'!D7),"",'ONR 1'!D7)</f>
-        <v>Avantages possibles : réduire les émissions de gaz à effet de serre de l’organisation et se préparer aux futures règles environnementales.
-Risque : payer plus cher à l’achat certains équipements conçus pour limiter leurs effets sur l’environnement.</v>
+        <f>IF(ISBLANK('ONR 1'!D7),"",'ONR 1'!D7)</f>
       </c>
       <c r="AE5" s="206" t="n">
-        <f t="shared" ref="AE5:AE11" si="8">IF(ISNUMBER(T5),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T5),0,1)</f>
       </c>
       <c r="AF5" s="206" t="n">
-        <f t="shared" ref="AF5:AL11" si="9">IF(L5=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(L5=TRUE,1,0)</f>
       </c>
       <c r="AG5" s="206" t="n">
-        <f t="shared" si="9">IF(M5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M5=TRUE,1,0)</f>
       </c>
       <c r="AH5" s="206" t="n">
-        <f t="shared" si="9">IF(N5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N5=TRUE,1,0)</f>
       </c>
       <c r="AI5" s="206" t="n">
-        <f t="shared" si="9">IF(O5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O5=TRUE,1,0)</f>
       </c>
       <c r="AJ5" s="206" t="n">
-        <f t="shared" si="9">IF(P5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P5=TRUE,1,0)</f>
       </c>
       <c r="AK5" s="206" t="n">
-        <f t="shared" si="9">IF(Q5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q5=TRUE,1,0)</f>
       </c>
       <c r="AL5" s="206" t="n">
-        <f t="shared" si="9">IF(R5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R5=TRUE,1,0)</f>
       </c>
       <c r="AM5" t="n">
         <f>IF(LEN(TRIM(W5))&gt;0,1,0)</f>
@@ -31367,56 +31350,43 @@
 Point faible : certains utilisateurs demandent du matériel neuf pour son apparence.</v>
       </c>
       <c r="J6" s="232" t="str">
-        <f t="shared" ref="J6:J9" si="10">IF(ISBLANK('ONR 1'!J8),"",'ONR 1'!J8)</f>
-        <v>Intervention à moyen terme</v>
+        <f>IF(ISBLANK('ONR 1'!J8),"",'ONR 1'!J8)</f>
       </c>
       <c r="K6" s="233" t="n">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K8),"",'ONR 1'!K8)</f>
-        <v>33</v>
+        <f>IF(ISBLANK('ONR 1'!K8),"",'ONR 1'!K8)</f>
       </c>
       <c r="L6" s="233" t="b">
-        <f t="shared" ref="L6:L9" si="11">IF(ISBLANK('ONR 1'!L8),"",'ONR 1'!L8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L8),"",'ONR 1'!L8)</f>
       </c>
       <c r="M6" s="233" t="b">
-        <f t="shared" ref="M6:M9" si="12">IF(ISBLANK('ONR 1'!M8),"",'ONR 1'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M8),"",'ONR 1'!M8)</f>
       </c>
       <c r="N6" s="233" t="b">
-        <f t="shared" ref="N6:N9" si="13">IF(ISBLANK('ONR 1'!N8),"",'ONR 1'!N8)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!N8),"",'ONR 1'!N8)</f>
       </c>
       <c r="O6" s="233" t="b">
-        <f t="shared" ref="O6:O9" si="14">IF(ISBLANK('ONR 1'!O8),"",'ONR 1'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O8),"",'ONR 1'!O8)</f>
       </c>
       <c r="P6" s="233" t="b">
-        <f t="shared" ref="P6:P9" si="15">IF(ISBLANK('ONR 1'!P8),"",'ONR 1'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P8),"",'ONR 1'!P8)</f>
       </c>
       <c r="Q6" s="233" t="b">
-        <f t="shared" ref="Q6:Q9" si="16">IF(ISBLANK('ONR 1'!Q8),"",'ONR 1'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q8),"",'ONR 1'!Q8)</f>
       </c>
       <c r="R6" s="233" t="b">
-        <f t="shared" ref="R6:R9" si="17">IF(ISBLANK('ONR 1'!R8),"",'ONR 1'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R8),"",'ONR 1'!R8)</f>
       </c>
       <c r="S6" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S8),"",'ONR 1'!S8)</f>
-        <v>Intervention à moyen terme</v>
+        <f>IF(ISBLANK('ONR 1'!S8),"",'ONR 1'!S8)</f>
       </c>
       <c r="T6" s="232" t="n">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T8),"",'ONR 1'!T8)</f>
-        <v>4</v>
+        <f>IF(ISBLANK('ONR 1'!T8),"",'ONR 1'!T8)</f>
       </c>
       <c r="U6" s="233" t="n">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U8),"",'ONR 1'!U8)</f>
-        <v>42</v>
+        <f>IF(ISBLANK('ONR 1'!U8),"",'ONR 1'!U8)</f>
       </c>
       <c r="V6" s="235" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G8),"",'ONR 1'!G8)</f>
-        <v>L’organisation a porté la durée de renouvellement des ordinateurs portables de trois à quatre ans l’année dernière. Elle dispose d’un contrat de maintenance.</v>
+        <f>IF(ISBLANK('ONR 1'!G8),"",'ONR 1'!G8)</f>
       </c>
       <c r="W6" s="235" t="str">
         <f>IF(ISBLANK('ONR 1'!V8),"",'ONR 1'!V8)</f>
@@ -31426,45 +31396,34 @@
         <f>IF(ISBLANK('ONR 1'!W8),"",'ONR 1'!W8)</f>
       </c>
       <c r="Y6" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I8),"",'ONR 1'!I8)</f>
-        <v>Point fort : l’équipe technique peut réparer les équipements en interne.
-Point faible : certains utilisateurs demandent du matériel neuf pour son apparence.</v>
+        <f>IF(ISBLANK('ONR 1'!I8),"",'ONR 1'!I8)</f>
       </c>
       <c r="Z6" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D8),"",'ONR 1'!D8)</f>
-        <v>Avantages possibles : réduire les dépenses d’achat de matériel et les déchets d’équipements électriques et électroniques (DEEE).</v>
+        <f>IF(ISBLANK('ONR 1'!D8),"",'ONR 1'!D8)</f>
       </c>
       <c r="AE6" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T6),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T6),0,1)</f>
       </c>
       <c r="AF6" s="206" t="n">
-        <f t="shared" si="9">IF(L6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L6=TRUE,1,0)</f>
       </c>
       <c r="AG6" s="206" t="n">
-        <f t="shared" si="9">IF(M6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M6=TRUE,1,0)</f>
       </c>
       <c r="AH6" s="206" t="n">
-        <f t="shared" si="9">IF(N6=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(N6=TRUE,1,0)</f>
       </c>
       <c r="AI6" s="206" t="n">
-        <f t="shared" si="9">IF(O6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O6=TRUE,1,0)</f>
       </c>
       <c r="AJ6" s="206" t="n">
-        <f t="shared" si="9">IF(P6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P6=TRUE,1,0)</f>
       </c>
       <c r="AK6" s="206" t="n">
-        <f t="shared" si="9">IF(Q6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q6=TRUE,1,0)</f>
       </c>
       <c r="AL6" s="206" t="n">
-        <f t="shared" si="9">IF(R6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R6=TRUE,1,0)</f>
       </c>
       <c r="AM6" t="n">
         <f>IF(LEN(TRIM(W6))&gt;0,1,0)</f>
@@ -31508,56 +31467,43 @@
 Points faibles : ils connaissent peu les guides pour concevoir des services numériques moins polluants, comme le RGESN. Ils savent peu comment relier leurs projets aux ODD.</v>
       </c>
       <c r="J7" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J9),"",'ONR 1'!J9)</f>
-        <v>Intervention prioritaire</v>
+        <f>IF(ISBLANK('ONR 1'!J9),"",'ONR 1'!J9)</f>
       </c>
       <c r="K7" s="233" t="n">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K9),"",'ONR 1'!K9)</f>
-        <v>32</v>
+        <f>IF(ISBLANK('ONR 1'!K9),"",'ONR 1'!K9)</f>
       </c>
       <c r="L7" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L9),"",'ONR 1'!L9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L9),"",'ONR 1'!L9)</f>
       </c>
       <c r="M7" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M9),"",'ONR 1'!M9)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!M9),"",'ONR 1'!M9)</f>
       </c>
       <c r="N7" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N9),"",'ONR 1'!N9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N9),"",'ONR 1'!N9)</f>
       </c>
       <c r="O7" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O9),"",'ONR 1'!O9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O9),"",'ONR 1'!O9)</f>
       </c>
       <c r="P7" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P9),"",'ONR 1'!P9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P9),"",'ONR 1'!P9)</f>
       </c>
       <c r="Q7" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q9),"",'ONR 1'!Q9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q9),"",'ONR 1'!Q9)</f>
       </c>
       <c r="R7" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R9),"",'ONR 1'!R9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R9),"",'ONR 1'!R9)</f>
       </c>
       <c r="S7" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S9),"",'ONR 1'!S9)</f>
-        <v>Intervention prioritaire</v>
+        <f>IF(ISBLANK('ONR 1'!S9),"",'ONR 1'!S9)</f>
       </c>
       <c r="T7" s="232" t="n">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T9),"",'ONR 1'!T9)</f>
-        <v>5</v>
+        <f>IF(ISBLANK('ONR 1'!T9),"",'ONR 1'!T9)</f>
       </c>
       <c r="U7" s="233" t="n">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U9),"",'ONR 1'!U9)</f>
-        <v>52</v>
+        <f>IF(ISBLANK('ONR 1'!U9),"",'ONR 1'!U9)</f>
       </c>
       <c r="V7" s="235" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G9),"",'ONR 1'!G9)</f>
-        <v>Les équipes valident les nouveaux services et sites web selon des critères fonctionnels, graphiques et financiers. Elles ne mesurent ni le poids des pages ni l’impact environnemental du code.</v>
+        <f>IF(ISBLANK('ONR 1'!G9),"",'ONR 1'!G9)</f>
       </c>
       <c r="W7" s="142" t="str">
         <f>IF(ISBLANK('ONR 1'!V9),"",'ONR 1'!V9)</f>
@@ -31569,46 +31515,34 @@
         <f>IF(ISBLANK('ONR 1'!W9),"",'ONR 1'!W9)</f>
       </c>
       <c r="Y7" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I9),"",'ONR 1'!I9)</f>
-        <v>Point fort : les développeurs et les chefs de produit s’intéressent aux effets de leurs activités sur la société et l’environnement.
-Points faibles : ils connaissent peu les guides pour concevoir des services numériques moins polluants, comme le RGESN. Ils savent peu comment relier leurs projets aux ODD.</v>
+        <f>IF(ISBLANK('ONR 1'!I9),"",'ONR 1'!I9)</f>
       </c>
       <c r="Z7" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D9),"",'ONR 1'!D9)</f>
-        <v>Avantages possibles : réduire les effets des services sur l’environnement dès leur conception, faciliter leur utilisation et contribuer aux Objectifs de développement durable (ODD).
-Risques : accumuler des problèmes techniques non résolus ou créer des logiciels trop gourmands en ressources, qui obligent à remplacer le matériel plus tôt.</v>
+        <f>IF(ISBLANK('ONR 1'!D9),"",'ONR 1'!D9)</f>
       </c>
       <c r="AE7" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T7),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T7),0,1)</f>
       </c>
       <c r="AF7" s="206" t="n">
-        <f t="shared" si="9">IF(L7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L7=TRUE,1,0)</f>
       </c>
       <c r="AG7" s="206" t="n">
-        <f t="shared" si="9">IF(M7=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(M7=TRUE,1,0)</f>
       </c>
       <c r="AH7" s="206" t="n">
-        <f t="shared" si="9">IF(N7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N7=TRUE,1,0)</f>
       </c>
       <c r="AI7" s="206" t="n">
-        <f t="shared" si="9">IF(O7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O7=TRUE,1,0)</f>
       </c>
       <c r="AJ7" s="206" t="n">
-        <f t="shared" si="9">IF(P7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P7=TRUE,1,0)</f>
       </c>
       <c r="AK7" s="206" t="n">
-        <f t="shared" si="9">IF(Q7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q7=TRUE,1,0)</f>
       </c>
       <c r="AL7" s="206" t="n">
-        <f t="shared" si="9">IF(R7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R7=TRUE,1,0)</f>
       </c>
       <c r="AM7" t="n">
         <f>IF(LEN(TRIM(W7))&gt;0,1,0)</f>
@@ -31644,50 +31578,43 @@
         <f>IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
       </c>
       <c r="J8" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J10),"",'ONR 1'!J10)</f>
+        <f>IF(ISBLANK('ONR 1'!J10),"",'ONR 1'!J10)</f>
       </c>
       <c r="K8" s="233" t="str">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K10),"",'ONR 1'!K10)</f>
+        <f>IF(ISBLANK('ONR 1'!K10),"",'ONR 1'!K10)</f>
       </c>
       <c r="L8" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L10),"",'ONR 1'!L10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L10),"",'ONR 1'!L10)</f>
       </c>
       <c r="M8" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M10),"",'ONR 1'!M10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M10),"",'ONR 1'!M10)</f>
       </c>
       <c r="N8" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N10),"",'ONR 1'!N10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N10),"",'ONR 1'!N10)</f>
       </c>
       <c r="O8" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O10),"",'ONR 1'!O10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O10),"",'ONR 1'!O10)</f>
       </c>
       <c r="P8" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P10),"",'ONR 1'!P10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P10),"",'ONR 1'!P10)</f>
       </c>
       <c r="Q8" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q10),"",'ONR 1'!Q10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q10),"",'ONR 1'!Q10)</f>
       </c>
       <c r="R8" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R10),"",'ONR 1'!R10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R10),"",'ONR 1'!R10)</f>
       </c>
       <c r="S8" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S10),"",'ONR 1'!S10)</f>
+        <f>IF(ISBLANK('ONR 1'!S10),"",'ONR 1'!S10)</f>
       </c>
       <c r="T8" s="232" t="str">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T10),"",'ONR 1'!T10)</f>
+        <f>IF(ISBLANK('ONR 1'!T10),"",'ONR 1'!T10)</f>
       </c>
       <c r="U8" s="233" t="str">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U10),"",'ONR 1'!U10)</f>
+        <f>IF(ISBLANK('ONR 1'!U10),"",'ONR 1'!U10)</f>
       </c>
       <c r="V8" s="239" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G10),"",'ONR 1'!G10)</f>
+        <f>IF(ISBLANK('ONR 1'!G10),"",'ONR 1'!G10)</f>
       </c>
       <c r="W8" s="210" t="str">
         <f>IF(ISBLANK('ONR 1'!V10),"",'ONR 1'!V10)</f>
@@ -31696,42 +31623,34 @@
         <f>IF(ISBLANK('ONR 1'!W10),"",'ONR 1'!W10)</f>
       </c>
       <c r="Y8" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
+        <f>IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
       </c>
       <c r="Z8" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D10),"",'ONR 1'!D10)</f>
+        <f>IF(ISBLANK('ONR 1'!D10),"",'ONR 1'!D10)</f>
       </c>
       <c r="AE8" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T8),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T8),0,1)</f>
       </c>
       <c r="AF8" s="206" t="n">
-        <f t="shared" si="9">IF(L8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L8=TRUE,1,0)</f>
       </c>
       <c r="AG8" s="206" t="n">
-        <f t="shared" si="9">IF(M8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M8=TRUE,1,0)</f>
       </c>
       <c r="AH8" s="206" t="n">
-        <f t="shared" si="9">IF(N8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N8=TRUE,1,0)</f>
       </c>
       <c r="AI8" s="206" t="n">
-        <f t="shared" si="9">IF(O8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O8=TRUE,1,0)</f>
       </c>
       <c r="AJ8" s="206" t="n">
-        <f t="shared" si="9">IF(P8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P8=TRUE,1,0)</f>
       </c>
       <c r="AK8" s="206" t="n">
-        <f t="shared" si="9">IF(Q8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q8=TRUE,1,0)</f>
       </c>
       <c r="AL8" s="206" t="n">
-        <f t="shared" si="9">IF(R8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R8=TRUE,1,0)</f>
       </c>
       <c r="AM8" t="n">
         <f>IF(LEN(TRIM(W8))&gt;0,1,0)</f>
@@ -31767,50 +31686,43 @@
         <f>IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
       </c>
       <c r="J9" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J11),"",'ONR 1'!J11)</f>
+        <f>IF(ISBLANK('ONR 1'!J11),"",'ONR 1'!J11)</f>
       </c>
       <c r="K9" s="233" t="str">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K11),"",'ONR 1'!K11)</f>
+        <f>IF(ISBLANK('ONR 1'!K11),"",'ONR 1'!K11)</f>
       </c>
       <c r="L9" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L11),"",'ONR 1'!L11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L11),"",'ONR 1'!L11)</f>
       </c>
       <c r="M9" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M11),"",'ONR 1'!M11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M11),"",'ONR 1'!M11)</f>
       </c>
       <c r="N9" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N11),"",'ONR 1'!N11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N11),"",'ONR 1'!N11)</f>
       </c>
       <c r="O9" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O11),"",'ONR 1'!O11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O11),"",'ONR 1'!O11)</f>
       </c>
       <c r="P9" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P11),"",'ONR 1'!P11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P11),"",'ONR 1'!P11)</f>
       </c>
       <c r="Q9" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q11),"",'ONR 1'!Q11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q11),"",'ONR 1'!Q11)</f>
       </c>
       <c r="R9" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R11),"",'ONR 1'!R11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R11),"",'ONR 1'!R11)</f>
       </c>
       <c r="S9" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S11),"",'ONR 1'!S11)</f>
+        <f>IF(ISBLANK('ONR 1'!S11),"",'ONR 1'!S11)</f>
       </c>
       <c r="T9" s="232" t="str">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T11),"",'ONR 1'!T11)</f>
+        <f>IF(ISBLANK('ONR 1'!T11),"",'ONR 1'!T11)</f>
       </c>
       <c r="U9" s="233" t="str">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U11),"",'ONR 1'!U11)</f>
+        <f>IF(ISBLANK('ONR 1'!U11),"",'ONR 1'!U11)</f>
       </c>
       <c r="V9" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G11),"",'ONR 1'!G11)</f>
+        <f>IF(ISBLANK('ONR 1'!G11),"",'ONR 1'!G11)</f>
       </c>
       <c r="W9" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V11),"",'ONR 1'!V11)</f>
@@ -31819,42 +31731,34 @@
         <f>IF(ISBLANK('ONR 1'!W11),"",'ONR 1'!W11)</f>
       </c>
       <c r="Y9" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
+        <f>IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
       </c>
       <c r="Z9" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D11),"",'ONR 1'!D11)</f>
+        <f>IF(ISBLANK('ONR 1'!D11),"",'ONR 1'!D11)</f>
       </c>
       <c r="AE9" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T9),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T9),0,1)</f>
       </c>
       <c r="AF9" s="206" t="n">
-        <f t="shared" si="9">IF(L9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L9=TRUE,1,0)</f>
       </c>
       <c r="AG9" s="206" t="n">
-        <f t="shared" si="9">IF(M9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M9=TRUE,1,0)</f>
       </c>
       <c r="AH9" s="206" t="n">
-        <f t="shared" si="9">IF(N9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N9=TRUE,1,0)</f>
       </c>
       <c r="AI9" s="206" t="n">
-        <f t="shared" si="9">IF(O9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O9=TRUE,1,0)</f>
       </c>
       <c r="AJ9" s="206" t="n">
-        <f t="shared" si="9">IF(P9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P9=TRUE,1,0)</f>
       </c>
       <c r="AK9" s="206" t="n">
-        <f t="shared" si="9">IF(Q9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q9=TRUE,1,0)</f>
       </c>
       <c r="AL9" s="206" t="n">
-        <f t="shared" si="9">IF(R9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R9=TRUE,1,0)</f>
       </c>
       <c r="AM9" t="n">
         <f>IF(LEN(TRIM(W9))&gt;0,1,0)</f>
@@ -31890,50 +31794,43 @@
         <f>IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
       </c>
       <c r="J10" s="232" t="str">
-        <f t="shared" ref="J10:J11" si="18">IF(ISBLANK('ONR 1'!J12),"",'ONR 1'!J12)</f>
+        <f>IF(ISBLANK('ONR 1'!J12),"",'ONR 1'!J12)</f>
       </c>
       <c r="K10" s="233" t="str">
-        <f t="shared" ref="K10:K11" si="19">IF(ISBLANK('ONR 1'!K12),"",'ONR 1'!K12)</f>
+        <f>IF(ISBLANK('ONR 1'!K12),"",'ONR 1'!K12)</f>
       </c>
       <c r="L10" s="233" t="b">
-        <f t="shared" ref="L10:L11" si="20">IF(ISBLANK('ONR 1'!L12),"",'ONR 1'!L12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L12),"",'ONR 1'!L12)</f>
       </c>
       <c r="M10" s="233" t="b">
-        <f t="shared" ref="M10:M11" si="21">IF(ISBLANK('ONR 1'!M12),"",'ONR 1'!M12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M12),"",'ONR 1'!M12)</f>
       </c>
       <c r="N10" s="233" t="b">
-        <f t="shared" ref="N10:N11" si="22">IF(ISBLANK('ONR 1'!N12),"",'ONR 1'!N12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N12),"",'ONR 1'!N12)</f>
       </c>
       <c r="O10" s="233" t="b">
-        <f t="shared" ref="O10:O11" si="23">IF(ISBLANK('ONR 1'!O12),"",'ONR 1'!O12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O12),"",'ONR 1'!O12)</f>
       </c>
       <c r="P10" s="233" t="b">
-        <f t="shared" ref="P10:P11" si="24">IF(ISBLANK('ONR 1'!P12),"",'ONR 1'!P12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P12),"",'ONR 1'!P12)</f>
       </c>
       <c r="Q10" s="233" t="b">
-        <f t="shared" ref="Q10:Q11" si="25">IF(ISBLANK('ONR 1'!Q12),"",'ONR 1'!Q12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q12),"",'ONR 1'!Q12)</f>
       </c>
       <c r="R10" s="233" t="b">
-        <f t="shared" ref="R10:R11" si="26">IF(ISBLANK('ONR 1'!R12),"",'ONR 1'!R12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R12),"",'ONR 1'!R12)</f>
       </c>
       <c r="S10" s="234" t="str">
-        <f t="shared" ref="S10:S11" si="27">IF(ISBLANK('ONR 1'!S12),"",'ONR 1'!S12)</f>
+        <f>IF(ISBLANK('ONR 1'!S12),"",'ONR 1'!S12)</f>
       </c>
       <c r="T10" s="232" t="str">
-        <f t="shared" ref="T10:T11" si="28">IF(ISBLANK('ONR 1'!T12),"",'ONR 1'!T12)</f>
+        <f>IF(ISBLANK('ONR 1'!T12),"",'ONR 1'!T12)</f>
       </c>
       <c r="U10" s="233" t="str">
-        <f t="shared" ref="U10:U11" si="29">IF(ISBLANK('ONR 1'!U12),"",'ONR 1'!U12)</f>
+        <f>IF(ISBLANK('ONR 1'!U12),"",'ONR 1'!U12)</f>
       </c>
       <c r="V10" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G12),"",'ONR 1'!G12)</f>
+        <f>IF(ISBLANK('ONR 1'!G12),"",'ONR 1'!G12)</f>
       </c>
       <c r="W10" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V12),"",'ONR 1'!V12)</f>
@@ -31942,42 +31839,34 @@
         <f>IF(ISBLANK('ONR 1'!W12),"",'ONR 1'!W12)</f>
       </c>
       <c r="Y10" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
+        <f>IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
       </c>
       <c r="Z10" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D12),"",'ONR 1'!D12)</f>
+        <f>IF(ISBLANK('ONR 1'!D12),"",'ONR 1'!D12)</f>
       </c>
       <c r="AE10" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T10),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T10),0,1)</f>
       </c>
       <c r="AF10" s="206" t="n">
-        <f t="shared" si="9">IF(L10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L10=TRUE,1,0)</f>
       </c>
       <c r="AG10" s="206" t="n">
-        <f t="shared" si="9">IF(M10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M10=TRUE,1,0)</f>
       </c>
       <c r="AH10" s="206" t="n">
-        <f t="shared" si="9">IF(N10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N10=TRUE,1,0)</f>
       </c>
       <c r="AI10" s="206" t="n">
-        <f t="shared" si="9">IF(O10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O10=TRUE,1,0)</f>
       </c>
       <c r="AJ10" s="206" t="n">
-        <f t="shared" si="9">IF(P10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P10=TRUE,1,0)</f>
       </c>
       <c r="AK10" s="206" t="n">
-        <f t="shared" si="9">IF(Q10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q10=TRUE,1,0)</f>
       </c>
       <c r="AL10" s="206" t="n">
-        <f t="shared" si="9">IF(R10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R10=TRUE,1,0)</f>
       </c>
       <c r="AM10" t="n">
         <f>IF(LEN(TRIM(W10))&gt;0,1,0)</f>
@@ -32021,56 +31910,43 @@
 Points faibles : elle connaît peu les méthodes pour mesurer et réduire la consommation de l’IA. Elle manque aussi de recul pour savoir quand l’IA est utile.</v>
       </c>
       <c r="J11" s="232" t="str">
-        <f t="shared" si="18">IF(ISBLANK('ONR 1'!J13),"",'ONR 1'!J13)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!J13),"",'ONR 1'!J13)</f>
       </c>
       <c r="K11" s="233" t="n">
-        <f t="shared" si="19">IF(ISBLANK('ONR 1'!K13),"",'ONR 1'!K13)</f>
-        <v>31</v>
+        <f>IF(ISBLANK('ONR 1'!K13),"",'ONR 1'!K13)</f>
       </c>
       <c r="L11" s="233" t="b">
-        <f t="shared" si="20">IF(ISBLANK('ONR 1'!L13),"",'ONR 1'!L13)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!L13),"",'ONR 1'!L13)</f>
       </c>
       <c r="M11" s="233" t="b">
-        <f t="shared" si="21">IF(ISBLANK('ONR 1'!M13),"",'ONR 1'!M13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M13),"",'ONR 1'!M13)</f>
       </c>
       <c r="N11" s="233" t="b">
-        <f t="shared" si="22">IF(ISBLANK('ONR 1'!N13),"",'ONR 1'!N13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N13),"",'ONR 1'!N13)</f>
       </c>
       <c r="O11" s="233" t="b">
-        <f t="shared" si="23">IF(ISBLANK('ONR 1'!O13),"",'ONR 1'!O13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O13),"",'ONR 1'!O13)</f>
       </c>
       <c r="P11" s="233" t="b">
-        <f t="shared" si="24">IF(ISBLANK('ONR 1'!P13),"",'ONR 1'!P13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P13),"",'ONR 1'!P13)</f>
       </c>
       <c r="Q11" s="233" t="b">
-        <f t="shared" si="25">IF(ISBLANK('ONR 1'!Q13),"",'ONR 1'!Q13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q13),"",'ONR 1'!Q13)</f>
       </c>
       <c r="R11" s="233" t="b">
-        <f t="shared" si="26">IF(ISBLANK('ONR 1'!R13),"",'ONR 1'!R13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R13),"",'ONR 1'!R13)</f>
       </c>
       <c r="S11" s="234" t="str">
-        <f t="shared" si="27">IF(ISBLANK('ONR 1'!S13),"",'ONR 1'!S13)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!S13),"",'ONR 1'!S13)</f>
       </c>
       <c r="T11" s="232" t="n">
-        <f t="shared" si="28">IF(ISBLANK('ONR 1'!T13),"",'ONR 1'!T13)</f>
-        <v>6</v>
+        <f>IF(ISBLANK('ONR 1'!T13),"",'ONR 1'!T13)</f>
       </c>
       <c r="U11" s="233" t="n">
-        <f t="shared" si="29">IF(ISBLANK('ONR 1'!U13),"",'ONR 1'!U13)</f>
-        <v>62</v>
+        <f>IF(ISBLANK('ONR 1'!U13),"",'ONR 1'!U13)</f>
       </c>
       <c r="V11" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G13),"",'ONR 1'!G13)</f>
-        <v>Les équipes métiers expérimentent plusieurs projets d’IA générative, dont des usages de ChatGPT. Elles ne mesurent pas leur impact énergétique et ne disposent pas de charte pour encadrer les besoins et les usages.</v>
+        <f>IF(ISBLANK('ONR 1'!G13),"",'ONR 1'!G13)</f>
       </c>
       <c r="W11" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V13),"",'ONR 1'!V13)</f>
@@ -32082,46 +31958,34 @@
         <f>IF(ISBLANK('ONR 1'!W13),"",'ONR 1'!W13)</f>
       </c>
       <c r="Y11" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I13),"",'ONR 1'!I13)</f>
-        <v>Point fort : l’équipe chargée des données et de l’informatique dispose de compétences techniques et souhaite explorer ces outils.
-Points faibles : elle connaît peu les méthodes pour mesurer et réduire la consommation de l’IA. Elle manque aussi de recul pour savoir quand l’IA est utile.</v>
+        <f>IF(ISBLANK('ONR 1'!I13),"",'ONR 1'!I13)</f>
       </c>
       <c r="Z11" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D13),"",'ONR 1'!D13)</f>
-        <v>Avantages possibles : maîtriser les coûts du matériel et des services d’IA, et réduire les émissions de gaz à effet de serre liées à leur entraînement et à leur utilisation.
-Risque : utiliser l’IA par effet de mode, sans besoin réel, et consommer davantage de ressources.</v>
+        <f>IF(ISBLANK('ONR 1'!D13),"",'ONR 1'!D13)</f>
       </c>
       <c r="AE11" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T11),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T11),0,1)</f>
       </c>
       <c r="AF11" s="206" t="n">
-        <f t="shared" si="9">IF(L11=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(L11=TRUE,1,0)</f>
       </c>
       <c r="AG11" s="206" t="n">
-        <f t="shared" si="9">IF(M11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M11=TRUE,1,0)</f>
       </c>
       <c r="AH11" s="206" t="n">
-        <f t="shared" si="9">IF(N11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N11=TRUE,1,0)</f>
       </c>
       <c r="AI11" s="206" t="n">
-        <f t="shared" si="9">IF(O11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O11=TRUE,1,0)</f>
       </c>
       <c r="AJ11" s="206" t="n">
-        <f t="shared" si="9">IF(P11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P11=TRUE,1,0)</f>
       </c>
       <c r="AK11" s="206" t="n">
-        <f t="shared" si="9">IF(Q11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q11=TRUE,1,0)</f>
       </c>
       <c r="AL11" s="206" t="n">
-        <f t="shared" si="9">IF(R11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R11=TRUE,1,0)</f>
       </c>
       <c r="AM11" t="n">
         <f>IF(LEN(TRIM(W11))&gt;0,1,0)</f>
@@ -32379,7 +32243,7 @@
         <f>IF(ISBLANK('ONR 2'!J7),"",'ONR 2'!J7)</f>
       </c>
       <c r="K14" s="227" t="str">
-        <f t="shared" ref="K14" si="31">IF(ISBLANK('ONR 2'!K7),"",'ONR 2'!K7)</f>
+        <f>IF(ISBLANK('ONR 2'!K7),"",'ONR 2'!K7)</f>
       </c>
       <c r="L14" s="227" t="b">
         <f>IF(ISBLANK('ONR 2'!L7),"",'ONR 2'!L7)</f>
@@ -32410,13 +32274,13 @@
         <v>0</v>
       </c>
       <c r="S14" s="228" t="str">
-        <f t="shared" ref="S14" si="32">IF(ISBLANK('ONR 2'!S7),"",'ONR 2'!S7)</f>
+        <f>IF(ISBLANK('ONR 2'!S7),"",'ONR 2'!S7)</f>
       </c>
       <c r="T14" s="226" t="str">
-        <f t="shared" ref="T14" si="33">IF(ISBLANK('ONR 2'!T7),"",'ONR 2'!T7)</f>
+        <f>IF(ISBLANK('ONR 2'!T7),"",'ONR 2'!T7)</f>
       </c>
       <c r="U14" s="242" t="str">
-        <f t="shared" ref="U14" si="34">IF(ISBLANK('ONR 2'!U7),"",'ONR 2'!U7)</f>
+        <f>IF(ISBLANK('ONR 2'!U7),"",'ONR 2'!U7)</f>
       </c>
       <c r="V14" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!G7),"",'ONR 2'!G7)</f>
@@ -32438,32 +32302,25 @@
         <v>1</v>
       </c>
       <c r="AF14" s="206" t="n">
-        <f t="shared" ref="AF14:AL17" si="35">IF(L14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L14=TRUE,1,0)</f>
       </c>
       <c r="AG14" s="206" t="n">
-        <f t="shared" si="35">IF(M14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M14=TRUE,1,0)</f>
       </c>
       <c r="AH14" s="206" t="n">
-        <f t="shared" si="35">IF(N14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N14=TRUE,1,0)</f>
       </c>
       <c r="AI14" s="206" t="n">
-        <f t="shared" si="35">IF(O14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O14=TRUE,1,0)</f>
       </c>
       <c r="AJ14" s="206" t="n">
-        <f t="shared" si="35">IF(P14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P14=TRUE,1,0)</f>
       </c>
       <c r="AK14" s="206" t="n">
-        <f t="shared" si="35">IF(Q14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q14=TRUE,1,0)</f>
       </c>
       <c r="AL14" s="206" t="n">
-        <f t="shared" si="35">IF(R14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R14=TRUE,1,0)</f>
       </c>
       <c r="AM14" t="n">
         <f>IF(LEN(TRIM(W14))&gt;0,1,0)</f>
@@ -32499,47 +32356,40 @@
         <f>IF(ISBLANK('ONR 2'!I8),"",'ONR 2'!I8)</f>
       </c>
       <c r="J15" s="218" t="str">
-        <f t="shared" ref="J15:J17" si="36">IF(ISBLANK('ONR 2'!J8),"",'ONR 2'!J8)</f>
+        <f>IF(ISBLANK('ONR 2'!J8),"",'ONR 2'!J8)</f>
       </c>
       <c r="K15" s="227" t="str">
-        <f t="shared" ref="K15:K17" si="37">IF(ISBLANK('ONR 2'!K8),"",'ONR 2'!K8)</f>
+        <f>IF(ISBLANK('ONR 2'!K8),"",'ONR 2'!K8)</f>
       </c>
       <c r="L15" s="227" t="b">
-        <f t="shared" ref="L15:L17" si="38">IF(ISBLANK('ONR 2'!L8),"",'ONR 2'!L8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!L8),"",'ONR 2'!L8)</f>
       </c>
       <c r="M15" s="227" t="b">
-        <f t="shared" ref="M15:M17" si="39">IF(ISBLANK('ONR 2'!M8),"",'ONR 2'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!M8),"",'ONR 2'!M8)</f>
       </c>
       <c r="N15" s="227" t="b">
-        <f t="shared" ref="N15:N17" si="40">IF(ISBLANK('ONR 2'!N8),"",'ONR 2'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!N8),"",'ONR 2'!N8)</f>
       </c>
       <c r="O15" s="227" t="b">
-        <f t="shared" ref="O15:O17" si="41">IF(ISBLANK('ONR 2'!O8),"",'ONR 2'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!O8),"",'ONR 2'!O8)</f>
       </c>
       <c r="P15" s="227" t="b">
-        <f t="shared" ref="P15:P17" si="42">IF(ISBLANK('ONR 2'!P8),"",'ONR 2'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!P8),"",'ONR 2'!P8)</f>
       </c>
       <c r="Q15" s="227" t="b">
-        <f t="shared" ref="Q15:Q17" si="43">IF(ISBLANK('ONR 2'!Q8),"",'ONR 2'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!Q8),"",'ONR 2'!Q8)</f>
       </c>
       <c r="R15" s="227" t="b">
-        <f t="shared" ref="R15:R17" si="44">IF(ISBLANK('ONR 2'!R8),"",'ONR 2'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!R8),"",'ONR 2'!R8)</f>
       </c>
       <c r="S15" s="228" t="str">
-        <f t="shared" ref="S15:S17" si="45">IF(ISBLANK('ONR 2'!S8),"",'ONR 2'!S8)</f>
+        <f>IF(ISBLANK('ONR 2'!S8),"",'ONR 2'!S8)</f>
       </c>
       <c r="T15" s="226" t="str">
-        <f t="shared" ref="T15:T17" si="46">IF(ISBLANK('ONR 2'!T8),"",'ONR 2'!T8)</f>
+        <f>IF(ISBLANK('ONR 2'!T8),"",'ONR 2'!T8)</f>
       </c>
       <c r="U15" s="242" t="str">
-        <f t="shared" ref="U15:U17" si="47">IF(ISBLANK('ONR 2'!U8),"",'ONR 2'!U8)</f>
+        <f>IF(ISBLANK('ONR 2'!U8),"",'ONR 2'!U8)</f>
       </c>
       <c r="V15" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!G8),"",'ONR 2'!G8)</f>
@@ -32561,32 +32411,25 @@
         <v>1</v>
       </c>
       <c r="AF15" s="206" t="n">
-        <f t="shared" si="35">IF(L15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L15=TRUE,1,0)</f>
       </c>
       <c r="AG15" s="206" t="n">
-        <f t="shared" si="35">IF(M15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M15=TRUE,1,0)</f>
       </c>
       <c r="AH15" s="206" t="n">
-        <f t="shared" si="35">IF(N15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N15=TRUE,1,0)</f>
       </c>
       <c r="AI15" s="206" t="n">
-        <f t="shared" si="35">IF(O15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O15=TRUE,1,0)</f>
       </c>
       <c r="AJ15" s="206" t="n">
-        <f t="shared" si="35">IF(P15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P15=TRUE,1,0)</f>
       </c>
       <c r="AK15" s="206" t="n">
-        <f t="shared" si="35">IF(Q15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q15=TRUE,1,0)</f>
       </c>
       <c r="AL15" s="206" t="n">
-        <f t="shared" si="35">IF(R15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R15=TRUE,1,0)</f>
       </c>
       <c r="AM15" t="n">
         <f>IF(LEN(TRIM(W15))&gt;0,1,0)</f>
@@ -32622,90 +32465,47 @@
         <f>IF(ISBLANK('ONR 2'!I9),"",'ONR 2'!I9)</f>
       </c>
       <c r="J16" s="218" t="str">
-        <f t="shared" si="36">IF(ISBLANK('ONR 2'!J9),"",'ONR 2'!J9)</f>
-      </c>
-      <c r="K17" s="227" t="str">
-        <f t="shared" si="37">IF(ISBLANK('ONR 2'!K10),"",'ONR 2'!K10)</f>
+        <f>IF(ISBLANK('ONR 2'!J9),"",'ONR 2'!J9)</f>
       </c>
       <c r="K16" t="str" s="227">
         <f>IF(ISBLANK('ONR 2'!K9),"",'ONR 2'!K9)</f>
-      </c>
-      <c r="L17" s="227" t="b">
-        <f t="shared" si="38">IF(ISBLANK('ONR 2'!L10),"",'ONR 2'!L10)</f>
-        <v>0</v>
       </c>
       <c r="L16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!L9),"",'ONR 2'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M17" s="227" t="b">
-        <f t="shared" si="39">IF(ISBLANK('ONR 2'!M10),"",'ONR 2'!M10)</f>
-        <v>0</v>
-      </c>
       <c r="M16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!M9),"",'ONR 2'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N17" s="227" t="b">
-        <f t="shared" si="40">IF(ISBLANK('ONR 2'!N10),"",'ONR 2'!N10)</f>
-        <v>0</v>
-      </c>
       <c r="N16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!N9),"",'ONR 2'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O17" s="227" t="b">
-        <f t="shared" si="41">IF(ISBLANK('ONR 2'!O10),"",'ONR 2'!O10)</f>
-        <v>0</v>
-      </c>
       <c r="O16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!O9),"",'ONR 2'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P17" s="227" t="b">
-        <f t="shared" si="42">IF(ISBLANK('ONR 2'!P10),"",'ONR 2'!P10)</f>
-        <v>0</v>
-      </c>
       <c r="P16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!P9),"",'ONR 2'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="227" t="b">
-        <f t="shared" si="43">IF(ISBLANK('ONR 2'!Q10),"",'ONR 2'!Q10)</f>
-        <v>0</v>
-      </c>
       <c r="Q16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!Q9),"",'ONR 2'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R17" s="227" t="b">
-        <f t="shared" si="44">IF(ISBLANK('ONR 2'!R10),"",'ONR 2'!R10)</f>
-        <v>0</v>
-      </c>
       <c r="R16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!R9),"",'ONR 2'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S17" s="228" t="str">
-        <f t="shared" si="45">IF(ISBLANK('ONR 2'!S10),"",'ONR 2'!S10)</f>
-      </c>
       <c r="S16" t="str" s="228">
         <f>IF(ISBLANK('ONR 2'!S9),"",'ONR 2'!S9)</f>
       </c>
-      <c r="T17" s="226" t="str">
-        <f t="shared" si="46">IF(ISBLANK('ONR 2'!T10),"",'ONR 2'!T10)</f>
-      </c>
       <c r="T16" t="str" s="226">
         <f>IF(ISBLANK('ONR 2'!T9),"",'ONR 2'!T9)</f>
       </c>
-      <c r="U17" s="242" t="str">
-        <f t="shared" si="47">IF(ISBLANK('ONR 2'!U10),"",'ONR 2'!U10)</f>
-      </c>
       <c r="U16" t="str" s="242">
         <f>IF(ISBLANK('ONR 2'!U9),"",'ONR 2'!U9)</f>
-      </c>
-      <c r="V17" s="229" t="str">
-        <f>IF(ISBLANK('ONR 2'!G10),"",'ONR 2'!G10)</f>
       </c>
       <c r="V16" t="str" s="229">
         <f>IF(ISBLANK('ONR 2'!G9),"",'ONR 2'!G9)</f>
@@ -32727,32 +32527,25 @@
         <v>1</v>
       </c>
       <c r="AF16" s="206" t="n">
-        <f t="shared" si="35">IF(L16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L16=TRUE,1,0)</f>
       </c>
       <c r="AG16" s="206" t="n">
-        <f t="shared" si="35">IF(M16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M16=TRUE,1,0)</f>
       </c>
       <c r="AH16" s="206" t="n">
-        <f t="shared" si="35">IF(N16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N16=TRUE,1,0)</f>
       </c>
       <c r="AI16" s="206" t="n">
-        <f t="shared" si="35">IF(O16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O16=TRUE,1,0)</f>
       </c>
       <c r="AJ16" s="206" t="n">
-        <f t="shared" si="35">IF(P16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P16=TRUE,1,0)</f>
       </c>
       <c r="AK16" s="206" t="n">
-        <f t="shared" si="35">IF(Q16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q16=TRUE,1,0)</f>
       </c>
       <c r="AL16" s="206" t="n">
-        <f t="shared" si="35">IF(R16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R16=TRUE,1,0)</f>
       </c>
       <c r="AM16" t="n">
         <f>IF(LEN(TRIM(W16))&gt;0,1,0)</f>
@@ -32788,43 +32581,43 @@
         <f>IF(ISBLANK('ONR 2'!I10),"",'ONR 2'!I10)</f>
       </c>
       <c r="J17" s="218" t="str">
-        <f t="shared" si="36">IF(ISBLANK('ONR 2'!J10),"",'ONR 2'!J10)</f>
-      </c>
-      <c r="K19" s="227">
-        <f t="shared" si="37"/>
-      </c>
-      <c r="L19" s="227">
-        <f t="shared" si="38"/>
-      </c>
-      <c r="M19" s="227">
-        <f t="shared" si="39"/>
-      </c>
-      <c r="N19" s="227">
-        <f t="shared" si="40"/>
-      </c>
-      <c r="O19" s="227">
-        <f t="shared" si="41"/>
-      </c>
-      <c r="P19" s="227">
-        <f t="shared" si="42"/>
-      </c>
-      <c r="Q19" s="227">
-        <f t="shared" si="43"/>
-      </c>
-      <c r="R19" s="227">
-        <f t="shared" si="44"/>
-      </c>
-      <c r="S19" s="228">
-        <f t="shared" si="45"/>
-      </c>
-      <c r="T19" s="226">
-        <f t="shared" si="46"/>
-      </c>
-      <c r="U19" s="242">
-        <f t="shared" si="47"/>
-      </c>
-      <c r="V19" s="229">
-        <f>G17</f>
+        <f>IF(ISBLANK('ONR 2'!J10),"",'ONR 2'!J10)</f>
+      </c>
+      <c r="K17" s="227" t="str">
+        <f>IF(ISBLANK('ONR 2'!K10),"",'ONR 2'!K10)</f>
+      </c>
+      <c r="L17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!L10),"",'ONR 2'!L10)</f>
+      </c>
+      <c r="M17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!M10),"",'ONR 2'!M10)</f>
+      </c>
+      <c r="N17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!N10),"",'ONR 2'!N10)</f>
+      </c>
+      <c r="O17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!O10),"",'ONR 2'!O10)</f>
+      </c>
+      <c r="P17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!P10),"",'ONR 2'!P10)</f>
+      </c>
+      <c r="Q17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!Q10),"",'ONR 2'!Q10)</f>
+      </c>
+      <c r="R17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!R10),"",'ONR 2'!R10)</f>
+      </c>
+      <c r="S17" s="228" t="str">
+        <f>IF(ISBLANK('ONR 2'!S10),"",'ONR 2'!S10)</f>
+      </c>
+      <c r="T17" s="226" t="str">
+        <f>IF(ISBLANK('ONR 2'!T10),"",'ONR 2'!T10)</f>
+      </c>
+      <c r="U17" s="242" t="str">
+        <f>IF(ISBLANK('ONR 2'!U10),"",'ONR 2'!U10)</f>
+      </c>
+      <c r="V17" s="229" t="str">
+        <f>IF(ISBLANK('ONR 2'!G10),"",'ONR 2'!G10)</f>
       </c>
       <c r="W17" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!V10),"",'ONR 2'!V10)</f>
@@ -32843,32 +32636,25 @@
         <v>1</v>
       </c>
       <c r="AF17" s="206" t="n">
-        <f t="shared" si="35">IF(L17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L17=TRUE,1,0)</f>
       </c>
       <c r="AG17" s="206" t="n">
-        <f t="shared" si="35">IF(M17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M17=TRUE,1,0)</f>
       </c>
       <c r="AH17" s="206" t="n">
-        <f t="shared" si="35">IF(N17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N17=TRUE,1,0)</f>
       </c>
       <c r="AI17" s="206" t="n">
-        <f t="shared" si="35">IF(O17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O17=TRUE,1,0)</f>
       </c>
       <c r="AJ17" s="206" t="n">
-        <f t="shared" si="35">IF(P17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P17=TRUE,1,0)</f>
       </c>
       <c r="AK17" s="206" t="n">
-        <f t="shared" si="35">IF(Q17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q17=TRUE,1,0)</f>
       </c>
       <c r="AL17" s="206" t="n">
-        <f t="shared" si="35">IF(R17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R17=TRUE,1,0)</f>
       </c>
       <c r="AM17" t="n">
         <f>IF(LEN(TRIM(W17))&gt;0,1,0)</f>
@@ -33103,50 +32889,43 @@
         <f>IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
       </c>
       <c r="J20" s="246" t="str">
-        <f t="shared" ref="J20:J25" si="49">IF(ISBLANK('ONR 3'!J7),"",'ONR 3'!J7)</f>
+        <f>IF(ISBLANK('ONR 3'!J7),"",'ONR 3'!J7)</f>
       </c>
       <c r="K20" s="247" t="str">
-        <f t="shared" ref="K20:K25" si="50">IF(ISBLANK('ONR 3'!K7),"",'ONR 3'!K7)</f>
+        <f>IF(ISBLANK('ONR 3'!K7),"",'ONR 3'!K7)</f>
       </c>
       <c r="L20" s="247" t="b">
-        <f t="shared" ref="L20:L25" si="51">IF(ISBLANK('ONR 3'!L7),"",'ONR 3'!L7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!L7),"",'ONR 3'!L7)</f>
       </c>
       <c r="M20" s="247" t="b">
-        <f t="shared" ref="M20:M25" si="52">IF(ISBLANK('ONR 3'!M7),"",'ONR 3'!M7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!M7),"",'ONR 3'!M7)</f>
       </c>
       <c r="N20" s="247" t="b">
-        <f t="shared" ref="N20:N25" si="53">IF(ISBLANK('ONR 3'!N7),"",'ONR 3'!N7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!N7),"",'ONR 3'!N7)</f>
       </c>
       <c r="O20" s="247" t="b">
-        <f t="shared" ref="O20:O25" si="54">IF(ISBLANK('ONR 3'!O7),"",'ONR 3'!O7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!O7),"",'ONR 3'!O7)</f>
       </c>
       <c r="P20" s="247" t="b">
-        <f t="shared" ref="P20:P25" si="55">IF(ISBLANK('ONR 3'!P7),"",'ONR 3'!P7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!P7),"",'ONR 3'!P7)</f>
       </c>
       <c r="Q20" s="247" t="b">
-        <f t="shared" ref="Q20:Q25" si="56">IF(ISBLANK('ONR 3'!Q7),"",'ONR 3'!Q7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!Q7),"",'ONR 3'!Q7)</f>
       </c>
       <c r="R20" s="247" t="b">
-        <f t="shared" ref="R20:R25" si="57">IF(ISBLANK('ONR 3'!R7),"",'ONR 3'!R7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!R7),"",'ONR 3'!R7)</f>
       </c>
       <c r="S20" s="248" t="str">
-        <f t="shared" ref="S20:S25" si="58">IF(ISBLANK('ONR 3'!S7),"",'ONR 3'!S7)</f>
+        <f>IF(ISBLANK('ONR 3'!S7),"",'ONR 3'!S7)</f>
       </c>
       <c r="T20" s="249" t="str">
-        <f t="shared" ref="T20:T25" si="59">IF(ISBLANK('ONR 3'!T7),"",'ONR 3'!T7)</f>
+        <f>IF(ISBLANK('ONR 3'!T7),"",'ONR 3'!T7)</f>
       </c>
       <c r="U20" s="250" t="str">
-        <f t="shared" ref="U20:U25" si="60">IF(ISBLANK('ONR 3'!U7),"",'ONR 3'!U7)</f>
+        <f>IF(ISBLANK('ONR 3'!U7),"",'ONR 3'!U7)</f>
       </c>
       <c r="V20" s="235" t="str">
-        <f t="shared" ref="V20:V26" si="61">IF(ISBLANK('ONR 3'!G7),"",'ONR 3'!G7)</f>
+        <f>IF(ISBLANK('ONR 3'!G7),"",'ONR 3'!G7)</f>
       </c>
       <c r="W20" s="235" t="str">
         <f>IF(ISBLANK('ONR 3'!V7),"",'ONR 3'!V7)</f>
@@ -33155,42 +32934,34 @@
         <f>IF(ISBLANK('ONR 3'!W7),"",'ONR 3'!W7)</f>
       </c>
       <c r="Y20" s="236" t="str">
-        <f t="shared" ref="Y20:Y26" si="62">IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
+        <f>IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
       </c>
       <c r="Z20" s="236" t="str">
-        <f t="shared" ref="Z20:Z26" si="63">IF(ISBLANK('ONR 3'!D7),"",'ONR 3'!D7)</f>
+        <f>IF(ISBLANK('ONR 3'!D7),"",'ONR 3'!D7)</f>
       </c>
       <c r="AE20" s="206" t="n">
-        <f t="shared" ref="AE20:AE26" si="64">IF(ISNUMBER(T20),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T20),0,1)</f>
       </c>
       <c r="AF20" s="206" t="n">
-        <f t="shared" ref="AF20:AL26" si="65">IF(L20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L20=TRUE,1,0)</f>
       </c>
       <c r="AG20" s="206" t="n">
-        <f t="shared" si="65">IF(M20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M20=TRUE,1,0)</f>
       </c>
       <c r="AH20" s="206" t="n">
-        <f t="shared" si="65">IF(N20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N20=TRUE,1,0)</f>
       </c>
       <c r="AI20" s="206" t="n">
-        <f t="shared" si="65">IF(O20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O20=TRUE,1,0)</f>
       </c>
       <c r="AJ20" s="206" t="n">
-        <f t="shared" si="65">IF(P20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P20=TRUE,1,0)</f>
       </c>
       <c r="AK20" s="206" t="n">
-        <f t="shared" si="65">IF(Q20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q20=TRUE,1,0)</f>
       </c>
       <c r="AL20" s="206" t="n">
-        <f t="shared" si="65">IF(R20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R20=TRUE,1,0)</f>
       </c>
       <c r="AM20" t="n">
         <f>IF(LEN(TRIM(W20))&gt;0,1,0)</f>
@@ -33226,97 +32997,51 @@
         <f>IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
       </c>
       <c r="J21" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J8),"",'ONR 3'!J8)</f>
-      </c>
-      <c r="K23" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K10),"",'ONR 3'!K10)</f>
+        <f>IF(ISBLANK('ONR 3'!J8),"",'ONR 3'!J8)</f>
       </c>
       <c r="K21" t="str" s="247">
         <f>IF(ISBLANK('ONR 3'!K8),"",'ONR 3'!K8)</f>
-      </c>
-      <c r="L23" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L10),"",'ONR 3'!L10)</f>
-        <v>0</v>
       </c>
       <c r="L21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!L8),"",'ONR 3'!L8)</f>
         <v>0</v>
       </c>
-      <c r="M23" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M10),"",'ONR 3'!M10)</f>
-        <v>0</v>
-      </c>
       <c r="M21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!M8),"",'ONR 3'!M8)</f>
         <v>0</v>
       </c>
-      <c r="N23" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N10),"",'ONR 3'!N10)</f>
-        <v>0</v>
-      </c>
       <c r="N21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!N8),"",'ONR 3'!N8)</f>
         <v>0</v>
       </c>
-      <c r="O23" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O10),"",'ONR 3'!O10)</f>
-        <v>0</v>
-      </c>
       <c r="O21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!O8),"",'ONR 3'!O8)</f>
         <v>0</v>
       </c>
-      <c r="P23" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P10),"",'ONR 3'!P10)</f>
-        <v>0</v>
-      </c>
       <c r="P21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!P8),"",'ONR 3'!P8)</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q10),"",'ONR 3'!Q10)</f>
-        <v>0</v>
-      </c>
       <c r="Q21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!Q8),"",'ONR 3'!Q8)</f>
         <v>0</v>
       </c>
-      <c r="R23" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R10),"",'ONR 3'!R10)</f>
-        <v>0</v>
-      </c>
       <c r="R21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!R8),"",'ONR 3'!R8)</f>
         <v>0</v>
       </c>
-      <c r="S23" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S10),"",'ONR 3'!S10)</f>
-      </c>
       <c r="S21" t="str" s="248">
         <f>IF(ISBLANK('ONR 3'!S8),"",'ONR 3'!S8)</f>
       </c>
-      <c r="T23" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T10),"",'ONR 3'!T10)</f>
-      </c>
       <c r="T21" t="str" s="249">
         <f>IF(ISBLANK('ONR 3'!T8),"",'ONR 3'!T8)</f>
       </c>
-      <c r="U23" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U10),"",'ONR 3'!U10)</f>
-      </c>
       <c r="U21" t="str" s="250">
         <f>IF(ISBLANK('ONR 3'!U8),"",'ONR 3'!U8)</f>
       </c>
-      <c r="V23" s="235" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G10),"",'ONR 3'!G10)</f>
-      </c>
       <c r="V21" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!G8),"",'ONR 3'!G8)</f>
       </c>
-      <c r="W23" s="235" t="str">
-        <f>IF(ISBLANK('ONR 3'!V10),"",'ONR 3'!V10)</f>
-      </c>
       <c r="W21" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!V8),"",'ONR 3'!V8)</f>
       </c>
@@ -33324,42 +33049,34 @@
         <f>IF(ISBLANK('ONR 3'!W8),"",'ONR 3'!W8)</f>
       </c>
       <c r="Y21" s="236" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
+        <f>IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
       </c>
       <c r="Z21" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D8),"",'ONR 3'!D8)</f>
+        <f>IF(ISBLANK('ONR 3'!D8),"",'ONR 3'!D8)</f>
       </c>
       <c r="AE21" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T21),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T21),0,1)</f>
       </c>
       <c r="AF21" s="206" t="n">
-        <f t="shared" si="65">IF(L21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L21=TRUE,1,0)</f>
       </c>
       <c r="AG21" s="206" t="n">
-        <f t="shared" si="65">IF(M21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M21=TRUE,1,0)</f>
       </c>
       <c r="AH21" s="206" t="n">
-        <f t="shared" si="65">IF(N21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N21=TRUE,1,0)</f>
       </c>
       <c r="AI21" s="206" t="n">
-        <f t="shared" si="65">IF(O21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O21=TRUE,1,0)</f>
       </c>
       <c r="AJ21" s="206" t="n">
-        <f t="shared" si="65">IF(P21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P21=TRUE,1,0)</f>
       </c>
       <c r="AK21" s="206" t="n">
-        <f t="shared" si="65">IF(Q21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q21=TRUE,1,0)</f>
       </c>
       <c r="AL21" s="206" t="n">
-        <f t="shared" si="65">IF(R21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R21=TRUE,1,0)</f>
       </c>
       <c r="AM21" t="n">
         <f>IF(LEN(TRIM(W21))&gt;0,1,0)</f>
@@ -33395,97 +33112,51 @@
         <f>IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
       </c>
       <c r="J22" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J9),"",'ONR 3'!J9)</f>
-      </c>
-      <c r="K24" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K11),"",'ONR 3'!K11)</f>
+        <f>IF(ISBLANK('ONR 3'!J9),"",'ONR 3'!J9)</f>
       </c>
       <c r="K22" t="str" s="247">
         <f>IF(ISBLANK('ONR 3'!K9),"",'ONR 3'!K9)</f>
-      </c>
-      <c r="L24" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L11),"",'ONR 3'!L11)</f>
-        <v>0</v>
       </c>
       <c r="L22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!L9),"",'ONR 3'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M24" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M11),"",'ONR 3'!M11)</f>
-        <v>0</v>
-      </c>
       <c r="M22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!M9),"",'ONR 3'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N24" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N11),"",'ONR 3'!N11)</f>
-        <v>0</v>
-      </c>
       <c r="N22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!N9),"",'ONR 3'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O24" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O11),"",'ONR 3'!O11)</f>
-        <v>0</v>
-      </c>
       <c r="O22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!O9),"",'ONR 3'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P24" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P11),"",'ONR 3'!P11)</f>
-        <v>0</v>
-      </c>
       <c r="P22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!P9),"",'ONR 3'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q24" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q11),"",'ONR 3'!Q11)</f>
-        <v>0</v>
-      </c>
       <c r="Q22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!Q9),"",'ONR 3'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R24" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R11),"",'ONR 3'!R11)</f>
-        <v>0</v>
-      </c>
       <c r="R22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!R9),"",'ONR 3'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S24" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S11),"",'ONR 3'!S11)</f>
-      </c>
       <c r="S22" t="str" s="248">
         <f>IF(ISBLANK('ONR 3'!S9),"",'ONR 3'!S9)</f>
       </c>
-      <c r="T24" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T11),"",'ONR 3'!T11)</f>
-      </c>
       <c r="T22" t="str" s="249">
         <f>IF(ISBLANK('ONR 3'!T9),"",'ONR 3'!T9)</f>
       </c>
-      <c r="U24" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U11),"",'ONR 3'!U11)</f>
-      </c>
       <c r="U22" t="str" s="250">
         <f>IF(ISBLANK('ONR 3'!U9),"",'ONR 3'!U9)</f>
       </c>
-      <c r="V24" s="235" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G11),"",'ONR 3'!G11)</f>
-      </c>
       <c r="V22" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!G9),"",'ONR 3'!G9)</f>
       </c>
-      <c r="W24" s="235" t="str">
-        <f>IF(ISBLANK('ONR 3'!V11),"",'ONR 3'!V11)</f>
-      </c>
       <c r="W22" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!V9),"",'ONR 3'!V9)</f>
       </c>
@@ -33493,42 +33164,34 @@
         <f>IF(ISBLANK('ONR 3'!W9),"",'ONR 3'!W9)</f>
       </c>
       <c r="Y22" s="236" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
+        <f>IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
       </c>
       <c r="Z22" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D9),"",'ONR 3'!D9)</f>
+        <f>IF(ISBLANK('ONR 3'!D9),"",'ONR 3'!D9)</f>
       </c>
       <c r="AE22" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T22),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T22),0,1)</f>
       </c>
       <c r="AF22" s="206" t="n">
-        <f t="shared" si="65">IF(L22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L22=TRUE,1,0)</f>
       </c>
       <c r="AG22" s="206" t="n">
-        <f t="shared" si="65">IF(M22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M22=TRUE,1,0)</f>
       </c>
       <c r="AH22" s="206" t="n">
-        <f t="shared" si="65">IF(N22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N22=TRUE,1,0)</f>
       </c>
       <c r="AI22" s="206" t="n">
-        <f t="shared" si="65">IF(O22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O22=TRUE,1,0)</f>
       </c>
       <c r="AJ22" s="206" t="n">
-        <f t="shared" si="65">IF(P22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P22=TRUE,1,0)</f>
       </c>
       <c r="AK22" s="206" t="n">
-        <f t="shared" si="65">IF(Q22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q22=TRUE,1,0)</f>
       </c>
       <c r="AL22" s="206" t="n">
-        <f t="shared" si="65">IF(R22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R22=TRUE,1,0)</f>
       </c>
       <c r="AM22" t="n">
         <f>IF(LEN(TRIM(W22))&gt;0,1,0)</f>
@@ -33564,94 +33227,79 @@
         <f>IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
       </c>
       <c r="J23" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J10),"",'ONR 3'!J10)</f>
-      </c>
-      <c r="K25" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K12),"",'ONR 3'!K12)</f>
-      </c>
-      <c r="L25" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L12),"",'ONR 3'!L12)</f>
-        <v>0</v>
-      </c>
-      <c r="M25" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M12),"",'ONR 3'!M12)</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N12),"",'ONR 3'!N12)</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O12),"",'ONR 3'!O12)</f>
-        <v>0</v>
-      </c>
-      <c r="P25" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P12),"",'ONR 3'!P12)</f>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q12),"",'ONR 3'!Q12)</f>
-        <v>0</v>
-      </c>
-      <c r="R25" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R12),"",'ONR 3'!R12)</f>
-        <v>0</v>
-      </c>
-      <c r="S25" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S12),"",'ONR 3'!S12)</f>
-      </c>
-      <c r="T25" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T12),"",'ONR 3'!T12)</f>
-      </c>
-      <c r="U25" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U12),"",'ONR 3'!U12)</f>
-      </c>
-      <c r="V25" s="252" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G12),"",'ONR 3'!G12)</f>
-      </c>
-      <c r="W25" s="252" t="str">
-        <f>IF(ISBLANK('ONR 3'!V12),"",'ONR 3'!V12)</f>
+        <f>IF(ISBLANK('ONR 3'!J10),"",'ONR 3'!J10)</f>
+      </c>
+      <c r="K23" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K10),"",'ONR 3'!K10)</f>
+      </c>
+      <c r="L23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L10),"",'ONR 3'!L10)</f>
+      </c>
+      <c r="M23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M10),"",'ONR 3'!M10)</f>
+      </c>
+      <c r="N23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N10),"",'ONR 3'!N10)</f>
+      </c>
+      <c r="O23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O10),"",'ONR 3'!O10)</f>
+      </c>
+      <c r="P23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P10),"",'ONR 3'!P10)</f>
+      </c>
+      <c r="Q23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q10),"",'ONR 3'!Q10)</f>
+      </c>
+      <c r="R23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R10),"",'ONR 3'!R10)</f>
+      </c>
+      <c r="S23" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S10),"",'ONR 3'!S10)</f>
+      </c>
+      <c r="T23" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T10),"",'ONR 3'!T10)</f>
+      </c>
+      <c r="U23" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U10),"",'ONR 3'!U10)</f>
+      </c>
+      <c r="V23" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!G10),"",'ONR 3'!G10)</f>
+      </c>
+      <c r="W23" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!V10),"",'ONR 3'!V10)</f>
       </c>
       <c r="X23" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W10),"",'ONR 3'!W10)</f>
       </c>
       <c r="Y23" s="253" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
+        <f>IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
       </c>
       <c r="Z23" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D10),"",'ONR 3'!D10)</f>
+        <f>IF(ISBLANK('ONR 3'!D10),"",'ONR 3'!D10)</f>
       </c>
       <c r="AE23" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T23),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T23),0,1)</f>
       </c>
       <c r="AF23" s="206" t="n">
-        <f t="shared" si="65">IF(L23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L23=TRUE,1,0)</f>
       </c>
       <c r="AG23" s="206" t="n">
-        <f t="shared" si="65">IF(M23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M23=TRUE,1,0)</f>
       </c>
       <c r="AH23" s="206" t="n">
-        <f t="shared" si="65">IF(N23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N23=TRUE,1,0)</f>
       </c>
       <c r="AI23" s="206" t="n">
-        <f t="shared" si="65">IF(O23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O23=TRUE,1,0)</f>
       </c>
       <c r="AJ23" s="206" t="n">
-        <f t="shared" si="65">IF(P23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P23=TRUE,1,0)</f>
       </c>
       <c r="AK23" s="206" t="n">
-        <f t="shared" si="65">IF(Q23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q23=TRUE,1,0)</f>
       </c>
       <c r="AL23" s="206" t="n">
-        <f t="shared" si="65">IF(R23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R23=TRUE,1,0)</f>
       </c>
       <c r="AM23" t="n">
         <f>IF(LEN(TRIM(W23))&gt;0,1,0)</f>
@@ -33687,94 +33335,79 @@
         <f>IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
       </c>
       <c r="J24" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J11),"",'ONR 3'!J11)</f>
-      </c>
-      <c r="K26" s="247" t="str">
-        <f t="shared" si="50"/>
-      </c>
-      <c r="L26" s="247" t="b">
-        <f t="shared" si="51"/>
-        <v>0</v>
-      </c>
-      <c r="M26" s="247" t="b">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="N26" s="247" t="b">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="O26" s="247" t="b">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="P26" s="247" t="b">
-        <f t="shared" si="55"/>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="247" t="b">
-        <f t="shared" si="56"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="247" t="b">
-        <f t="shared" si="57"/>
-        <v>0</v>
-      </c>
-      <c r="S26" s="248" t="str">
-        <f t="shared" si="58"/>
-      </c>
-      <c r="T26" s="249" t="str">
-        <f t="shared" si="59"/>
-      </c>
-      <c r="U26" s="250" t="str">
-        <f t="shared" si="60"/>
-      </c>
-      <c r="V26" s="252" t="str">
-        <f t="shared" si="61"/>
-      </c>
-      <c r="W26" s="145" t="str">
-        <f>IF(ISBLANK('ONR 3'!V13),"",'ONR 3'!V13)</f>
+        <f>IF(ISBLANK('ONR 3'!J11),"",'ONR 3'!J11)</f>
+      </c>
+      <c r="K24" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K11),"",'ONR 3'!K11)</f>
+      </c>
+      <c r="L24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L11),"",'ONR 3'!L11)</f>
+      </c>
+      <c r="M24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M11),"",'ONR 3'!M11)</f>
+      </c>
+      <c r="N24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N11),"",'ONR 3'!N11)</f>
+      </c>
+      <c r="O24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O11),"",'ONR 3'!O11)</f>
+      </c>
+      <c r="P24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P11),"",'ONR 3'!P11)</f>
+      </c>
+      <c r="Q24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q11),"",'ONR 3'!Q11)</f>
+      </c>
+      <c r="R24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R11),"",'ONR 3'!R11)</f>
+      </c>
+      <c r="S24" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S11),"",'ONR 3'!S11)</f>
+      </c>
+      <c r="T24" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T11),"",'ONR 3'!T11)</f>
+      </c>
+      <c r="U24" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U11),"",'ONR 3'!U11)</f>
+      </c>
+      <c r="V24" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!G11),"",'ONR 3'!G11)</f>
+      </c>
+      <c r="W24" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!V11),"",'ONR 3'!V11)</f>
       </c>
       <c r="X24" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W11),"",'ONR 3'!W11)</f>
       </c>
       <c r="Y24" s="253" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
+        <f>IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
       </c>
       <c r="Z24" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D11),"",'ONR 3'!D11)</f>
+        <f>IF(ISBLANK('ONR 3'!D11),"",'ONR 3'!D11)</f>
       </c>
       <c r="AE24" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T24),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T24),0,1)</f>
       </c>
       <c r="AF24" s="206" t="n">
-        <f t="shared" si="65">IF(L24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L24=TRUE,1,0)</f>
       </c>
       <c r="AG24" s="206" t="n">
-        <f t="shared" si="65">IF(M24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M24=TRUE,1,0)</f>
       </c>
       <c r="AH24" s="206" t="n">
-        <f t="shared" si="65">IF(N24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N24=TRUE,1,0)</f>
       </c>
       <c r="AI24" s="206" t="n">
-        <f t="shared" si="65">IF(O24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O24=TRUE,1,0)</f>
       </c>
       <c r="AJ24" s="206" t="n">
-        <f t="shared" si="65">IF(P24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P24=TRUE,1,0)</f>
       </c>
       <c r="AK24" s="206" t="n">
-        <f t="shared" si="65">IF(Q24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q24=TRUE,1,0)</f>
       </c>
       <c r="AL24" s="206" t="n">
-        <f t="shared" si="65">IF(R24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R24=TRUE,1,0)</f>
       </c>
       <c r="AM24" t="n">
         <f>IF(LEN(TRIM(W24))&gt;0,1,0)</f>
@@ -33810,87 +33443,79 @@
         <f>IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
       </c>
       <c r="J25" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J12),"",'ONR 3'!J12)</f>
-      </c>
-      <c r="K28" s="247">
-        <f t="shared" si="50"/>
-      </c>
-      <c r="L28" s="247">
-        <f t="shared" si="51"/>
-      </c>
-      <c r="M28" s="247">
-        <f t="shared" si="52"/>
-      </c>
-      <c r="N28" s="247">
-        <f t="shared" si="53"/>
-      </c>
-      <c r="O28" s="247">
-        <f t="shared" si="54"/>
-      </c>
-      <c r="P28" s="247">
-        <f t="shared" si="55"/>
-      </c>
-      <c r="Q28" s="247">
-        <f t="shared" si="56"/>
-      </c>
-      <c r="R28" s="247">
-        <f t="shared" si="57"/>
-      </c>
-      <c r="S28" s="248">
-        <f t="shared" si="58"/>
-      </c>
-      <c r="T28" s="249">
-        <f t="shared" si="59"/>
-      </c>
-      <c r="U28" s="250">
-        <f t="shared" si="60"/>
-      </c>
-      <c r="V28" s="241">
-        <f t="shared" si="61"/>
-      </c>
-      <c r="W28" s="148">
-        <f>'ONR 3'!V12</f>
+        <f>IF(ISBLANK('ONR 3'!J12),"",'ONR 3'!J12)</f>
+      </c>
+      <c r="K25" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K12),"",'ONR 3'!K12)</f>
+      </c>
+      <c r="L25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L12),"",'ONR 3'!L12)</f>
+      </c>
+      <c r="M25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M12),"",'ONR 3'!M12)</f>
+      </c>
+      <c r="N25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N12),"",'ONR 3'!N12)</f>
+      </c>
+      <c r="O25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O12),"",'ONR 3'!O12)</f>
+      </c>
+      <c r="P25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P12),"",'ONR 3'!P12)</f>
+      </c>
+      <c r="Q25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q12),"",'ONR 3'!Q12)</f>
+      </c>
+      <c r="R25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R12),"",'ONR 3'!R12)</f>
+      </c>
+      <c r="S25" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S12),"",'ONR 3'!S12)</f>
+      </c>
+      <c r="T25" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T12),"",'ONR 3'!T12)</f>
+      </c>
+      <c r="U25" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U12),"",'ONR 3'!U12)</f>
+      </c>
+      <c r="V25" s="252" t="str">
+        <f>IF(ISBLANK('ONR 3'!G12),"",'ONR 3'!G12)</f>
+      </c>
+      <c r="W25" s="252" t="str">
+        <f>IF(ISBLANK('ONR 3'!V12),"",'ONR 3'!V12)</f>
       </c>
       <c r="X25" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W12),"",'ONR 3'!W12)</f>
       </c>
       <c r="Y25" s="254" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
+        <f>IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
       </c>
       <c r="Z25" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D12),"",'ONR 3'!D12)</f>
+        <f>IF(ISBLANK('ONR 3'!D12),"",'ONR 3'!D12)</f>
       </c>
       <c r="AE25" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T25),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T25),0,1)</f>
       </c>
       <c r="AF25" s="206" t="n">
-        <f t="shared" si="65">IF(L25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L25=TRUE,1,0)</f>
       </c>
       <c r="AG25" s="206" t="n">
-        <f t="shared" si="65">IF(M25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M25=TRUE,1,0)</f>
       </c>
       <c r="AH25" s="206" t="n">
-        <f t="shared" si="65">IF(N25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N25=TRUE,1,0)</f>
       </c>
       <c r="AI25" s="206" t="n">
-        <f t="shared" si="65">IF(O25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O25=TRUE,1,0)</f>
       </c>
       <c r="AJ25" s="206" t="n">
-        <f t="shared" si="65">IF(P25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P25=TRUE,1,0)</f>
       </c>
       <c r="AK25" s="206" t="n">
-        <f t="shared" si="65">IF(Q25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q25=TRUE,1,0)</f>
       </c>
       <c r="AL25" s="206" t="n">
-        <f t="shared" si="65">IF(R25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R25=TRUE,1,0)</f>
       </c>
       <c r="AM25" t="n">
         <f>IF(LEN(TRIM(W25))&gt;0,1,0)</f>
@@ -33926,94 +33551,79 @@
         <f>IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
       </c>
       <c r="J26" s="246" t="str">
-        <f t="shared" ref="J26" si="66">IF(ISBLANK('ONR 3'!J13),"",'ONR 3'!J13)</f>
+        <f>IF(ISBLANK('ONR 3'!J13),"",'ONR 3'!J13)</f>
       </c>
       <c r="K26" s="247" t="str">
-        <f t="shared" ref="K26" si="67">IF(ISBLANK('ONR 3'!K13),"",'ONR 3'!K13)</f>
+        <f>IF(ISBLANK('ONR 3'!K13),"",'ONR 3'!K13)</f>
       </c>
       <c r="L26" s="247" t="b">
-        <f t="shared" ref="L26" si="68">IF(ISBLANK('ONR 3'!L13),"",'ONR 3'!L13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!L13),"",'ONR 3'!L13)</f>
       </c>
       <c r="M26" s="247" t="b">
-        <f t="shared" ref="M26" si="69">IF(ISBLANK('ONR 3'!M13),"",'ONR 3'!M13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!M13),"",'ONR 3'!M13)</f>
       </c>
       <c r="N26" s="247" t="b">
-        <f t="shared" ref="N26" si="70">IF(ISBLANK('ONR 3'!N13),"",'ONR 3'!N13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!N13),"",'ONR 3'!N13)</f>
       </c>
       <c r="O26" s="247" t="b">
-        <f t="shared" ref="O26" si="71">IF(ISBLANK('ONR 3'!O13),"",'ONR 3'!O13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!O13),"",'ONR 3'!O13)</f>
       </c>
       <c r="P26" s="247" t="b">
-        <f t="shared" ref="P26" si="72">IF(ISBLANK('ONR 3'!P13),"",'ONR 3'!P13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!P13),"",'ONR 3'!P13)</f>
       </c>
       <c r="Q26" s="247" t="b">
-        <f t="shared" ref="Q26" si="73">IF(ISBLANK('ONR 3'!Q13),"",'ONR 3'!Q13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!Q13),"",'ONR 3'!Q13)</f>
       </c>
       <c r="R26" s="247" t="b">
-        <f t="shared" ref="R26" si="74">IF(ISBLANK('ONR 3'!R13),"",'ONR 3'!R13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!R13),"",'ONR 3'!R13)</f>
       </c>
       <c r="S26" s="248" t="str">
-        <f t="shared" ref="S26" si="75">IF(ISBLANK('ONR 3'!S13),"",'ONR 3'!S13)</f>
+        <f>IF(ISBLANK('ONR 3'!S13),"",'ONR 3'!S13)</f>
       </c>
       <c r="T26" s="249" t="str">
-        <f t="shared" ref="T26" si="76">IF(ISBLANK('ONR 3'!T13),"",'ONR 3'!T13)</f>
+        <f>IF(ISBLANK('ONR 3'!T13),"",'ONR 3'!T13)</f>
       </c>
       <c r="U26" s="250" t="str">
-        <f t="shared" ref="U26" si="77">IF(ISBLANK('ONR 3'!U13),"",'ONR 3'!U13)</f>
+        <f>IF(ISBLANK('ONR 3'!U13),"",'ONR 3'!U13)</f>
       </c>
       <c r="V26" s="255" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G13),"",'ONR 3'!G13)</f>
-      </c>
-      <c r="W29" s="215" t="str">
-        <f>'ONR 3'!V13</f>
+        <f>IF(ISBLANK('ONR 3'!G13),"",'ONR 3'!G13)</f>
+      </c>
+      <c r="W26" s="145" t="str">
+        <f>IF(ISBLANK('ONR 3'!V13),"",'ONR 3'!V13)</f>
       </c>
       <c r="X26" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W13),"",'ONR 3'!W13)</f>
       </c>
       <c r="Y26" s="251" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
+        <f>IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
       </c>
       <c r="Z26" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D13),"",'ONR 3'!D13)</f>
+        <f>IF(ISBLANK('ONR 3'!D13),"",'ONR 3'!D13)</f>
       </c>
       <c r="AE26" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T26),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T26),0,1)</f>
       </c>
       <c r="AF26" s="206" t="n">
-        <f t="shared" si="65">IF(L26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L26=TRUE,1,0)</f>
       </c>
       <c r="AG26" s="206" t="n">
-        <f t="shared" si="65">IF(M26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M26=TRUE,1,0)</f>
       </c>
       <c r="AH26" s="206" t="n">
-        <f t="shared" si="65">IF(N26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N26=TRUE,1,0)</f>
       </c>
       <c r="AI26" s="206" t="n">
-        <f t="shared" si="65">IF(O26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O26=TRUE,1,0)</f>
       </c>
       <c r="AJ26" s="206" t="n">
-        <f t="shared" si="65">IF(P26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P26=TRUE,1,0)</f>
       </c>
       <c r="AK26" s="206" t="n">
-        <f t="shared" si="65">IF(Q26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q26=TRUE,1,0)</f>
       </c>
       <c r="AL26" s="206" t="n">
-        <f t="shared" si="65">IF(R26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R26=TRUE,1,0)</f>
       </c>
       <c r="AM26" t="n">
         <f>IF(LEN(TRIM(W26))&gt;0,1,0)</f>
@@ -34251,7 +33861,7 @@
         <f>IF(ISBLANK('ONR 4'!J7),"",'ONR 4'!J7)</f>
       </c>
       <c r="K29" s="227" t="str">
-        <f t="shared" ref="K29:K30" si="79">IF(ISBLANK('ONR 4'!K7),"",'ONR 4'!K7)</f>
+        <f>IF(ISBLANK('ONR 4'!K7),"",'ONR 4'!K7)</f>
       </c>
       <c r="L29" s="227" t="b">
         <f>IF(ISBLANK('ONR 4'!L7),"",'ONR 4'!L7)</f>
@@ -34282,13 +33892,13 @@
         <v>0</v>
       </c>
       <c r="S29" s="228" t="str">
-        <f t="shared" ref="S29:S30" si="80">IF(ISBLANK('ONR 4'!S7),"",'ONR 4'!S7)</f>
+        <f>IF(ISBLANK('ONR 4'!S7),"",'ONR 4'!S7)</f>
       </c>
       <c r="T29" s="226" t="str">
-        <f t="shared" ref="T29" si="81">IF(ISBLANK('ONR 4'!T7),"",'ONR 4'!T7)</f>
+        <f>IF(ISBLANK('ONR 4'!T7),"",'ONR 4'!T7)</f>
       </c>
       <c r="U29" s="242" t="str">
-        <f t="shared" ref="U29" si="82">IF(ISBLANK('ONR 4'!U7),"",'ONR 4'!U7)</f>
+        <f>IF(ISBLANK('ONR 4'!U7),"",'ONR 4'!U7)</f>
       </c>
       <c r="V29" s="229" t="str">
         <f>IF(ISBLANK('ONR 4'!G7),"",'ONR 4'!G7)</f>
@@ -34310,32 +33920,25 @@
         <v>1</v>
       </c>
       <c r="AF29" s="206" t="n">
-        <f t="shared" ref="AF29:AL32" si="83">IF(L29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L29=TRUE,1,0)</f>
       </c>
       <c r="AG29" s="206" t="n">
-        <f t="shared" si="83">IF(M29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M29=TRUE,1,0)</f>
       </c>
       <c r="AH29" s="206" t="n">
-        <f t="shared" si="83">IF(N29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N29=TRUE,1,0)</f>
       </c>
       <c r="AI29" s="206" t="n">
-        <f t="shared" si="83">IF(O29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O29=TRUE,1,0)</f>
       </c>
       <c r="AJ29" s="206" t="n">
-        <f t="shared" si="83">IF(P29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P29=TRUE,1,0)</f>
       </c>
       <c r="AK29" s="206" t="n">
-        <f t="shared" si="83">IF(Q29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q29=TRUE,1,0)</f>
       </c>
       <c r="AL29" s="206" t="n">
-        <f t="shared" si="83">IF(R29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R29=TRUE,1,0)</f>
       </c>
       <c r="AM29" t="n">
         <f>IF(LEN(TRIM(W29))&gt;0,1,0)</f>
@@ -34371,59 +33974,41 @@
         <f>IF(ISBLANK('ONR 4'!I8),"",'ONR 4'!I8)</f>
       </c>
       <c r="J30" s="219" t="str">
-        <f t="shared" ref="J30:J38" si="84">IF(ISBLANK('ONR 4'!J8),"",'ONR 4'!J8)</f>
+        <f>IF(ISBLANK('ONR 4'!J8),"",'ONR 4'!J8)</f>
       </c>
       <c r="K30" s="233" t="str">
-        <f t="shared" si="79">IF(ISBLANK('ONR 4'!K8),"",'ONR 4'!K8)</f>
-      </c>
-      <c r="L33" s="233">
-        <f t="shared" ref="L33" si="85">OR(K30=31)</f>
+        <f>IF(ISBLANK('ONR 4'!K8),"",'ONR 4'!K8)</f>
       </c>
       <c r="L30" t="b" s="227">
         <f>IF(ISBLANK('ONR 4'!L8),"",'ONR 4'!L8)</f>
         <v>0</v>
       </c>
       <c r="M30" s="233" t="b">
-        <f t="shared" ref="M30" si="86">IF(ISBLANK('ONR 4'!M8),"",'ONR 4'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!M8),"",'ONR 4'!M8)</f>
       </c>
       <c r="N30" s="233" t="b">
-        <f t="shared" ref="N30" si="87">IF(ISBLANK('ONR 4'!N8),"",'ONR 4'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!N8),"",'ONR 4'!N8)</f>
       </c>
       <c r="O30" s="233" t="b">
-        <f t="shared" ref="O30" si="88">IF(ISBLANK('ONR 4'!O8),"",'ONR 4'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!O8),"",'ONR 4'!O8)</f>
       </c>
       <c r="P30" s="233" t="b">
-        <f t="shared" ref="P30" si="89">IF(ISBLANK('ONR 4'!P8),"",'ONR 4'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!P8),"",'ONR 4'!P8)</f>
       </c>
       <c r="Q30" s="233" t="b">
-        <f t="shared" ref="Q30" si="90">IF(ISBLANK('ONR 4'!Q8),"",'ONR 4'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!Q8),"",'ONR 4'!Q8)</f>
       </c>
       <c r="R30" s="233" t="b">
-        <f t="shared" ref="R30" si="91">IF(ISBLANK('ONR 4'!R8),"",'ONR 4'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!R8),"",'ONR 4'!R8)</f>
       </c>
       <c r="S30" s="234" t="str">
-        <f t="shared" si="80">IF(ISBLANK('ONR 4'!S8),"",'ONR 4'!S8)</f>
-      </c>
-      <c r="T33" s="232">
-        <f t="shared" si="81"/>
+        <f>IF(ISBLANK('ONR 4'!S8),"",'ONR 4'!S8)</f>
       </c>
       <c r="T30" t="str" s="226">
         <f>IF(ISBLANK('ONR 4'!T8),"",'ONR 4'!T8)</f>
       </c>
-      <c r="U33" s="243">
-        <f t="shared" si="82"/>
-      </c>
       <c r="U30" t="str" s="242">
         <f>IF(ISBLANK('ONR 4'!U8),"",'ONR 4'!U8)</f>
-      </c>
-      <c r="V33" s="235">
-        <f>G30</f>
       </c>
       <c r="V30" t="str" s="229">
         <f>IF(ISBLANK('ONR 4'!G8),"",'ONR 4'!G8)</f>
@@ -34445,32 +34030,25 @@
         <v>1</v>
       </c>
       <c r="AF30" s="206" t="n">
-        <f t="shared" si="83">IF(L30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L30=TRUE,1,0)</f>
       </c>
       <c r="AG30" s="206" t="n">
-        <f t="shared" si="83">IF(M30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M30=TRUE,1,0)</f>
       </c>
       <c r="AH30" s="206" t="n">
-        <f t="shared" si="83">IF(N30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N30=TRUE,1,0)</f>
       </c>
       <c r="AI30" s="206" t="n">
-        <f t="shared" si="83">IF(O30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O30=TRUE,1,0)</f>
       </c>
       <c r="AJ30" s="206" t="n">
-        <f t="shared" si="83">IF(P30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P30=TRUE,1,0)</f>
       </c>
       <c r="AK30" s="206" t="n">
-        <f t="shared" si="83">IF(Q30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q30=TRUE,1,0)</f>
       </c>
       <c r="AL30" s="206" t="n">
-        <f t="shared" si="83">IF(R30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R30=TRUE,1,0)</f>
       </c>
       <c r="AM30" t="n">
         <f>IF(LEN(TRIM(W30))&gt;0,1,0)</f>
@@ -34506,47 +34084,40 @@
         <f>IF(ISBLANK('ONR 4'!I9),"",'ONR 4'!I9)</f>
       </c>
       <c r="J31" s="219" t="str">
-        <f t="shared" ref="J31:J32" si="92">IF(ISBLANK('ONR 4'!J9),"",'ONR 4'!J9)</f>
+        <f>IF(ISBLANK('ONR 4'!J9),"",'ONR 4'!J9)</f>
       </c>
       <c r="K31" s="233" t="str">
-        <f t="shared" ref="K31:K35" si="93">IF(ISBLANK('ONR 4'!K9),"",'ONR 4'!K9)</f>
+        <f>IF(ISBLANK('ONR 4'!K9),"",'ONR 4'!K9)</f>
       </c>
       <c r="L31" s="233" t="b">
-        <f t="shared" ref="L31:L35" si="94">IF(ISBLANK('ONR 4'!L9),"",'ONR 4'!L9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!L9),"",'ONR 4'!L9)</f>
       </c>
       <c r="M31" s="233" t="b">
-        <f t="shared" ref="M31" si="95">IF(ISBLANK('ONR 4'!M9),"",'ONR 4'!M9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!M9),"",'ONR 4'!M9)</f>
       </c>
       <c r="N31" s="233" t="b">
-        <f t="shared" ref="N31" si="96">IF(ISBLANK('ONR 4'!N9),"",'ONR 4'!N9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!N9),"",'ONR 4'!N9)</f>
       </c>
       <c r="O31" s="233" t="b">
-        <f t="shared" ref="O31" si="97">IF(ISBLANK('ONR 4'!O9),"",'ONR 4'!O9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!O9),"",'ONR 4'!O9)</f>
       </c>
       <c r="P31" s="233" t="b">
-        <f t="shared" ref="P31" si="98">IF(ISBLANK('ONR 4'!P9),"",'ONR 4'!P9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!P9),"",'ONR 4'!P9)</f>
       </c>
       <c r="Q31" s="233" t="b">
-        <f t="shared" ref="Q31" si="99">IF(ISBLANK('ONR 4'!Q9),"",'ONR 4'!Q9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!Q9),"",'ONR 4'!Q9)</f>
       </c>
       <c r="R31" s="233" t="b">
-        <f t="shared" ref="R31" si="100">IF(ISBLANK('ONR 4'!R9),"",'ONR 4'!R9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!R9),"",'ONR 4'!R9)</f>
       </c>
       <c r="S31" s="234" t="str">
-        <f t="shared" ref="S31" si="101">IF(ISBLANK('ONR 4'!S9),"",'ONR 4'!S9)</f>
+        <f>IF(ISBLANK('ONR 4'!S9),"",'ONR 4'!S9)</f>
       </c>
       <c r="T31" s="232" t="str">
-        <f t="shared" ref="T31:T35" si="102">IF(ISBLANK('ONR 4'!T9),"",'ONR 4'!T9)</f>
+        <f>IF(ISBLANK('ONR 4'!T9),"",'ONR 4'!T9)</f>
       </c>
       <c r="U31" s="243" t="str">
-        <f t="shared" ref="U31:U35" si="103">IF(ISBLANK('ONR 4'!U9),"",'ONR 4'!U9)</f>
+        <f>IF(ISBLANK('ONR 4'!U9),"",'ONR 4'!U9)</f>
       </c>
       <c r="V31" s="235" t="str">
         <f>IF(ISBLANK('ONR 4'!G9),"",'ONR 4'!G9)</f>
@@ -34568,32 +34139,25 @@
         <v>1</v>
       </c>
       <c r="AF31" s="206" t="n">
-        <f t="shared" si="83">IF(L31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L31=TRUE,1,0)</f>
       </c>
       <c r="AG31" s="206" t="n">
-        <f t="shared" si="83">IF(M31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M31=TRUE,1,0)</f>
       </c>
       <c r="AH31" s="206" t="n">
-        <f t="shared" si="83">IF(N31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N31=TRUE,1,0)</f>
       </c>
       <c r="AI31" s="206" t="n">
-        <f t="shared" si="83">IF(O31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O31=TRUE,1,0)</f>
       </c>
       <c r="AJ31" s="206" t="n">
-        <f t="shared" si="83">IF(P31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P31=TRUE,1,0)</f>
       </c>
       <c r="AK31" s="206" t="n">
-        <f t="shared" si="83">IF(Q31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q31=TRUE,1,0)</f>
       </c>
       <c r="AL31" s="206" t="n">
-        <f t="shared" si="83">IF(R31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R31=TRUE,1,0)</f>
       </c>
       <c r="AM31" t="n">
         <f>IF(LEN(TRIM(W31))&gt;0,1,0)</f>
@@ -34629,91 +34193,47 @@
         <f>IF(ISBLANK('ONR 4'!I10),"",'ONR 4'!I10)</f>
       </c>
       <c r="J32" s="219" t="n">
-        <f t="shared" si="92">IF(ISBLANK('ONR 4'!J10),"",'ONR 4'!J10)</f>
-        <v>0</v>
-      </c>
-      <c r="K35" s="233" t="str">
-        <f t="shared" si="93">IF(ISBLANK('ONR 5'!K8),"",'ONR 5'!K8)</f>
+        <f>IF(ISBLANK('ONR 4'!J10),"",'ONR 4'!J10)</f>
       </c>
       <c r="K32" t="str" s="233">
         <f>IF(ISBLANK('ONR 4'!K10),"",'ONR 4'!K10)</f>
-      </c>
-      <c r="L35" s="233" t="b">
-        <f t="shared" si="94">IF(ISBLANK('ONR 5'!L8),"",'ONR 5'!L8)</f>
-        <v>0</v>
       </c>
       <c r="L32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!L10),"",'ONR 4'!L10)</f>
         <v>0</v>
       </c>
-      <c r="M35" s="233" t="b">
-        <f t="shared" si="95"/>
-        <v>0</v>
-      </c>
       <c r="M32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!M10),"",'ONR 4'!M10)</f>
         <v>0</v>
       </c>
-      <c r="N35" s="233" t="b">
-        <f t="shared" si="96"/>
-        <v>0</v>
-      </c>
       <c r="N32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!N10),"",'ONR 4'!N10)</f>
         <v>0</v>
       </c>
-      <c r="O35" s="233" t="b">
-        <f t="shared" si="97"/>
-        <v>0</v>
-      </c>
       <c r="O32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!O10),"",'ONR 4'!O10)</f>
         <v>0</v>
       </c>
-      <c r="P35" s="233" t="b">
-        <f t="shared" si="98"/>
-        <v>0</v>
-      </c>
       <c r="P32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!P10),"",'ONR 4'!P10)</f>
         <v>0</v>
       </c>
-      <c r="Q35" s="233" t="b">
-        <f t="shared" si="99"/>
-        <v>0</v>
-      </c>
       <c r="Q32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!Q10),"",'ONR 4'!Q10)</f>
         <v>0</v>
       </c>
-      <c r="R35" s="233" t="b">
-        <f t="shared" si="100"/>
-        <v>0</v>
-      </c>
       <c r="R32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!R10),"",'ONR 4'!R10)</f>
         <v>0</v>
       </c>
-      <c r="S35" s="234" t="str">
-        <f t="shared" si="101"/>
-      </c>
       <c r="S32" t="str" s="234">
         <f>IF(ISBLANK('ONR 4'!S10),"",'ONR 4'!S10)</f>
       </c>
-      <c r="T35" s="232" t="str">
-        <f t="shared" si="102">IF(ISBLANK('ONR 5'!T8),"",'ONR 5'!T8)</f>
-      </c>
       <c r="T32" t="str" s="232">
         <f>IF(ISBLANK('ONR 4'!T10),"",'ONR 4'!T10)</f>
       </c>
-      <c r="U35" s="243" t="str">
-        <f t="shared" si="103">IF(ISBLANK('ONR 5'!U8),"",'ONR 5'!U8)</f>
-      </c>
       <c r="U32" t="str" s="243">
         <f>IF(ISBLANK('ONR 4'!U10),"",'ONR 4'!U10)</f>
-      </c>
-      <c r="V35" s="235" t="str">
-        <f>IF(ISBLANK('ONR 5'!G8),"",'ONR 5'!G8)</f>
       </c>
       <c r="V32" t="str" s="235">
         <f>IF(ISBLANK('ONR 4'!G10),"",'ONR 4'!G10)</f>
@@ -34735,32 +34255,25 @@
         <v>1</v>
       </c>
       <c r="AF32" s="206" t="n">
-        <f t="shared" si="83">IF(L32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L32=TRUE,1,0)</f>
       </c>
       <c r="AG32" s="206" t="n">
-        <f t="shared" si="83">IF(M32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M32=TRUE,1,0)</f>
       </c>
       <c r="AH32" s="206" t="n">
-        <f t="shared" si="83">IF(N32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N32=TRUE,1,0)</f>
       </c>
       <c r="AI32" s="206" t="n">
-        <f t="shared" si="83">IF(O32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O32=TRUE,1,0)</f>
       </c>
       <c r="AJ32" s="206" t="n">
-        <f t="shared" si="83">IF(P32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P32=TRUE,1,0)</f>
       </c>
       <c r="AK32" s="206" t="n">
-        <f t="shared" si="83">IF(Q32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q32=TRUE,1,0)</f>
       </c>
       <c r="AL32" s="206" t="n">
-        <f t="shared" si="83">IF(R32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R32=TRUE,1,0)</f>
       </c>
       <c r="AM32" t="n">
         <f>IF(LEN(TRIM(W32))&gt;0,1,0)</f>
@@ -34871,10 +34384,7 @@
         <f>IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
       </c>
       <c r="J34" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J7),"",'ONR 5'!J7)</f>
-      </c>
-      <c r="K37" s="227" t="str">
-        <f t="shared" ref="K37:K38" si="105">E34*10+F34</f>
+        <f>IF(ISBLANK('ONR 5'!J7),"",'ONR 5'!J7)</f>
       </c>
       <c r="K34" t="str" s="362">
         <f>IF(ISBLANK('ONR 5'!K7),"",'ONR 5'!K7)</f>
@@ -34908,16 +34418,16 @@
         <v>0</v>
       </c>
       <c r="S34" s="228" t="str">
-        <f t="shared" ref="S34:S38" si="106">IF(ISBLANK('ONR 5'!S7),"",'ONR 5'!S7)</f>
+        <f>IF(ISBLANK('ONR 5'!S7),"",'ONR 5'!S7)</f>
       </c>
       <c r="T34" s="226" t="str">
-        <f t="shared" ref="T34:T38" si="107">IF(ISBLANK('ONR 5'!T7),"",'ONR 5'!T7)</f>
+        <f>IF(ISBLANK('ONR 5'!T7),"",'ONR 5'!T7)</f>
       </c>
       <c r="U34" s="242" t="str">
-        <f t="shared" ref="U34:U38" si="108">IF(ISBLANK('ONR 5'!U7),"",'ONR 5'!U7)</f>
+        <f>IF(ISBLANK('ONR 5'!U7),"",'ONR 5'!U7)</f>
       </c>
       <c r="V34" s="229" t="str">
-        <f t="shared" ref="V34:V38" si="109">IF(ISBLANK('ONR 5'!G7),"",'ONR 5'!G7)</f>
+        <f>IF(ISBLANK('ONR 5'!G7),"",'ONR 5'!G7)</f>
       </c>
       <c r="W34" s="203" t="str">
         <f>IF(ISBLANK('ONR 5'!V7),"",'ONR 5'!V7)</f>
@@ -34926,42 +34436,34 @@
         <f>IF(ISBLANK('ONR 5'!W7),"",'ONR 5'!W7)</f>
       </c>
       <c r="Y34" s="257" t="str">
-        <f t="shared" ref="Y34:Y38" si="110">IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
+        <f>IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
       </c>
       <c r="Z34" s="256" t="str">
         <f>IF(ISBLANK('ONR 5'!D7),"",'ONR 5'!D7)</f>
       </c>
       <c r="AE34" s="206" t="n">
-        <f t="shared" ref="AE34:AE38" si="111">IF(ISNUMBER(T34),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T34),0,1)</f>
       </c>
       <c r="AF34" s="206" t="n">
-        <f t="shared" ref="AF34:AF38" si="112">IF(L34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L34=TRUE,1,0)</f>
       </c>
       <c r="AG34" s="206" t="n">
-        <f t="shared" ref="AG34:AG38" si="113">IF(M34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M34=TRUE,1,0)</f>
       </c>
       <c r="AH34" s="206" t="n">
-        <f t="shared" ref="AH34:AH38" si="114">IF(N34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N34=TRUE,1,0)</f>
       </c>
       <c r="AI34" s="206" t="n">
-        <f t="shared" ref="AI34:AI38" si="115">IF(O34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O34=TRUE,1,0)</f>
       </c>
       <c r="AJ34" s="206" t="n">
-        <f t="shared" ref="AJ34:AJ38" si="116">IF(P34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P34=TRUE,1,0)</f>
       </c>
       <c r="AK34" s="206" t="n">
-        <f t="shared" ref="AK34:AK38" si="117">IF(Q34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q34=TRUE,1,0)</f>
       </c>
       <c r="AL34" s="206" t="n">
-        <f t="shared" ref="AL34:AL38" si="118">IF(R34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R34=TRUE,1,0)</f>
       </c>
       <c r="AM34" t="n">
         <f>IF(LEN(TRIM(W34))&gt;0,1,0)</f>
@@ -34997,53 +34499,43 @@
         <f>IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
       </c>
       <c r="J35" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J8),"",'ONR 5'!J8)</f>
-      </c>
-      <c r="K38" s="233" t="str">
-        <f t="shared" si="105"/>
-      </c>
-      <c r="L38" s="233" t="b">
-        <f t="shared" ref="L38:L38" si="119">OR(K35=31)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!J8),"",'ONR 5'!J8)</f>
+      </c>
+      <c r="K35" s="233" t="str">
+        <f>IF(ISBLANK('ONR 5'!K8),"",'ONR 5'!K8)</f>
+      </c>
+      <c r="L35" s="233" t="b">
+        <f>IF(ISBLANK('ONR 5'!L8),"",'ONR 5'!L8)</f>
       </c>
       <c r="M35" s="233" t="b">
-        <f t="shared" ref="M35:M38" si="120">IF(ISBLANK('ONR 5'!M8),"",'ONR 5'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M8),"",'ONR 5'!M8)</f>
       </c>
       <c r="N35" s="233" t="b">
-        <f t="shared" ref="N35:N38" si="121">IF(ISBLANK('ONR 5'!N8),"",'ONR 5'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N8),"",'ONR 5'!N8)</f>
       </c>
       <c r="O35" s="233" t="b">
-        <f t="shared" ref="O35:O38" si="122">IF(ISBLANK('ONR 5'!O8),"",'ONR 5'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O8),"",'ONR 5'!O8)</f>
       </c>
       <c r="P35" s="233" t="b">
-        <f t="shared" ref="P35:P38" si="123">IF(ISBLANK('ONR 5'!P8),"",'ONR 5'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P8),"",'ONR 5'!P8)</f>
       </c>
       <c r="Q35" s="233" t="b">
-        <f t="shared" ref="Q35:Q38" si="124">IF(ISBLANK('ONR 5'!Q8),"",'ONR 5'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q8),"",'ONR 5'!Q8)</f>
       </c>
       <c r="R35" s="233" t="b">
-        <f t="shared" ref="R35:R38" si="125">IF(ISBLANK('ONR 5'!R8),"",'ONR 5'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R8),"",'ONR 5'!R8)</f>
       </c>
       <c r="S35" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S8),"",'ONR 5'!S8)</f>
-      </c>
-      <c r="T38" s="232" t="str">
-        <f t="shared" si="107"/>
-      </c>
-      <c r="U38" s="243" t="str">
-        <f t="shared" si="108"/>
-      </c>
-      <c r="V38" s="235" t="str">
-        <f t="shared" si="109"/>
-      </c>
-      <c r="W38" s="142" t="str">
-        <f>'ONR 5'!V8</f>
+        <f>IF(ISBLANK('ONR 5'!S8),"",'ONR 5'!S8)</f>
+      </c>
+      <c r="T35" s="232" t="str">
+        <f>IF(ISBLANK('ONR 5'!T8),"",'ONR 5'!T8)</f>
+      </c>
+      <c r="U35" s="243" t="str">
+        <f>IF(ISBLANK('ONR 5'!U8),"",'ONR 5'!U8)</f>
+      </c>
+      <c r="V35" s="235" t="str">
+        <f>IF(ISBLANK('ONR 5'!G8),"",'ONR 5'!G8)</f>
       </c>
       <c r="W35" t="str" s="203">
         <f>IF(ISBLANK('ONR 5'!V8),"",'ONR 5'!V8)</f>
@@ -35052,45 +34544,34 @@
         <f>IF(ISBLANK('ONR 5'!W8),"",'ONR 5'!W8)</f>
       </c>
       <c r="Y35" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
-      </c>
-      <c r="Z38" s="256" t="str">
-        <f t="shared" ref="Z38:Z38" si="126">D35</f>
+        <f>IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
       </c>
       <c r="Z35" t="str" s="256">
         <f>IF(ISBLANK('ONR 5'!D8),"",'ONR 5'!D8)</f>
       </c>
       <c r="AE35" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T35),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T35),0,1)</f>
       </c>
       <c r="AF35" s="206" t="n">
-        <f t="shared" si="112">IF(L35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L35=TRUE,1,0)</f>
       </c>
       <c r="AG35" s="206" t="n">
-        <f t="shared" si="113">IF(M35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M35=TRUE,1,0)</f>
       </c>
       <c r="AH35" s="206" t="n">
-        <f t="shared" si="114">IF(N35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N35=TRUE,1,0)</f>
       </c>
       <c r="AI35" s="206" t="n">
-        <f t="shared" si="115">IF(O35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O35=TRUE,1,0)</f>
       </c>
       <c r="AJ35" s="206" t="n">
-        <f t="shared" si="116">IF(P35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P35=TRUE,1,0)</f>
       </c>
       <c r="AK35" s="206" t="n">
-        <f t="shared" si="117">IF(Q35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q35=TRUE,1,0)</f>
       </c>
       <c r="AL35" s="206" t="n">
-        <f t="shared" si="118">IF(R35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R35=TRUE,1,0)</f>
       </c>
       <c r="AM35" t="n">
         <f>IF(LEN(TRIM(W35))&gt;0,1,0)</f>
@@ -35126,97 +34607,51 @@
         <f>IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
       </c>
       <c r="J36" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J9),"",'ONR 5'!J9)</f>
-      </c>
-      <c r="K39" s="233" t="str">
-        <f t="shared" si="105"/>
+        <f>IF(ISBLANK('ONR 5'!J9),"",'ONR 5'!J9)</f>
       </c>
       <c r="K36" t="str" s="233">
         <f>IF(ISBLANK('ONR 5'!K9),"",'ONR 5'!K9)</f>
-      </c>
-      <c r="L39" s="233" t="b">
-        <f t="shared" si="119"/>
-        <v>0</v>
       </c>
       <c r="L36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!L9),"",'ONR 5'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M39" s="233" t="b">
-        <f t="shared" si="120"/>
-        <v>0</v>
-      </c>
       <c r="M36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!M9),"",'ONR 5'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N39" s="233" t="b">
-        <f t="shared" si="121"/>
-        <v>0</v>
-      </c>
       <c r="N36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!N9),"",'ONR 5'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O39" s="233" t="b">
-        <f t="shared" si="122"/>
-        <v>0</v>
-      </c>
       <c r="O36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!O9),"",'ONR 5'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P39" s="233" t="b">
-        <f t="shared" si="123"/>
-        <v>0</v>
-      </c>
       <c r="P36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!P9),"",'ONR 5'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q39" s="233" t="b">
-        <f t="shared" si="124"/>
-        <v>0</v>
-      </c>
       <c r="Q36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!Q9),"",'ONR 5'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R39" s="233" t="b">
-        <f t="shared" si="125"/>
-        <v>0</v>
-      </c>
       <c r="R36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!R9),"",'ONR 5'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S39" s="234" t="str">
-        <f t="shared" si="106"/>
-      </c>
       <c r="S36" t="str" s="234">
         <f>IF(ISBLANK('ONR 5'!S9),"",'ONR 5'!S9)</f>
       </c>
-      <c r="T39" s="232" t="str">
-        <f t="shared" si="107"/>
-      </c>
       <c r="T36" t="str" s="232">
         <f>IF(ISBLANK('ONR 5'!T9),"",'ONR 5'!T9)</f>
       </c>
-      <c r="U39" s="243" t="str">
-        <f t="shared" si="108"/>
-      </c>
       <c r="U36" t="str" s="243">
         <f>IF(ISBLANK('ONR 5'!U9),"",'ONR 5'!U9)</f>
       </c>
-      <c r="V39" s="235" t="str">
-        <f t="shared" si="109"/>
-      </c>
       <c r="V36" t="str" s="235">
         <f>IF(ISBLANK('ONR 5'!G9),"",'ONR 5'!G9)</f>
       </c>
-      <c r="W39" s="142" t="str">
-        <f>'ONR 5'!V9</f>
-      </c>
       <c r="W36" t="str" s="142">
         <f>IF(ISBLANK('ONR 5'!V9),"",'ONR 5'!V9)</f>
       </c>
@@ -35224,42 +34659,34 @@
         <f>IF(ISBLANK('ONR 5'!W9),"",'ONR 5'!W9)</f>
       </c>
       <c r="Y36" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
+        <f>IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
       </c>
       <c r="Z36" s="256" t="str">
-        <f t="shared" si="126">IF(ISBLANK('ONR 5'!D9),"",'ONR 5'!D9)</f>
+        <f>IF(ISBLANK('ONR 5'!D9),"",'ONR 5'!D9)</f>
       </c>
       <c r="AE36" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T36),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T36),0,1)</f>
       </c>
       <c r="AF36" s="206" t="n">
-        <f t="shared" si="112">IF(L36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L36=TRUE,1,0)</f>
       </c>
       <c r="AG36" s="206" t="n">
-        <f t="shared" si="113">IF(M36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M36=TRUE,1,0)</f>
       </c>
       <c r="AH36" s="206" t="n">
-        <f t="shared" si="114">IF(N36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N36=TRUE,1,0)</f>
       </c>
       <c r="AI36" s="206" t="n">
-        <f t="shared" si="115">IF(O36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O36=TRUE,1,0)</f>
       </c>
       <c r="AJ36" s="206" t="n">
-        <f t="shared" si="116">IF(P36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P36=TRUE,1,0)</f>
       </c>
       <c r="AK36" s="206" t="n">
-        <f t="shared" si="117">IF(Q36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q36=TRUE,1,0)</f>
       </c>
       <c r="AL36" s="206" t="n">
-        <f t="shared" si="118">IF(R36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R36=TRUE,1,0)</f>
       </c>
       <c r="AM36" t="n">
         <f>IF(LEN(TRIM(W36))&gt;0,1,0)</f>
@@ -35295,50 +34722,43 @@
         <f>IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
       </c>
       <c r="J37" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J10),"",'ONR 5'!J10)</f>
+        <f>IF(ISBLANK('ONR 5'!J10),"",'ONR 5'!J10)</f>
       </c>
       <c r="K37" s="233" t="str">
-        <f t="shared" ref="K37:K38" si="105">IF(ISBLANK('ONR 5'!K10),"",'ONR 5'!K10)</f>
+        <f>IF(ISBLANK('ONR 5'!K10),"",'ONR 5'!K10)</f>
       </c>
       <c r="L37" s="233" t="b">
-        <f t="shared" si="119">IF(ISBLANK('ONR 5'!L10),"",'ONR 5'!L10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L10),"",'ONR 5'!L10)</f>
       </c>
       <c r="M37" s="233" t="b">
-        <f t="shared" si="120">IF(ISBLANK('ONR 5'!M10),"",'ONR 5'!M10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M10),"",'ONR 5'!M10)</f>
       </c>
       <c r="N37" s="233" t="b">
-        <f t="shared" si="121">IF(ISBLANK('ONR 5'!N10),"",'ONR 5'!N10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N10),"",'ONR 5'!N10)</f>
       </c>
       <c r="O37" s="233" t="b">
-        <f t="shared" si="122">IF(ISBLANK('ONR 5'!O10),"",'ONR 5'!O10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O10),"",'ONR 5'!O10)</f>
       </c>
       <c r="P37" s="233" t="b">
-        <f t="shared" si="123">IF(ISBLANK('ONR 5'!P10),"",'ONR 5'!P10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P10),"",'ONR 5'!P10)</f>
       </c>
       <c r="Q37" s="233" t="b">
-        <f t="shared" si="124">IF(ISBLANK('ONR 5'!Q10),"",'ONR 5'!Q10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q10),"",'ONR 5'!Q10)</f>
       </c>
       <c r="R37" s="233" t="b">
-        <f t="shared" si="125">IF(ISBLANK('ONR 5'!R10),"",'ONR 5'!R10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R10),"",'ONR 5'!R10)</f>
       </c>
       <c r="S37" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S10),"",'ONR 5'!S10)</f>
+        <f>IF(ISBLANK('ONR 5'!S10),"",'ONR 5'!S10)</f>
       </c>
       <c r="T37" s="232" t="str">
-        <f t="shared" si="107">IF(ISBLANK('ONR 5'!T10),"",'ONR 5'!T10)</f>
+        <f>IF(ISBLANK('ONR 5'!T10),"",'ONR 5'!T10)</f>
       </c>
       <c r="U37" s="243" t="str">
-        <f t="shared" si="108">IF(ISBLANK('ONR 5'!U10),"",'ONR 5'!U10)</f>
+        <f>IF(ISBLANK('ONR 5'!U10),"",'ONR 5'!U10)</f>
       </c>
       <c r="V37" s="235" t="str">
-        <f t="shared" si="109">IF(ISBLANK('ONR 5'!G10),"",'ONR 5'!G10)</f>
+        <f>IF(ISBLANK('ONR 5'!G10),"",'ONR 5'!G10)</f>
       </c>
       <c r="W37" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V10),"",'ONR 5'!V10)</f>
@@ -35347,42 +34767,34 @@
         <f>IF(ISBLANK('ONR 5'!W10),"",'ONR 5'!W10)</f>
       </c>
       <c r="Y37" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
+        <f>IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
       </c>
       <c r="Z37" s="256" t="str">
-        <f t="shared" si="126">IF(ISBLANK('ONR 5'!D10),"",'ONR 5'!D10)</f>
+        <f>IF(ISBLANK('ONR 5'!D10),"",'ONR 5'!D10)</f>
       </c>
       <c r="AE37" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T37),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T37),0,1)</f>
       </c>
       <c r="AF37" s="206" t="n">
-        <f t="shared" si="112">IF(L37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L37=TRUE,1,0)</f>
       </c>
       <c r="AG37" s="206" t="n">
-        <f t="shared" si="113">IF(M37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M37=TRUE,1,0)</f>
       </c>
       <c r="AH37" s="206" t="n">
-        <f t="shared" si="114">IF(N37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N37=TRUE,1,0)</f>
       </c>
       <c r="AI37" s="206" t="n">
-        <f t="shared" si="115">IF(O37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O37=TRUE,1,0)</f>
       </c>
       <c r="AJ37" s="206" t="n">
-        <f t="shared" si="116">IF(P37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P37=TRUE,1,0)</f>
       </c>
       <c r="AK37" s="206" t="n">
-        <f t="shared" si="117">IF(Q37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q37=TRUE,1,0)</f>
       </c>
       <c r="AL37" s="206" t="n">
-        <f t="shared" si="118">IF(R37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R37=TRUE,1,0)</f>
       </c>
       <c r="AM37" t="n">
         <f>IF(LEN(TRIM(W37))&gt;0,1,0)</f>
@@ -35418,50 +34830,43 @@
         <f>IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
       </c>
       <c r="J38" s="219" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J11),"",'ONR 5'!J11)</f>
+        <f>IF(ISBLANK('ONR 5'!J11),"",'ONR 5'!J11)</f>
       </c>
       <c r="K38" s="233" t="str">
-        <f t="shared" si="105">IF(ISBLANK('ONR 5'!K11),"",'ONR 5'!K11)</f>
+        <f>IF(ISBLANK('ONR 5'!K11),"",'ONR 5'!K11)</f>
       </c>
       <c r="L38" s="233" t="b">
-        <f t="shared" ref="L37:L38" si="119">IF(ISBLANK('ONR 5'!L11),"",'ONR 5'!L11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L11),"",'ONR 5'!L11)</f>
       </c>
       <c r="M38" s="233" t="b">
-        <f t="shared" si="120">IF(ISBLANK('ONR 5'!M11),"",'ONR 5'!M11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M11),"",'ONR 5'!M11)</f>
       </c>
       <c r="N38" s="233" t="b">
-        <f t="shared" si="121">IF(ISBLANK('ONR 5'!N11),"",'ONR 5'!N11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N11),"",'ONR 5'!N11)</f>
       </c>
       <c r="O38" s="233" t="b">
-        <f t="shared" si="122">IF(ISBLANK('ONR 5'!O11),"",'ONR 5'!O11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O11),"",'ONR 5'!O11)</f>
       </c>
       <c r="P38" s="233" t="b">
-        <f t="shared" si="123">IF(ISBLANK('ONR 5'!P11),"",'ONR 5'!P11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P11),"",'ONR 5'!P11)</f>
       </c>
       <c r="Q38" s="233" t="b">
-        <f t="shared" si="124">IF(ISBLANK('ONR 5'!Q11),"",'ONR 5'!Q11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q11),"",'ONR 5'!Q11)</f>
       </c>
       <c r="R38" s="233" t="b">
-        <f t="shared" si="125">IF(ISBLANK('ONR 5'!R11),"",'ONR 5'!R11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R11),"",'ONR 5'!R11)</f>
       </c>
       <c r="S38" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S11),"",'ONR 5'!S11)</f>
+        <f>IF(ISBLANK('ONR 5'!S11),"",'ONR 5'!S11)</f>
       </c>
       <c r="T38" s="232" t="str">
-        <f t="shared" si="107">IF(ISBLANK('ONR 5'!T11),"",'ONR 5'!T11)</f>
+        <f>IF(ISBLANK('ONR 5'!T11),"",'ONR 5'!T11)</f>
       </c>
       <c r="U38" s="243" t="str">
-        <f t="shared" si="108">IF(ISBLANK('ONR 5'!U11),"",'ONR 5'!U11)</f>
+        <f>IF(ISBLANK('ONR 5'!U11),"",'ONR 5'!U11)</f>
       </c>
       <c r="V38" s="235" t="str">
-        <f t="shared" si="109">IF(ISBLANK('ONR 5'!G11),"",'ONR 5'!G11)</f>
+        <f>IF(ISBLANK('ONR 5'!G11),"",'ONR 5'!G11)</f>
       </c>
       <c r="W38" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V11),"",'ONR 5'!V11)</f>
@@ -35470,42 +34875,34 @@
         <f>IF(ISBLANK('ONR 5'!W11),"",'ONR 5'!W11)</f>
       </c>
       <c r="Y38" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
+        <f>IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
       </c>
       <c r="Z38" s="236" t="str">
-        <f t="shared" ref="Z36:Z38" si="126">IF(ISBLANK('ONR 5'!D11),"",'ONR 5'!D11)</f>
+        <f>IF(ISBLANK('ONR 5'!D11),"",'ONR 5'!D11)</f>
       </c>
       <c r="AE38" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T38),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T38),0,1)</f>
       </c>
       <c r="AF38" s="206" t="n">
-        <f t="shared" si="112">IF(L38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L38=TRUE,1,0)</f>
       </c>
       <c r="AG38" s="206" t="n">
-        <f t="shared" si="113">IF(M38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M38=TRUE,1,0)</f>
       </c>
       <c r="AH38" s="206" t="n">
-        <f t="shared" si="114">IF(N38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N38=TRUE,1,0)</f>
       </c>
       <c r="AI38" s="206" t="n">
-        <f t="shared" si="115">IF(O38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O38=TRUE,1,0)</f>
       </c>
       <c r="AJ38" s="206" t="n">
-        <f t="shared" si="116">IF(P38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P38=TRUE,1,0)</f>
       </c>
       <c r="AK38" s="206" t="n">
-        <f t="shared" si="117">IF(Q38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q38=TRUE,1,0)</f>
       </c>
       <c r="AL38" s="206" t="n">
-        <f t="shared" si="118">IF(R38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R38=TRUE,1,0)</f>
       </c>
       <c r="AM38" t="n">
         <f>IF(LEN(TRIM(W38))&gt;0,1,0)</f>
@@ -35540,50 +34937,43 @@
         <f>IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
       </c>
       <c r="J39" s="219" t="str">
-        <f t="shared" ref="J39" si="127">IF(ISBLANK('ONR 5'!J12),"",'ONR 5'!J12)</f>
+        <f>IF(ISBLANK('ONR 5'!J12),"",'ONR 5'!J12)</f>
       </c>
       <c r="K39" s="233" t="str">
-        <f t="shared" ref="K39" si="128">IF(ISBLANK('ONR 5'!K12),"",'ONR 5'!K12)</f>
+        <f>IF(ISBLANK('ONR 5'!K12),"",'ONR 5'!K12)</f>
       </c>
       <c r="L39" s="233" t="b">
-        <f t="shared" ref="L39" si="129">IF(ISBLANK('ONR 5'!L12),"",'ONR 5'!L12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L12),"",'ONR 5'!L12)</f>
       </c>
       <c r="M39" s="233" t="b">
-        <f t="shared" ref="M39" si="130">IF(ISBLANK('ONR 5'!M12),"",'ONR 5'!M12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M12),"",'ONR 5'!M12)</f>
       </c>
       <c r="N39" s="233" t="b">
-        <f t="shared" ref="N39" si="131">IF(ISBLANK('ONR 5'!N12),"",'ONR 5'!N12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N12),"",'ONR 5'!N12)</f>
       </c>
       <c r="O39" s="233" t="b">
-        <f t="shared" ref="O39" si="132">IF(ISBLANK('ONR 5'!O12),"",'ONR 5'!O12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O12),"",'ONR 5'!O12)</f>
       </c>
       <c r="P39" s="233" t="b">
-        <f t="shared" ref="P39" si="133">IF(ISBLANK('ONR 5'!P12),"",'ONR 5'!P12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P12),"",'ONR 5'!P12)</f>
       </c>
       <c r="Q39" s="233" t="b">
-        <f t="shared" ref="Q39" si="134">IF(ISBLANK('ONR 5'!Q12),"",'ONR 5'!Q12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q12),"",'ONR 5'!Q12)</f>
       </c>
       <c r="R39" s="233" t="b">
-        <f t="shared" ref="R39" si="135">IF(ISBLANK('ONR 5'!R12),"",'ONR 5'!R12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R12),"",'ONR 5'!R12)</f>
       </c>
       <c r="S39" s="234" t="str">
-        <f t="shared" ref="S39" si="136">IF(ISBLANK('ONR 5'!S12),"",'ONR 5'!S12)</f>
+        <f>IF(ISBLANK('ONR 5'!S12),"",'ONR 5'!S12)</f>
       </c>
       <c r="T39" s="232" t="str">
-        <f t="shared" ref="T39" si="137">IF(ISBLANK('ONR 5'!T12),"",'ONR 5'!T12)</f>
+        <f>IF(ISBLANK('ONR 5'!T12),"",'ONR 5'!T12)</f>
       </c>
       <c r="U39" s="243" t="str">
-        <f t="shared" ref="U39" si="138">IF(ISBLANK('ONR 5'!U12),"",'ONR 5'!U12)</f>
+        <f>IF(ISBLANK('ONR 5'!U12),"",'ONR 5'!U12)</f>
       </c>
       <c r="V39" s="235" t="str">
-        <f t="shared" ref="V39" si="139">IF(ISBLANK('ONR 5'!G12),"",'ONR 5'!G12)</f>
+        <f>IF(ISBLANK('ONR 5'!G12),"",'ONR 5'!G12)</f>
       </c>
       <c r="W39" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V12),"",'ONR 5'!V12)</f>
@@ -35592,42 +34982,34 @@
         <f>IF(ISBLANK('ONR 5'!W12),"",'ONR 5'!W12)</f>
       </c>
       <c r="Y39" s="258" t="str">
-        <f t="shared" ref="Y39" si="140">IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
+        <f>IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
       </c>
       <c r="Z39" s="236" t="str">
-        <f t="shared" ref="Z39" si="141">IF(ISBLANK('ONR 5'!D12),"",'ONR 5'!D12)</f>
+        <f>IF(ISBLANK('ONR 5'!D12),"",'ONR 5'!D12)</f>
       </c>
       <c r="AE39" s="206" t="n">
-        <f t="shared" ref="AE39" si="142">IF(ISNUMBER(T39),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T39),0,1)</f>
       </c>
       <c r="AF39" s="206" t="n">
-        <f t="shared" ref="AF39" si="143">IF(L39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L39=TRUE,1,0)</f>
       </c>
       <c r="AG39" s="206" t="n">
-        <f t="shared" ref="AG39" si="144">IF(M39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M39=TRUE,1,0)</f>
       </c>
       <c r="AH39" s="206" t="n">
-        <f t="shared" ref="AH39" si="145">IF(N39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N39=TRUE,1,0)</f>
       </c>
       <c r="AI39" s="206" t="n">
-        <f t="shared" ref="AI39" si="146">IF(O39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O39=TRUE,1,0)</f>
       </c>
       <c r="AJ39" s="206" t="n">
-        <f t="shared" ref="AJ39" si="147">IF(P39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P39=TRUE,1,0)</f>
       </c>
       <c r="AK39" s="206" t="n">
-        <f t="shared" ref="AK39" si="148">IF(Q39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q39=TRUE,1,0)</f>
       </c>
       <c r="AL39" s="206" t="n">
-        <f t="shared" ref="AL39" si="149">IF(R39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R39=TRUE,1,0)</f>
       </c>
       <c r="AM39" t="n">
         <f>IF(LEN(TRIM(W39))&gt;0,1,0)</f>

</xml_diff>

<commit_message>
fix(classeurs): réparer « Résultats détaillés » et repositionner les logos (#16)
Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/INR_GPC_ONR Exemple.xlsx
+++ b/INR_GPC_ONR Exemple.xlsx
@@ -31230,8 +31230,7 @@
         <v>Intervention urgente</v>
       </c>
       <c r="K5" s="227" t="n">
-        <f t="shared" ref="K5:K9" si="1">IF(ISBLANK('ONR 1'!K7),"",'ONR 1'!K7)</f>
-        <v>31</v>
+        <f>IF(ISBLANK('ONR 1'!K7),"",'ONR 1'!K7)</f>
       </c>
       <c r="L5" s="227" t="b">
         <f>IF(ISBLANK('ONR 1'!L7),"",'ONR 1'!L7)</f>
@@ -31262,20 +31261,16 @@
         <v>0</v>
       </c>
       <c r="S5" s="228" t="str">
-        <f t="shared" ref="S5:S9" si="2">IF(ISBLANK('ONR 1'!S7),"",'ONR 1'!S7)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!S7),"",'ONR 1'!S7)</f>
       </c>
       <c r="T5" s="226" t="n">
-        <f t="shared" ref="T5:T9" si="3">IF(ISBLANK('ONR 1'!T7),"",'ONR 1'!T7)</f>
-        <v>6</v>
+        <f>IF(ISBLANK('ONR 1'!T7),"",'ONR 1'!T7)</f>
       </c>
       <c r="U5" s="227" t="n">
-        <f t="shared" ref="U5:U9" si="4">IF(ISBLANK('ONR 1'!U7),"",'ONR 1'!U7)</f>
-        <v>63</v>
+        <f>IF(ISBLANK('ONR 1'!U7),"",'ONR 1'!U7)</f>
       </c>
       <c r="V5" s="229" t="str">
-        <f t="shared" ref="V5:V11" si="5">IF(ISBLANK('ONR 1'!G7),"",'ONR 1'!G7)</f>
-        <v>L’équipe Achats retient le prix d’achat comme seul critère de choix. Elle ne demande pas d’analyse du cycle de vie (ACV) aux fournisseurs dans les appels d’offres.</v>
+        <f>IF(ISBLANK('ONR 1'!G7),"",'ONR 1'!G7)</f>
       </c>
       <c r="W5" s="203" t="str">
         <f>IF(ISBLANK('ONR 1'!V7),"",'ONR 1'!V7)</f>
@@ -31285,46 +31280,34 @@
         <f>IF(ISBLANK('ONR 1'!W7),"",'ONR 1'!W7)</f>
       </c>
       <c r="Y5" s="230" t="str">
-        <f t="shared" ref="Y5:Y11" si="6">IF(ISBLANK('ONR 1'!I7),"",'ONR 1'!I7)</f>
-        <v>Point fort : la direction des achats souhaite adopter des pratiques plus durables.
-Point faible : l’équipe connaît peu les labels environnementaux des équipements informatiques.</v>
+        <f>IF(ISBLANK('ONR 1'!I7),"",'ONR 1'!I7)</f>
       </c>
       <c r="Z5" s="230" t="str">
-        <f t="shared" ref="Z5:Z11" si="7">IF(ISBLANK('ONR 1'!D7),"",'ONR 1'!D7)</f>
-        <v>Avantages possibles : réduire les émissions de gaz à effet de serre de l’organisation et se préparer aux futures règles environnementales.
-Risque : payer plus cher à l’achat certains équipements conçus pour limiter leurs effets sur l’environnement.</v>
+        <f>IF(ISBLANK('ONR 1'!D7),"",'ONR 1'!D7)</f>
       </c>
       <c r="AE5" s="206" t="n">
-        <f t="shared" ref="AE5:AE11" si="8">IF(ISNUMBER(T5),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T5),0,1)</f>
       </c>
       <c r="AF5" s="206" t="n">
-        <f t="shared" ref="AF5:AL11" si="9">IF(L5=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(L5=TRUE,1,0)</f>
       </c>
       <c r="AG5" s="206" t="n">
-        <f t="shared" si="9">IF(M5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M5=TRUE,1,0)</f>
       </c>
       <c r="AH5" s="206" t="n">
-        <f t="shared" si="9">IF(N5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N5=TRUE,1,0)</f>
       </c>
       <c r="AI5" s="206" t="n">
-        <f t="shared" si="9">IF(O5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O5=TRUE,1,0)</f>
       </c>
       <c r="AJ5" s="206" t="n">
-        <f t="shared" si="9">IF(P5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P5=TRUE,1,0)</f>
       </c>
       <c r="AK5" s="206" t="n">
-        <f t="shared" si="9">IF(Q5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q5=TRUE,1,0)</f>
       </c>
       <c r="AL5" s="206" t="n">
-        <f t="shared" si="9">IF(R5=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R5=TRUE,1,0)</f>
       </c>
       <c r="AM5" t="n">
         <f>IF(LEN(TRIM(W5))&gt;0,1,0)</f>
@@ -31367,56 +31350,43 @@
 Point faible : certains utilisateurs demandent du matériel neuf pour son apparence.</v>
       </c>
       <c r="J6" s="232" t="str">
-        <f t="shared" ref="J6:J9" si="10">IF(ISBLANK('ONR 1'!J8),"",'ONR 1'!J8)</f>
-        <v>Intervention à moyen terme</v>
+        <f>IF(ISBLANK('ONR 1'!J8),"",'ONR 1'!J8)</f>
       </c>
       <c r="K6" s="233" t="n">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K8),"",'ONR 1'!K8)</f>
-        <v>33</v>
+        <f>IF(ISBLANK('ONR 1'!K8),"",'ONR 1'!K8)</f>
       </c>
       <c r="L6" s="233" t="b">
-        <f t="shared" ref="L6:L9" si="11">IF(ISBLANK('ONR 1'!L8),"",'ONR 1'!L8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L8),"",'ONR 1'!L8)</f>
       </c>
       <c r="M6" s="233" t="b">
-        <f t="shared" ref="M6:M9" si="12">IF(ISBLANK('ONR 1'!M8),"",'ONR 1'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M8),"",'ONR 1'!M8)</f>
       </c>
       <c r="N6" s="233" t="b">
-        <f t="shared" ref="N6:N9" si="13">IF(ISBLANK('ONR 1'!N8),"",'ONR 1'!N8)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!N8),"",'ONR 1'!N8)</f>
       </c>
       <c r="O6" s="233" t="b">
-        <f t="shared" ref="O6:O9" si="14">IF(ISBLANK('ONR 1'!O8),"",'ONR 1'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O8),"",'ONR 1'!O8)</f>
       </c>
       <c r="P6" s="233" t="b">
-        <f t="shared" ref="P6:P9" si="15">IF(ISBLANK('ONR 1'!P8),"",'ONR 1'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P8),"",'ONR 1'!P8)</f>
       </c>
       <c r="Q6" s="233" t="b">
-        <f t="shared" ref="Q6:Q9" si="16">IF(ISBLANK('ONR 1'!Q8),"",'ONR 1'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q8),"",'ONR 1'!Q8)</f>
       </c>
       <c r="R6" s="233" t="b">
-        <f t="shared" ref="R6:R9" si="17">IF(ISBLANK('ONR 1'!R8),"",'ONR 1'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R8),"",'ONR 1'!R8)</f>
       </c>
       <c r="S6" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S8),"",'ONR 1'!S8)</f>
-        <v>Intervention à moyen terme</v>
+        <f>IF(ISBLANK('ONR 1'!S8),"",'ONR 1'!S8)</f>
       </c>
       <c r="T6" s="232" t="n">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T8),"",'ONR 1'!T8)</f>
-        <v>4</v>
+        <f>IF(ISBLANK('ONR 1'!T8),"",'ONR 1'!T8)</f>
       </c>
       <c r="U6" s="233" t="n">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U8),"",'ONR 1'!U8)</f>
-        <v>42</v>
+        <f>IF(ISBLANK('ONR 1'!U8),"",'ONR 1'!U8)</f>
       </c>
       <c r="V6" s="235" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G8),"",'ONR 1'!G8)</f>
-        <v>L’organisation a porté la durée de renouvellement des ordinateurs portables de trois à quatre ans l’année dernière. Elle dispose d’un contrat de maintenance.</v>
+        <f>IF(ISBLANK('ONR 1'!G8),"",'ONR 1'!G8)</f>
       </c>
       <c r="W6" s="235" t="str">
         <f>IF(ISBLANK('ONR 1'!V8),"",'ONR 1'!V8)</f>
@@ -31426,45 +31396,34 @@
         <f>IF(ISBLANK('ONR 1'!W8),"",'ONR 1'!W8)</f>
       </c>
       <c r="Y6" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I8),"",'ONR 1'!I8)</f>
-        <v>Point fort : l’équipe technique peut réparer les équipements en interne.
-Point faible : certains utilisateurs demandent du matériel neuf pour son apparence.</v>
+        <f>IF(ISBLANK('ONR 1'!I8),"",'ONR 1'!I8)</f>
       </c>
       <c r="Z6" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D8),"",'ONR 1'!D8)</f>
-        <v>Avantages possibles : réduire les dépenses d’achat de matériel et les déchets d’équipements électriques et électroniques (DEEE).</v>
+        <f>IF(ISBLANK('ONR 1'!D8),"",'ONR 1'!D8)</f>
       </c>
       <c r="AE6" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T6),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T6),0,1)</f>
       </c>
       <c r="AF6" s="206" t="n">
-        <f t="shared" si="9">IF(L6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L6=TRUE,1,0)</f>
       </c>
       <c r="AG6" s="206" t="n">
-        <f t="shared" si="9">IF(M6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M6=TRUE,1,0)</f>
       </c>
       <c r="AH6" s="206" t="n">
-        <f t="shared" si="9">IF(N6=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(N6=TRUE,1,0)</f>
       </c>
       <c r="AI6" s="206" t="n">
-        <f t="shared" si="9">IF(O6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O6=TRUE,1,0)</f>
       </c>
       <c r="AJ6" s="206" t="n">
-        <f t="shared" si="9">IF(P6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P6=TRUE,1,0)</f>
       </c>
       <c r="AK6" s="206" t="n">
-        <f t="shared" si="9">IF(Q6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q6=TRUE,1,0)</f>
       </c>
       <c r="AL6" s="206" t="n">
-        <f t="shared" si="9">IF(R6=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R6=TRUE,1,0)</f>
       </c>
       <c r="AM6" t="n">
         <f>IF(LEN(TRIM(W6))&gt;0,1,0)</f>
@@ -31508,56 +31467,43 @@
 Points faibles : ils connaissent peu les guides pour concevoir des services numériques moins polluants, comme le RGESN. Ils savent peu comment relier leurs projets aux ODD.</v>
       </c>
       <c r="J7" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J9),"",'ONR 1'!J9)</f>
-        <v>Intervention prioritaire</v>
+        <f>IF(ISBLANK('ONR 1'!J9),"",'ONR 1'!J9)</f>
       </c>
       <c r="K7" s="233" t="n">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K9),"",'ONR 1'!K9)</f>
-        <v>32</v>
+        <f>IF(ISBLANK('ONR 1'!K9),"",'ONR 1'!K9)</f>
       </c>
       <c r="L7" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L9),"",'ONR 1'!L9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L9),"",'ONR 1'!L9)</f>
       </c>
       <c r="M7" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M9),"",'ONR 1'!M9)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!M9),"",'ONR 1'!M9)</f>
       </c>
       <c r="N7" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N9),"",'ONR 1'!N9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N9),"",'ONR 1'!N9)</f>
       </c>
       <c r="O7" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O9),"",'ONR 1'!O9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O9),"",'ONR 1'!O9)</f>
       </c>
       <c r="P7" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P9),"",'ONR 1'!P9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P9),"",'ONR 1'!P9)</f>
       </c>
       <c r="Q7" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q9),"",'ONR 1'!Q9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q9),"",'ONR 1'!Q9)</f>
       </c>
       <c r="R7" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R9),"",'ONR 1'!R9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R9),"",'ONR 1'!R9)</f>
       </c>
       <c r="S7" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S9),"",'ONR 1'!S9)</f>
-        <v>Intervention prioritaire</v>
+        <f>IF(ISBLANK('ONR 1'!S9),"",'ONR 1'!S9)</f>
       </c>
       <c r="T7" s="232" t="n">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T9),"",'ONR 1'!T9)</f>
-        <v>5</v>
+        <f>IF(ISBLANK('ONR 1'!T9),"",'ONR 1'!T9)</f>
       </c>
       <c r="U7" s="233" t="n">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U9),"",'ONR 1'!U9)</f>
-        <v>52</v>
+        <f>IF(ISBLANK('ONR 1'!U9),"",'ONR 1'!U9)</f>
       </c>
       <c r="V7" s="235" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G9),"",'ONR 1'!G9)</f>
-        <v>Les équipes valident les nouveaux services et sites web selon des critères fonctionnels, graphiques et financiers. Elles ne mesurent ni le poids des pages ni l’impact environnemental du code.</v>
+        <f>IF(ISBLANK('ONR 1'!G9),"",'ONR 1'!G9)</f>
       </c>
       <c r="W7" s="142" t="str">
         <f>IF(ISBLANK('ONR 1'!V9),"",'ONR 1'!V9)</f>
@@ -31569,46 +31515,34 @@
         <f>IF(ISBLANK('ONR 1'!W9),"",'ONR 1'!W9)</f>
       </c>
       <c r="Y7" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I9),"",'ONR 1'!I9)</f>
-        <v>Point fort : les développeurs et les chefs de produit s’intéressent aux effets de leurs activités sur la société et l’environnement.
-Points faibles : ils connaissent peu les guides pour concevoir des services numériques moins polluants, comme le RGESN. Ils savent peu comment relier leurs projets aux ODD.</v>
+        <f>IF(ISBLANK('ONR 1'!I9),"",'ONR 1'!I9)</f>
       </c>
       <c r="Z7" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D9),"",'ONR 1'!D9)</f>
-        <v>Avantages possibles : réduire les effets des services sur l’environnement dès leur conception, faciliter leur utilisation et contribuer aux Objectifs de développement durable (ODD).
-Risques : accumuler des problèmes techniques non résolus ou créer des logiciels trop gourmands en ressources, qui obligent à remplacer le matériel plus tôt.</v>
+        <f>IF(ISBLANK('ONR 1'!D9),"",'ONR 1'!D9)</f>
       </c>
       <c r="AE7" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T7),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T7),0,1)</f>
       </c>
       <c r="AF7" s="206" t="n">
-        <f t="shared" si="9">IF(L7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L7=TRUE,1,0)</f>
       </c>
       <c r="AG7" s="206" t="n">
-        <f t="shared" si="9">IF(M7=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(M7=TRUE,1,0)</f>
       </c>
       <c r="AH7" s="206" t="n">
-        <f t="shared" si="9">IF(N7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N7=TRUE,1,0)</f>
       </c>
       <c r="AI7" s="206" t="n">
-        <f t="shared" si="9">IF(O7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O7=TRUE,1,0)</f>
       </c>
       <c r="AJ7" s="206" t="n">
-        <f t="shared" si="9">IF(P7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P7=TRUE,1,0)</f>
       </c>
       <c r="AK7" s="206" t="n">
-        <f t="shared" si="9">IF(Q7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q7=TRUE,1,0)</f>
       </c>
       <c r="AL7" s="206" t="n">
-        <f t="shared" si="9">IF(R7=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R7=TRUE,1,0)</f>
       </c>
       <c r="AM7" t="n">
         <f>IF(LEN(TRIM(W7))&gt;0,1,0)</f>
@@ -31644,50 +31578,43 @@
         <f>IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
       </c>
       <c r="J8" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J10),"",'ONR 1'!J10)</f>
+        <f>IF(ISBLANK('ONR 1'!J10),"",'ONR 1'!J10)</f>
       </c>
       <c r="K8" s="233" t="str">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K10),"",'ONR 1'!K10)</f>
+        <f>IF(ISBLANK('ONR 1'!K10),"",'ONR 1'!K10)</f>
       </c>
       <c r="L8" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L10),"",'ONR 1'!L10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L10),"",'ONR 1'!L10)</f>
       </c>
       <c r="M8" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M10),"",'ONR 1'!M10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M10),"",'ONR 1'!M10)</f>
       </c>
       <c r="N8" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N10),"",'ONR 1'!N10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N10),"",'ONR 1'!N10)</f>
       </c>
       <c r="O8" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O10),"",'ONR 1'!O10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O10),"",'ONR 1'!O10)</f>
       </c>
       <c r="P8" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P10),"",'ONR 1'!P10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P10),"",'ONR 1'!P10)</f>
       </c>
       <c r="Q8" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q10),"",'ONR 1'!Q10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q10),"",'ONR 1'!Q10)</f>
       </c>
       <c r="R8" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R10),"",'ONR 1'!R10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R10),"",'ONR 1'!R10)</f>
       </c>
       <c r="S8" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S10),"",'ONR 1'!S10)</f>
+        <f>IF(ISBLANK('ONR 1'!S10),"",'ONR 1'!S10)</f>
       </c>
       <c r="T8" s="232" t="str">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T10),"",'ONR 1'!T10)</f>
+        <f>IF(ISBLANK('ONR 1'!T10),"",'ONR 1'!T10)</f>
       </c>
       <c r="U8" s="233" t="str">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U10),"",'ONR 1'!U10)</f>
+        <f>IF(ISBLANK('ONR 1'!U10),"",'ONR 1'!U10)</f>
       </c>
       <c r="V8" s="239" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G10),"",'ONR 1'!G10)</f>
+        <f>IF(ISBLANK('ONR 1'!G10),"",'ONR 1'!G10)</f>
       </c>
       <c r="W8" s="210" t="str">
         <f>IF(ISBLANK('ONR 1'!V10),"",'ONR 1'!V10)</f>
@@ -31696,42 +31623,34 @@
         <f>IF(ISBLANK('ONR 1'!W10),"",'ONR 1'!W10)</f>
       </c>
       <c r="Y8" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
+        <f>IF(ISBLANK('ONR 1'!I10),"",'ONR 1'!I10)</f>
       </c>
       <c r="Z8" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D10),"",'ONR 1'!D10)</f>
+        <f>IF(ISBLANK('ONR 1'!D10),"",'ONR 1'!D10)</f>
       </c>
       <c r="AE8" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T8),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T8),0,1)</f>
       </c>
       <c r="AF8" s="206" t="n">
-        <f t="shared" si="9">IF(L8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L8=TRUE,1,0)</f>
       </c>
       <c r="AG8" s="206" t="n">
-        <f t="shared" si="9">IF(M8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M8=TRUE,1,0)</f>
       </c>
       <c r="AH8" s="206" t="n">
-        <f t="shared" si="9">IF(N8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N8=TRUE,1,0)</f>
       </c>
       <c r="AI8" s="206" t="n">
-        <f t="shared" si="9">IF(O8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O8=TRUE,1,0)</f>
       </c>
       <c r="AJ8" s="206" t="n">
-        <f t="shared" si="9">IF(P8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P8=TRUE,1,0)</f>
       </c>
       <c r="AK8" s="206" t="n">
-        <f t="shared" si="9">IF(Q8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q8=TRUE,1,0)</f>
       </c>
       <c r="AL8" s="206" t="n">
-        <f t="shared" si="9">IF(R8=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R8=TRUE,1,0)</f>
       </c>
       <c r="AM8" t="n">
         <f>IF(LEN(TRIM(W8))&gt;0,1,0)</f>
@@ -31767,50 +31686,43 @@
         <f>IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
       </c>
       <c r="J9" s="232" t="str">
-        <f t="shared" si="10">IF(ISBLANK('ONR 1'!J11),"",'ONR 1'!J11)</f>
+        <f>IF(ISBLANK('ONR 1'!J11),"",'ONR 1'!J11)</f>
       </c>
       <c r="K9" s="233" t="str">
-        <f t="shared" si="1">IF(ISBLANK('ONR 1'!K11),"",'ONR 1'!K11)</f>
+        <f>IF(ISBLANK('ONR 1'!K11),"",'ONR 1'!K11)</f>
       </c>
       <c r="L9" s="233" t="b">
-        <f t="shared" si="11">IF(ISBLANK('ONR 1'!L11),"",'ONR 1'!L11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L11),"",'ONR 1'!L11)</f>
       </c>
       <c r="M9" s="233" t="b">
-        <f t="shared" si="12">IF(ISBLANK('ONR 1'!M11),"",'ONR 1'!M11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M11),"",'ONR 1'!M11)</f>
       </c>
       <c r="N9" s="233" t="b">
-        <f t="shared" si="13">IF(ISBLANK('ONR 1'!N11),"",'ONR 1'!N11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N11),"",'ONR 1'!N11)</f>
       </c>
       <c r="O9" s="233" t="b">
-        <f t="shared" si="14">IF(ISBLANK('ONR 1'!O11),"",'ONR 1'!O11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O11),"",'ONR 1'!O11)</f>
       </c>
       <c r="P9" s="233" t="b">
-        <f t="shared" si="15">IF(ISBLANK('ONR 1'!P11),"",'ONR 1'!P11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P11),"",'ONR 1'!P11)</f>
       </c>
       <c r="Q9" s="233" t="b">
-        <f t="shared" si="16">IF(ISBLANK('ONR 1'!Q11),"",'ONR 1'!Q11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q11),"",'ONR 1'!Q11)</f>
       </c>
       <c r="R9" s="233" t="b">
-        <f t="shared" si="17">IF(ISBLANK('ONR 1'!R11),"",'ONR 1'!R11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R11),"",'ONR 1'!R11)</f>
       </c>
       <c r="S9" s="234" t="str">
-        <f t="shared" si="2">IF(ISBLANK('ONR 1'!S11),"",'ONR 1'!S11)</f>
+        <f>IF(ISBLANK('ONR 1'!S11),"",'ONR 1'!S11)</f>
       </c>
       <c r="T9" s="232" t="str">
-        <f t="shared" si="3">IF(ISBLANK('ONR 1'!T11),"",'ONR 1'!T11)</f>
+        <f>IF(ISBLANK('ONR 1'!T11),"",'ONR 1'!T11)</f>
       </c>
       <c r="U9" s="233" t="str">
-        <f t="shared" si="4">IF(ISBLANK('ONR 1'!U11),"",'ONR 1'!U11)</f>
+        <f>IF(ISBLANK('ONR 1'!U11),"",'ONR 1'!U11)</f>
       </c>
       <c r="V9" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G11),"",'ONR 1'!G11)</f>
+        <f>IF(ISBLANK('ONR 1'!G11),"",'ONR 1'!G11)</f>
       </c>
       <c r="W9" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V11),"",'ONR 1'!V11)</f>
@@ -31819,42 +31731,34 @@
         <f>IF(ISBLANK('ONR 1'!W11),"",'ONR 1'!W11)</f>
       </c>
       <c r="Y9" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
+        <f>IF(ISBLANK('ONR 1'!I11),"",'ONR 1'!I11)</f>
       </c>
       <c r="Z9" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D11),"",'ONR 1'!D11)</f>
+        <f>IF(ISBLANK('ONR 1'!D11),"",'ONR 1'!D11)</f>
       </c>
       <c r="AE9" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T9),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T9),0,1)</f>
       </c>
       <c r="AF9" s="206" t="n">
-        <f t="shared" si="9">IF(L9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L9=TRUE,1,0)</f>
       </c>
       <c r="AG9" s="206" t="n">
-        <f t="shared" si="9">IF(M9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M9=TRUE,1,0)</f>
       </c>
       <c r="AH9" s="206" t="n">
-        <f t="shared" si="9">IF(N9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N9=TRUE,1,0)</f>
       </c>
       <c r="AI9" s="206" t="n">
-        <f t="shared" si="9">IF(O9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O9=TRUE,1,0)</f>
       </c>
       <c r="AJ9" s="206" t="n">
-        <f t="shared" si="9">IF(P9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P9=TRUE,1,0)</f>
       </c>
       <c r="AK9" s="206" t="n">
-        <f t="shared" si="9">IF(Q9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q9=TRUE,1,0)</f>
       </c>
       <c r="AL9" s="206" t="n">
-        <f t="shared" si="9">IF(R9=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R9=TRUE,1,0)</f>
       </c>
       <c r="AM9" t="n">
         <f>IF(LEN(TRIM(W9))&gt;0,1,0)</f>
@@ -31890,50 +31794,43 @@
         <f>IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
       </c>
       <c r="J10" s="232" t="str">
-        <f t="shared" ref="J10:J11" si="18">IF(ISBLANK('ONR 1'!J12),"",'ONR 1'!J12)</f>
+        <f>IF(ISBLANK('ONR 1'!J12),"",'ONR 1'!J12)</f>
       </c>
       <c r="K10" s="233" t="str">
-        <f t="shared" ref="K10:K11" si="19">IF(ISBLANK('ONR 1'!K12),"",'ONR 1'!K12)</f>
+        <f>IF(ISBLANK('ONR 1'!K12),"",'ONR 1'!K12)</f>
       </c>
       <c r="L10" s="233" t="b">
-        <f t="shared" ref="L10:L11" si="20">IF(ISBLANK('ONR 1'!L12),"",'ONR 1'!L12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!L12),"",'ONR 1'!L12)</f>
       </c>
       <c r="M10" s="233" t="b">
-        <f t="shared" ref="M10:M11" si="21">IF(ISBLANK('ONR 1'!M12),"",'ONR 1'!M12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M12),"",'ONR 1'!M12)</f>
       </c>
       <c r="N10" s="233" t="b">
-        <f t="shared" ref="N10:N11" si="22">IF(ISBLANK('ONR 1'!N12),"",'ONR 1'!N12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N12),"",'ONR 1'!N12)</f>
       </c>
       <c r="O10" s="233" t="b">
-        <f t="shared" ref="O10:O11" si="23">IF(ISBLANK('ONR 1'!O12),"",'ONR 1'!O12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O12),"",'ONR 1'!O12)</f>
       </c>
       <c r="P10" s="233" t="b">
-        <f t="shared" ref="P10:P11" si="24">IF(ISBLANK('ONR 1'!P12),"",'ONR 1'!P12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P12),"",'ONR 1'!P12)</f>
       </c>
       <c r="Q10" s="233" t="b">
-        <f t="shared" ref="Q10:Q11" si="25">IF(ISBLANK('ONR 1'!Q12),"",'ONR 1'!Q12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q12),"",'ONR 1'!Q12)</f>
       </c>
       <c r="R10" s="233" t="b">
-        <f t="shared" ref="R10:R11" si="26">IF(ISBLANK('ONR 1'!R12),"",'ONR 1'!R12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R12),"",'ONR 1'!R12)</f>
       </c>
       <c r="S10" s="234" t="str">
-        <f t="shared" ref="S10:S11" si="27">IF(ISBLANK('ONR 1'!S12),"",'ONR 1'!S12)</f>
+        <f>IF(ISBLANK('ONR 1'!S12),"",'ONR 1'!S12)</f>
       </c>
       <c r="T10" s="232" t="str">
-        <f t="shared" ref="T10:T11" si="28">IF(ISBLANK('ONR 1'!T12),"",'ONR 1'!T12)</f>
+        <f>IF(ISBLANK('ONR 1'!T12),"",'ONR 1'!T12)</f>
       </c>
       <c r="U10" s="233" t="str">
-        <f t="shared" ref="U10:U11" si="29">IF(ISBLANK('ONR 1'!U12),"",'ONR 1'!U12)</f>
+        <f>IF(ISBLANK('ONR 1'!U12),"",'ONR 1'!U12)</f>
       </c>
       <c r="V10" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G12),"",'ONR 1'!G12)</f>
+        <f>IF(ISBLANK('ONR 1'!G12),"",'ONR 1'!G12)</f>
       </c>
       <c r="W10" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V12),"",'ONR 1'!V12)</f>
@@ -31942,42 +31839,34 @@
         <f>IF(ISBLANK('ONR 1'!W12),"",'ONR 1'!W12)</f>
       </c>
       <c r="Y10" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
+        <f>IF(ISBLANK('ONR 1'!I12),"",'ONR 1'!I12)</f>
       </c>
       <c r="Z10" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D12),"",'ONR 1'!D12)</f>
+        <f>IF(ISBLANK('ONR 1'!D12),"",'ONR 1'!D12)</f>
       </c>
       <c r="AE10" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T10),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T10),0,1)</f>
       </c>
       <c r="AF10" s="206" t="n">
-        <f t="shared" si="9">IF(L10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L10=TRUE,1,0)</f>
       </c>
       <c r="AG10" s="206" t="n">
-        <f t="shared" si="9">IF(M10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M10=TRUE,1,0)</f>
       </c>
       <c r="AH10" s="206" t="n">
-        <f t="shared" si="9">IF(N10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N10=TRUE,1,0)</f>
       </c>
       <c r="AI10" s="206" t="n">
-        <f t="shared" si="9">IF(O10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O10=TRUE,1,0)</f>
       </c>
       <c r="AJ10" s="206" t="n">
-        <f t="shared" si="9">IF(P10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P10=TRUE,1,0)</f>
       </c>
       <c r="AK10" s="206" t="n">
-        <f t="shared" si="9">IF(Q10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q10=TRUE,1,0)</f>
       </c>
       <c r="AL10" s="206" t="n">
-        <f t="shared" si="9">IF(R10=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R10=TRUE,1,0)</f>
       </c>
       <c r="AM10" t="n">
         <f>IF(LEN(TRIM(W10))&gt;0,1,0)</f>
@@ -32021,56 +31910,43 @@
 Points faibles : elle connaît peu les méthodes pour mesurer et réduire la consommation de l’IA. Elle manque aussi de recul pour savoir quand l’IA est utile.</v>
       </c>
       <c r="J11" s="232" t="str">
-        <f t="shared" si="18">IF(ISBLANK('ONR 1'!J13),"",'ONR 1'!J13)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!J13),"",'ONR 1'!J13)</f>
       </c>
       <c r="K11" s="233" t="n">
-        <f t="shared" si="19">IF(ISBLANK('ONR 1'!K13),"",'ONR 1'!K13)</f>
-        <v>31</v>
+        <f>IF(ISBLANK('ONR 1'!K13),"",'ONR 1'!K13)</f>
       </c>
       <c r="L11" s="233" t="b">
-        <f t="shared" si="20">IF(ISBLANK('ONR 1'!L13),"",'ONR 1'!L13)</f>
-        <v>1</v>
+        <f>IF(ISBLANK('ONR 1'!L13),"",'ONR 1'!L13)</f>
       </c>
       <c r="M11" s="233" t="b">
-        <f t="shared" si="21">IF(ISBLANK('ONR 1'!M13),"",'ONR 1'!M13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!M13),"",'ONR 1'!M13)</f>
       </c>
       <c r="N11" s="233" t="b">
-        <f t="shared" si="22">IF(ISBLANK('ONR 1'!N13),"",'ONR 1'!N13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!N13),"",'ONR 1'!N13)</f>
       </c>
       <c r="O11" s="233" t="b">
-        <f t="shared" si="23">IF(ISBLANK('ONR 1'!O13),"",'ONR 1'!O13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!O13),"",'ONR 1'!O13)</f>
       </c>
       <c r="P11" s="233" t="b">
-        <f t="shared" si="24">IF(ISBLANK('ONR 1'!P13),"",'ONR 1'!P13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!P13),"",'ONR 1'!P13)</f>
       </c>
       <c r="Q11" s="233" t="b">
-        <f t="shared" si="25">IF(ISBLANK('ONR 1'!Q13),"",'ONR 1'!Q13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!Q13),"",'ONR 1'!Q13)</f>
       </c>
       <c r="R11" s="233" t="b">
-        <f t="shared" si="26">IF(ISBLANK('ONR 1'!R13),"",'ONR 1'!R13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 1'!R13),"",'ONR 1'!R13)</f>
       </c>
       <c r="S11" s="234" t="str">
-        <f t="shared" si="27">IF(ISBLANK('ONR 1'!S13),"",'ONR 1'!S13)</f>
-        <v>Intervention urgente</v>
+        <f>IF(ISBLANK('ONR 1'!S13),"",'ONR 1'!S13)</f>
       </c>
       <c r="T11" s="232" t="n">
-        <f t="shared" si="28">IF(ISBLANK('ONR 1'!T13),"",'ONR 1'!T13)</f>
-        <v>6</v>
+        <f>IF(ISBLANK('ONR 1'!T13),"",'ONR 1'!T13)</f>
       </c>
       <c r="U11" s="233" t="n">
-        <f t="shared" si="29">IF(ISBLANK('ONR 1'!U13),"",'ONR 1'!U13)</f>
-        <v>62</v>
+        <f>IF(ISBLANK('ONR 1'!U13),"",'ONR 1'!U13)</f>
       </c>
       <c r="V11" s="241" t="str">
-        <f t="shared" si="5">IF(ISBLANK('ONR 1'!G13),"",'ONR 1'!G13)</f>
-        <v>Les équipes métiers expérimentent plusieurs projets d’IA générative, dont des usages de ChatGPT. Elles ne mesurent pas leur impact énergétique et ne disposent pas de charte pour encadrer les besoins et les usages.</v>
+        <f>IF(ISBLANK('ONR 1'!G13),"",'ONR 1'!G13)</f>
       </c>
       <c r="W11" s="241" t="str">
         <f>IF(ISBLANK('ONR 1'!V13),"",'ONR 1'!V13)</f>
@@ -32082,46 +31958,34 @@
         <f>IF(ISBLANK('ONR 1'!W13),"",'ONR 1'!W13)</f>
       </c>
       <c r="Y11" s="236" t="str">
-        <f t="shared" si="6">IF(ISBLANK('ONR 1'!I13),"",'ONR 1'!I13)</f>
-        <v>Point fort : l’équipe chargée des données et de l’informatique dispose de compétences techniques et souhaite explorer ces outils.
-Points faibles : elle connaît peu les méthodes pour mesurer et réduire la consommation de l’IA. Elle manque aussi de recul pour savoir quand l’IA est utile.</v>
+        <f>IF(ISBLANK('ONR 1'!I13),"",'ONR 1'!I13)</f>
       </c>
       <c r="Z11" s="236" t="str">
-        <f t="shared" si="7">IF(ISBLANK('ONR 1'!D13),"",'ONR 1'!D13)</f>
-        <v>Avantages possibles : maîtriser les coûts du matériel et des services d’IA, et réduire les émissions de gaz à effet de serre liées à leur entraînement et à leur utilisation.
-Risque : utiliser l’IA par effet de mode, sans besoin réel, et consommer davantage de ressources.</v>
+        <f>IF(ISBLANK('ONR 1'!D13),"",'ONR 1'!D13)</f>
       </c>
       <c r="AE11" s="206" t="n">
-        <f t="shared" si="8">IF(ISNUMBER(T11),0,1)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(T11),0,1)</f>
       </c>
       <c r="AF11" s="206" t="n">
-        <f t="shared" si="9">IF(L11=TRUE,1,0)</f>
-        <v>1</v>
+        <f>IF(L11=TRUE,1,0)</f>
       </c>
       <c r="AG11" s="206" t="n">
-        <f t="shared" si="9">IF(M11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M11=TRUE,1,0)</f>
       </c>
       <c r="AH11" s="206" t="n">
-        <f t="shared" si="9">IF(N11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N11=TRUE,1,0)</f>
       </c>
       <c r="AI11" s="206" t="n">
-        <f t="shared" si="9">IF(O11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O11=TRUE,1,0)</f>
       </c>
       <c r="AJ11" s="206" t="n">
-        <f t="shared" si="9">IF(P11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P11=TRUE,1,0)</f>
       </c>
       <c r="AK11" s="206" t="n">
-        <f t="shared" si="9">IF(Q11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q11=TRUE,1,0)</f>
       </c>
       <c r="AL11" s="206" t="n">
-        <f t="shared" si="9">IF(R11=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R11=TRUE,1,0)</f>
       </c>
       <c r="AM11" t="n">
         <f>IF(LEN(TRIM(W11))&gt;0,1,0)</f>
@@ -32379,7 +32243,7 @@
         <f>IF(ISBLANK('ONR 2'!J7),"",'ONR 2'!J7)</f>
       </c>
       <c r="K14" s="227" t="str">
-        <f t="shared" ref="K14" si="31">IF(ISBLANK('ONR 2'!K7),"",'ONR 2'!K7)</f>
+        <f>IF(ISBLANK('ONR 2'!K7),"",'ONR 2'!K7)</f>
       </c>
       <c r="L14" s="227" t="b">
         <f>IF(ISBLANK('ONR 2'!L7),"",'ONR 2'!L7)</f>
@@ -32410,13 +32274,13 @@
         <v>0</v>
       </c>
       <c r="S14" s="228" t="str">
-        <f t="shared" ref="S14" si="32">IF(ISBLANK('ONR 2'!S7),"",'ONR 2'!S7)</f>
+        <f>IF(ISBLANK('ONR 2'!S7),"",'ONR 2'!S7)</f>
       </c>
       <c r="T14" s="226" t="str">
-        <f t="shared" ref="T14" si="33">IF(ISBLANK('ONR 2'!T7),"",'ONR 2'!T7)</f>
+        <f>IF(ISBLANK('ONR 2'!T7),"",'ONR 2'!T7)</f>
       </c>
       <c r="U14" s="242" t="str">
-        <f t="shared" ref="U14" si="34">IF(ISBLANK('ONR 2'!U7),"",'ONR 2'!U7)</f>
+        <f>IF(ISBLANK('ONR 2'!U7),"",'ONR 2'!U7)</f>
       </c>
       <c r="V14" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!G7),"",'ONR 2'!G7)</f>
@@ -32438,32 +32302,25 @@
         <v>1</v>
       </c>
       <c r="AF14" s="206" t="n">
-        <f t="shared" ref="AF14:AL17" si="35">IF(L14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L14=TRUE,1,0)</f>
       </c>
       <c r="AG14" s="206" t="n">
-        <f t="shared" si="35">IF(M14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M14=TRUE,1,0)</f>
       </c>
       <c r="AH14" s="206" t="n">
-        <f t="shared" si="35">IF(N14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N14=TRUE,1,0)</f>
       </c>
       <c r="AI14" s="206" t="n">
-        <f t="shared" si="35">IF(O14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O14=TRUE,1,0)</f>
       </c>
       <c r="AJ14" s="206" t="n">
-        <f t="shared" si="35">IF(P14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P14=TRUE,1,0)</f>
       </c>
       <c r="AK14" s="206" t="n">
-        <f t="shared" si="35">IF(Q14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q14=TRUE,1,0)</f>
       </c>
       <c r="AL14" s="206" t="n">
-        <f t="shared" si="35">IF(R14=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R14=TRUE,1,0)</f>
       </c>
       <c r="AM14" t="n">
         <f>IF(LEN(TRIM(W14))&gt;0,1,0)</f>
@@ -32499,47 +32356,40 @@
         <f>IF(ISBLANK('ONR 2'!I8),"",'ONR 2'!I8)</f>
       </c>
       <c r="J15" s="218" t="str">
-        <f t="shared" ref="J15:J17" si="36">IF(ISBLANK('ONR 2'!J8),"",'ONR 2'!J8)</f>
+        <f>IF(ISBLANK('ONR 2'!J8),"",'ONR 2'!J8)</f>
       </c>
       <c r="K15" s="227" t="str">
-        <f t="shared" ref="K15:K17" si="37">IF(ISBLANK('ONR 2'!K8),"",'ONR 2'!K8)</f>
+        <f>IF(ISBLANK('ONR 2'!K8),"",'ONR 2'!K8)</f>
       </c>
       <c r="L15" s="227" t="b">
-        <f t="shared" ref="L15:L17" si="38">IF(ISBLANK('ONR 2'!L8),"",'ONR 2'!L8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!L8),"",'ONR 2'!L8)</f>
       </c>
       <c r="M15" s="227" t="b">
-        <f t="shared" ref="M15:M17" si="39">IF(ISBLANK('ONR 2'!M8),"",'ONR 2'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!M8),"",'ONR 2'!M8)</f>
       </c>
       <c r="N15" s="227" t="b">
-        <f t="shared" ref="N15:N17" si="40">IF(ISBLANK('ONR 2'!N8),"",'ONR 2'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!N8),"",'ONR 2'!N8)</f>
       </c>
       <c r="O15" s="227" t="b">
-        <f t="shared" ref="O15:O17" si="41">IF(ISBLANK('ONR 2'!O8),"",'ONR 2'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!O8),"",'ONR 2'!O8)</f>
       </c>
       <c r="P15" s="227" t="b">
-        <f t="shared" ref="P15:P17" si="42">IF(ISBLANK('ONR 2'!P8),"",'ONR 2'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!P8),"",'ONR 2'!P8)</f>
       </c>
       <c r="Q15" s="227" t="b">
-        <f t="shared" ref="Q15:Q17" si="43">IF(ISBLANK('ONR 2'!Q8),"",'ONR 2'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!Q8),"",'ONR 2'!Q8)</f>
       </c>
       <c r="R15" s="227" t="b">
-        <f t="shared" ref="R15:R17" si="44">IF(ISBLANK('ONR 2'!R8),"",'ONR 2'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 2'!R8),"",'ONR 2'!R8)</f>
       </c>
       <c r="S15" s="228" t="str">
-        <f t="shared" ref="S15:S17" si="45">IF(ISBLANK('ONR 2'!S8),"",'ONR 2'!S8)</f>
+        <f>IF(ISBLANK('ONR 2'!S8),"",'ONR 2'!S8)</f>
       </c>
       <c r="T15" s="226" t="str">
-        <f t="shared" ref="T15:T17" si="46">IF(ISBLANK('ONR 2'!T8),"",'ONR 2'!T8)</f>
+        <f>IF(ISBLANK('ONR 2'!T8),"",'ONR 2'!T8)</f>
       </c>
       <c r="U15" s="242" t="str">
-        <f t="shared" ref="U15:U17" si="47">IF(ISBLANK('ONR 2'!U8),"",'ONR 2'!U8)</f>
+        <f>IF(ISBLANK('ONR 2'!U8),"",'ONR 2'!U8)</f>
       </c>
       <c r="V15" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!G8),"",'ONR 2'!G8)</f>
@@ -32561,32 +32411,25 @@
         <v>1</v>
       </c>
       <c r="AF15" s="206" t="n">
-        <f t="shared" si="35">IF(L15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L15=TRUE,1,0)</f>
       </c>
       <c r="AG15" s="206" t="n">
-        <f t="shared" si="35">IF(M15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M15=TRUE,1,0)</f>
       </c>
       <c r="AH15" s="206" t="n">
-        <f t="shared" si="35">IF(N15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N15=TRUE,1,0)</f>
       </c>
       <c r="AI15" s="206" t="n">
-        <f t="shared" si="35">IF(O15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O15=TRUE,1,0)</f>
       </c>
       <c r="AJ15" s="206" t="n">
-        <f t="shared" si="35">IF(P15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P15=TRUE,1,0)</f>
       </c>
       <c r="AK15" s="206" t="n">
-        <f t="shared" si="35">IF(Q15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q15=TRUE,1,0)</f>
       </c>
       <c r="AL15" s="206" t="n">
-        <f t="shared" si="35">IF(R15=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R15=TRUE,1,0)</f>
       </c>
       <c r="AM15" t="n">
         <f>IF(LEN(TRIM(W15))&gt;0,1,0)</f>
@@ -32622,90 +32465,47 @@
         <f>IF(ISBLANK('ONR 2'!I9),"",'ONR 2'!I9)</f>
       </c>
       <c r="J16" s="218" t="str">
-        <f t="shared" si="36">IF(ISBLANK('ONR 2'!J9),"",'ONR 2'!J9)</f>
-      </c>
-      <c r="K17" s="227" t="str">
-        <f t="shared" si="37">IF(ISBLANK('ONR 2'!K10),"",'ONR 2'!K10)</f>
+        <f>IF(ISBLANK('ONR 2'!J9),"",'ONR 2'!J9)</f>
       </c>
       <c r="K16" t="str" s="227">
         <f>IF(ISBLANK('ONR 2'!K9),"",'ONR 2'!K9)</f>
-      </c>
-      <c r="L17" s="227" t="b">
-        <f t="shared" si="38">IF(ISBLANK('ONR 2'!L10),"",'ONR 2'!L10)</f>
-        <v>0</v>
       </c>
       <c r="L16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!L9),"",'ONR 2'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M17" s="227" t="b">
-        <f t="shared" si="39">IF(ISBLANK('ONR 2'!M10),"",'ONR 2'!M10)</f>
-        <v>0</v>
-      </c>
       <c r="M16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!M9),"",'ONR 2'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N17" s="227" t="b">
-        <f t="shared" si="40">IF(ISBLANK('ONR 2'!N10),"",'ONR 2'!N10)</f>
-        <v>0</v>
-      </c>
       <c r="N16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!N9),"",'ONR 2'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O17" s="227" t="b">
-        <f t="shared" si="41">IF(ISBLANK('ONR 2'!O10),"",'ONR 2'!O10)</f>
-        <v>0</v>
-      </c>
       <c r="O16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!O9),"",'ONR 2'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P17" s="227" t="b">
-        <f t="shared" si="42">IF(ISBLANK('ONR 2'!P10),"",'ONR 2'!P10)</f>
-        <v>0</v>
-      </c>
       <c r="P16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!P9),"",'ONR 2'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="227" t="b">
-        <f t="shared" si="43">IF(ISBLANK('ONR 2'!Q10),"",'ONR 2'!Q10)</f>
-        <v>0</v>
-      </c>
       <c r="Q16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!Q9),"",'ONR 2'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R17" s="227" t="b">
-        <f t="shared" si="44">IF(ISBLANK('ONR 2'!R10),"",'ONR 2'!R10)</f>
-        <v>0</v>
-      </c>
       <c r="R16" t="b" s="227">
         <f>IF(ISBLANK('ONR 2'!R9),"",'ONR 2'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S17" s="228" t="str">
-        <f t="shared" si="45">IF(ISBLANK('ONR 2'!S10),"",'ONR 2'!S10)</f>
-      </c>
       <c r="S16" t="str" s="228">
         <f>IF(ISBLANK('ONR 2'!S9),"",'ONR 2'!S9)</f>
       </c>
-      <c r="T17" s="226" t="str">
-        <f t="shared" si="46">IF(ISBLANK('ONR 2'!T10),"",'ONR 2'!T10)</f>
-      </c>
       <c r="T16" t="str" s="226">
         <f>IF(ISBLANK('ONR 2'!T9),"",'ONR 2'!T9)</f>
       </c>
-      <c r="U17" s="242" t="str">
-        <f t="shared" si="47">IF(ISBLANK('ONR 2'!U10),"",'ONR 2'!U10)</f>
-      </c>
       <c r="U16" t="str" s="242">
         <f>IF(ISBLANK('ONR 2'!U9),"",'ONR 2'!U9)</f>
-      </c>
-      <c r="V17" s="229" t="str">
-        <f>IF(ISBLANK('ONR 2'!G10),"",'ONR 2'!G10)</f>
       </c>
       <c r="V16" t="str" s="229">
         <f>IF(ISBLANK('ONR 2'!G9),"",'ONR 2'!G9)</f>
@@ -32727,32 +32527,25 @@
         <v>1</v>
       </c>
       <c r="AF16" s="206" t="n">
-        <f t="shared" si="35">IF(L16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L16=TRUE,1,0)</f>
       </c>
       <c r="AG16" s="206" t="n">
-        <f t="shared" si="35">IF(M16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M16=TRUE,1,0)</f>
       </c>
       <c r="AH16" s="206" t="n">
-        <f t="shared" si="35">IF(N16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N16=TRUE,1,0)</f>
       </c>
       <c r="AI16" s="206" t="n">
-        <f t="shared" si="35">IF(O16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O16=TRUE,1,0)</f>
       </c>
       <c r="AJ16" s="206" t="n">
-        <f t="shared" si="35">IF(P16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P16=TRUE,1,0)</f>
       </c>
       <c r="AK16" s="206" t="n">
-        <f t="shared" si="35">IF(Q16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q16=TRUE,1,0)</f>
       </c>
       <c r="AL16" s="206" t="n">
-        <f t="shared" si="35">IF(R16=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R16=TRUE,1,0)</f>
       </c>
       <c r="AM16" t="n">
         <f>IF(LEN(TRIM(W16))&gt;0,1,0)</f>
@@ -32788,43 +32581,43 @@
         <f>IF(ISBLANK('ONR 2'!I10),"",'ONR 2'!I10)</f>
       </c>
       <c r="J17" s="218" t="str">
-        <f t="shared" si="36">IF(ISBLANK('ONR 2'!J10),"",'ONR 2'!J10)</f>
-      </c>
-      <c r="K19" s="227">
-        <f t="shared" si="37"/>
-      </c>
-      <c r="L19" s="227">
-        <f t="shared" si="38"/>
-      </c>
-      <c r="M19" s="227">
-        <f t="shared" si="39"/>
-      </c>
-      <c r="N19" s="227">
-        <f t="shared" si="40"/>
-      </c>
-      <c r="O19" s="227">
-        <f t="shared" si="41"/>
-      </c>
-      <c r="P19" s="227">
-        <f t="shared" si="42"/>
-      </c>
-      <c r="Q19" s="227">
-        <f t="shared" si="43"/>
-      </c>
-      <c r="R19" s="227">
-        <f t="shared" si="44"/>
-      </c>
-      <c r="S19" s="228">
-        <f t="shared" si="45"/>
-      </c>
-      <c r="T19" s="226">
-        <f t="shared" si="46"/>
-      </c>
-      <c r="U19" s="242">
-        <f t="shared" si="47"/>
-      </c>
-      <c r="V19" s="229">
-        <f>G17</f>
+        <f>IF(ISBLANK('ONR 2'!J10),"",'ONR 2'!J10)</f>
+      </c>
+      <c r="K17" s="227" t="str">
+        <f>IF(ISBLANK('ONR 2'!K10),"",'ONR 2'!K10)</f>
+      </c>
+      <c r="L17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!L10),"",'ONR 2'!L10)</f>
+      </c>
+      <c r="M17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!M10),"",'ONR 2'!M10)</f>
+      </c>
+      <c r="N17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!N10),"",'ONR 2'!N10)</f>
+      </c>
+      <c r="O17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!O10),"",'ONR 2'!O10)</f>
+      </c>
+      <c r="P17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!P10),"",'ONR 2'!P10)</f>
+      </c>
+      <c r="Q17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!Q10),"",'ONR 2'!Q10)</f>
+      </c>
+      <c r="R17" s="227" t="b">
+        <f>IF(ISBLANK('ONR 2'!R10),"",'ONR 2'!R10)</f>
+      </c>
+      <c r="S17" s="228" t="str">
+        <f>IF(ISBLANK('ONR 2'!S10),"",'ONR 2'!S10)</f>
+      </c>
+      <c r="T17" s="226" t="str">
+        <f>IF(ISBLANK('ONR 2'!T10),"",'ONR 2'!T10)</f>
+      </c>
+      <c r="U17" s="242" t="str">
+        <f>IF(ISBLANK('ONR 2'!U10),"",'ONR 2'!U10)</f>
+      </c>
+      <c r="V17" s="229" t="str">
+        <f>IF(ISBLANK('ONR 2'!G10),"",'ONR 2'!G10)</f>
       </c>
       <c r="W17" s="229" t="str">
         <f>IF(ISBLANK('ONR 2'!V10),"",'ONR 2'!V10)</f>
@@ -32843,32 +32636,25 @@
         <v>1</v>
       </c>
       <c r="AF17" s="206" t="n">
-        <f t="shared" si="35">IF(L17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L17=TRUE,1,0)</f>
       </c>
       <c r="AG17" s="206" t="n">
-        <f t="shared" si="35">IF(M17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M17=TRUE,1,0)</f>
       </c>
       <c r="AH17" s="206" t="n">
-        <f t="shared" si="35">IF(N17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N17=TRUE,1,0)</f>
       </c>
       <c r="AI17" s="206" t="n">
-        <f t="shared" si="35">IF(O17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O17=TRUE,1,0)</f>
       </c>
       <c r="AJ17" s="206" t="n">
-        <f t="shared" si="35">IF(P17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P17=TRUE,1,0)</f>
       </c>
       <c r="AK17" s="206" t="n">
-        <f t="shared" si="35">IF(Q17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q17=TRUE,1,0)</f>
       </c>
       <c r="AL17" s="206" t="n">
-        <f t="shared" si="35">IF(R17=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R17=TRUE,1,0)</f>
       </c>
       <c r="AM17" t="n">
         <f>IF(LEN(TRIM(W17))&gt;0,1,0)</f>
@@ -33103,50 +32889,43 @@
         <f>IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
       </c>
       <c r="J20" s="246" t="str">
-        <f t="shared" ref="J20:J25" si="49">IF(ISBLANK('ONR 3'!J7),"",'ONR 3'!J7)</f>
+        <f>IF(ISBLANK('ONR 3'!J7),"",'ONR 3'!J7)</f>
       </c>
       <c r="K20" s="247" t="str">
-        <f t="shared" ref="K20:K25" si="50">IF(ISBLANK('ONR 3'!K7),"",'ONR 3'!K7)</f>
+        <f>IF(ISBLANK('ONR 3'!K7),"",'ONR 3'!K7)</f>
       </c>
       <c r="L20" s="247" t="b">
-        <f t="shared" ref="L20:L25" si="51">IF(ISBLANK('ONR 3'!L7),"",'ONR 3'!L7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!L7),"",'ONR 3'!L7)</f>
       </c>
       <c r="M20" s="247" t="b">
-        <f t="shared" ref="M20:M25" si="52">IF(ISBLANK('ONR 3'!M7),"",'ONR 3'!M7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!M7),"",'ONR 3'!M7)</f>
       </c>
       <c r="N20" s="247" t="b">
-        <f t="shared" ref="N20:N25" si="53">IF(ISBLANK('ONR 3'!N7),"",'ONR 3'!N7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!N7),"",'ONR 3'!N7)</f>
       </c>
       <c r="O20" s="247" t="b">
-        <f t="shared" ref="O20:O25" si="54">IF(ISBLANK('ONR 3'!O7),"",'ONR 3'!O7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!O7),"",'ONR 3'!O7)</f>
       </c>
       <c r="P20" s="247" t="b">
-        <f t="shared" ref="P20:P25" si="55">IF(ISBLANK('ONR 3'!P7),"",'ONR 3'!P7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!P7),"",'ONR 3'!P7)</f>
       </c>
       <c r="Q20" s="247" t="b">
-        <f t="shared" ref="Q20:Q25" si="56">IF(ISBLANK('ONR 3'!Q7),"",'ONR 3'!Q7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!Q7),"",'ONR 3'!Q7)</f>
       </c>
       <c r="R20" s="247" t="b">
-        <f t="shared" ref="R20:R25" si="57">IF(ISBLANK('ONR 3'!R7),"",'ONR 3'!R7)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!R7),"",'ONR 3'!R7)</f>
       </c>
       <c r="S20" s="248" t="str">
-        <f t="shared" ref="S20:S25" si="58">IF(ISBLANK('ONR 3'!S7),"",'ONR 3'!S7)</f>
+        <f>IF(ISBLANK('ONR 3'!S7),"",'ONR 3'!S7)</f>
       </c>
       <c r="T20" s="249" t="str">
-        <f t="shared" ref="T20:T25" si="59">IF(ISBLANK('ONR 3'!T7),"",'ONR 3'!T7)</f>
+        <f>IF(ISBLANK('ONR 3'!T7),"",'ONR 3'!T7)</f>
       </c>
       <c r="U20" s="250" t="str">
-        <f t="shared" ref="U20:U25" si="60">IF(ISBLANK('ONR 3'!U7),"",'ONR 3'!U7)</f>
+        <f>IF(ISBLANK('ONR 3'!U7),"",'ONR 3'!U7)</f>
       </c>
       <c r="V20" s="235" t="str">
-        <f t="shared" ref="V20:V26" si="61">IF(ISBLANK('ONR 3'!G7),"",'ONR 3'!G7)</f>
+        <f>IF(ISBLANK('ONR 3'!G7),"",'ONR 3'!G7)</f>
       </c>
       <c r="W20" s="235" t="str">
         <f>IF(ISBLANK('ONR 3'!V7),"",'ONR 3'!V7)</f>
@@ -33155,42 +32934,34 @@
         <f>IF(ISBLANK('ONR 3'!W7),"",'ONR 3'!W7)</f>
       </c>
       <c r="Y20" s="236" t="str">
-        <f t="shared" ref="Y20:Y26" si="62">IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
+        <f>IF(ISBLANK('ONR 3'!I7),"",'ONR 3'!I7)</f>
       </c>
       <c r="Z20" s="236" t="str">
-        <f t="shared" ref="Z20:Z26" si="63">IF(ISBLANK('ONR 3'!D7),"",'ONR 3'!D7)</f>
+        <f>IF(ISBLANK('ONR 3'!D7),"",'ONR 3'!D7)</f>
       </c>
       <c r="AE20" s="206" t="n">
-        <f t="shared" ref="AE20:AE26" si="64">IF(ISNUMBER(T20),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T20),0,1)</f>
       </c>
       <c r="AF20" s="206" t="n">
-        <f t="shared" ref="AF20:AL26" si="65">IF(L20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L20=TRUE,1,0)</f>
       </c>
       <c r="AG20" s="206" t="n">
-        <f t="shared" si="65">IF(M20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M20=TRUE,1,0)</f>
       </c>
       <c r="AH20" s="206" t="n">
-        <f t="shared" si="65">IF(N20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N20=TRUE,1,0)</f>
       </c>
       <c r="AI20" s="206" t="n">
-        <f t="shared" si="65">IF(O20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O20=TRUE,1,0)</f>
       </c>
       <c r="AJ20" s="206" t="n">
-        <f t="shared" si="65">IF(P20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P20=TRUE,1,0)</f>
       </c>
       <c r="AK20" s="206" t="n">
-        <f t="shared" si="65">IF(Q20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q20=TRUE,1,0)</f>
       </c>
       <c r="AL20" s="206" t="n">
-        <f t="shared" si="65">IF(R20=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R20=TRUE,1,0)</f>
       </c>
       <c r="AM20" t="n">
         <f>IF(LEN(TRIM(W20))&gt;0,1,0)</f>
@@ -33226,97 +32997,51 @@
         <f>IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
       </c>
       <c r="J21" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J8),"",'ONR 3'!J8)</f>
-      </c>
-      <c r="K23" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K10),"",'ONR 3'!K10)</f>
+        <f>IF(ISBLANK('ONR 3'!J8),"",'ONR 3'!J8)</f>
       </c>
       <c r="K21" t="str" s="247">
         <f>IF(ISBLANK('ONR 3'!K8),"",'ONR 3'!K8)</f>
-      </c>
-      <c r="L23" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L10),"",'ONR 3'!L10)</f>
-        <v>0</v>
       </c>
       <c r="L21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!L8),"",'ONR 3'!L8)</f>
         <v>0</v>
       </c>
-      <c r="M23" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M10),"",'ONR 3'!M10)</f>
-        <v>0</v>
-      </c>
       <c r="M21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!M8),"",'ONR 3'!M8)</f>
         <v>0</v>
       </c>
-      <c r="N23" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N10),"",'ONR 3'!N10)</f>
-        <v>0</v>
-      </c>
       <c r="N21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!N8),"",'ONR 3'!N8)</f>
         <v>0</v>
       </c>
-      <c r="O23" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O10),"",'ONR 3'!O10)</f>
-        <v>0</v>
-      </c>
       <c r="O21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!O8),"",'ONR 3'!O8)</f>
         <v>0</v>
       </c>
-      <c r="P23" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P10),"",'ONR 3'!P10)</f>
-        <v>0</v>
-      </c>
       <c r="P21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!P8),"",'ONR 3'!P8)</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q10),"",'ONR 3'!Q10)</f>
-        <v>0</v>
-      </c>
       <c r="Q21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!Q8),"",'ONR 3'!Q8)</f>
         <v>0</v>
       </c>
-      <c r="R23" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R10),"",'ONR 3'!R10)</f>
-        <v>0</v>
-      </c>
       <c r="R21" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!R8),"",'ONR 3'!R8)</f>
         <v>0</v>
       </c>
-      <c r="S23" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S10),"",'ONR 3'!S10)</f>
-      </c>
       <c r="S21" t="str" s="248">
         <f>IF(ISBLANK('ONR 3'!S8),"",'ONR 3'!S8)</f>
       </c>
-      <c r="T23" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T10),"",'ONR 3'!T10)</f>
-      </c>
       <c r="T21" t="str" s="249">
         <f>IF(ISBLANK('ONR 3'!T8),"",'ONR 3'!T8)</f>
       </c>
-      <c r="U23" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U10),"",'ONR 3'!U10)</f>
-      </c>
       <c r="U21" t="str" s="250">
         <f>IF(ISBLANK('ONR 3'!U8),"",'ONR 3'!U8)</f>
       </c>
-      <c r="V23" s="235" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G10),"",'ONR 3'!G10)</f>
-      </c>
       <c r="V21" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!G8),"",'ONR 3'!G8)</f>
       </c>
-      <c r="W23" s="235" t="str">
-        <f>IF(ISBLANK('ONR 3'!V10),"",'ONR 3'!V10)</f>
-      </c>
       <c r="W21" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!V8),"",'ONR 3'!V8)</f>
       </c>
@@ -33324,42 +33049,34 @@
         <f>IF(ISBLANK('ONR 3'!W8),"",'ONR 3'!W8)</f>
       </c>
       <c r="Y21" s="236" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
+        <f>IF(ISBLANK('ONR 3'!I8),"",'ONR 3'!I8)</f>
       </c>
       <c r="Z21" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D8),"",'ONR 3'!D8)</f>
+        <f>IF(ISBLANK('ONR 3'!D8),"",'ONR 3'!D8)</f>
       </c>
       <c r="AE21" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T21),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T21),0,1)</f>
       </c>
       <c r="AF21" s="206" t="n">
-        <f t="shared" si="65">IF(L21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L21=TRUE,1,0)</f>
       </c>
       <c r="AG21" s="206" t="n">
-        <f t="shared" si="65">IF(M21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M21=TRUE,1,0)</f>
       </c>
       <c r="AH21" s="206" t="n">
-        <f t="shared" si="65">IF(N21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N21=TRUE,1,0)</f>
       </c>
       <c r="AI21" s="206" t="n">
-        <f t="shared" si="65">IF(O21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O21=TRUE,1,0)</f>
       </c>
       <c r="AJ21" s="206" t="n">
-        <f t="shared" si="65">IF(P21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P21=TRUE,1,0)</f>
       </c>
       <c r="AK21" s="206" t="n">
-        <f t="shared" si="65">IF(Q21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q21=TRUE,1,0)</f>
       </c>
       <c r="AL21" s="206" t="n">
-        <f t="shared" si="65">IF(R21=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R21=TRUE,1,0)</f>
       </c>
       <c r="AM21" t="n">
         <f>IF(LEN(TRIM(W21))&gt;0,1,0)</f>
@@ -33395,97 +33112,51 @@
         <f>IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
       </c>
       <c r="J22" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J9),"",'ONR 3'!J9)</f>
-      </c>
-      <c r="K24" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K11),"",'ONR 3'!K11)</f>
+        <f>IF(ISBLANK('ONR 3'!J9),"",'ONR 3'!J9)</f>
       </c>
       <c r="K22" t="str" s="247">
         <f>IF(ISBLANK('ONR 3'!K9),"",'ONR 3'!K9)</f>
-      </c>
-      <c r="L24" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L11),"",'ONR 3'!L11)</f>
-        <v>0</v>
       </c>
       <c r="L22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!L9),"",'ONR 3'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M24" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M11),"",'ONR 3'!M11)</f>
-        <v>0</v>
-      </c>
       <c r="M22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!M9),"",'ONR 3'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N24" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N11),"",'ONR 3'!N11)</f>
-        <v>0</v>
-      </c>
       <c r="N22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!N9),"",'ONR 3'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O24" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O11),"",'ONR 3'!O11)</f>
-        <v>0</v>
-      </c>
       <c r="O22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!O9),"",'ONR 3'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P24" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P11),"",'ONR 3'!P11)</f>
-        <v>0</v>
-      </c>
       <c r="P22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!P9),"",'ONR 3'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q24" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q11),"",'ONR 3'!Q11)</f>
-        <v>0</v>
-      </c>
       <c r="Q22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!Q9),"",'ONR 3'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R24" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R11),"",'ONR 3'!R11)</f>
-        <v>0</v>
-      </c>
       <c r="R22" t="b" s="247">
         <f>IF(ISBLANK('ONR 3'!R9),"",'ONR 3'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S24" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S11),"",'ONR 3'!S11)</f>
-      </c>
       <c r="S22" t="str" s="248">
         <f>IF(ISBLANK('ONR 3'!S9),"",'ONR 3'!S9)</f>
       </c>
-      <c r="T24" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T11),"",'ONR 3'!T11)</f>
-      </c>
       <c r="T22" t="str" s="249">
         <f>IF(ISBLANK('ONR 3'!T9),"",'ONR 3'!T9)</f>
       </c>
-      <c r="U24" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U11),"",'ONR 3'!U11)</f>
-      </c>
       <c r="U22" t="str" s="250">
         <f>IF(ISBLANK('ONR 3'!U9),"",'ONR 3'!U9)</f>
       </c>
-      <c r="V24" s="235" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G11),"",'ONR 3'!G11)</f>
-      </c>
       <c r="V22" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!G9),"",'ONR 3'!G9)</f>
       </c>
-      <c r="W24" s="235" t="str">
-        <f>IF(ISBLANK('ONR 3'!V11),"",'ONR 3'!V11)</f>
-      </c>
       <c r="W22" t="str" s="235">
         <f>IF(ISBLANK('ONR 3'!V9),"",'ONR 3'!V9)</f>
       </c>
@@ -33493,42 +33164,34 @@
         <f>IF(ISBLANK('ONR 3'!W9),"",'ONR 3'!W9)</f>
       </c>
       <c r="Y22" s="236" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
+        <f>IF(ISBLANK('ONR 3'!I9),"",'ONR 3'!I9)</f>
       </c>
       <c r="Z22" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D9),"",'ONR 3'!D9)</f>
+        <f>IF(ISBLANK('ONR 3'!D9),"",'ONR 3'!D9)</f>
       </c>
       <c r="AE22" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T22),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T22),0,1)</f>
       </c>
       <c r="AF22" s="206" t="n">
-        <f t="shared" si="65">IF(L22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L22=TRUE,1,0)</f>
       </c>
       <c r="AG22" s="206" t="n">
-        <f t="shared" si="65">IF(M22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M22=TRUE,1,0)</f>
       </c>
       <c r="AH22" s="206" t="n">
-        <f t="shared" si="65">IF(N22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N22=TRUE,1,0)</f>
       </c>
       <c r="AI22" s="206" t="n">
-        <f t="shared" si="65">IF(O22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O22=TRUE,1,0)</f>
       </c>
       <c r="AJ22" s="206" t="n">
-        <f t="shared" si="65">IF(P22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P22=TRUE,1,0)</f>
       </c>
       <c r="AK22" s="206" t="n">
-        <f t="shared" si="65">IF(Q22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q22=TRUE,1,0)</f>
       </c>
       <c r="AL22" s="206" t="n">
-        <f t="shared" si="65">IF(R22=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R22=TRUE,1,0)</f>
       </c>
       <c r="AM22" t="n">
         <f>IF(LEN(TRIM(W22))&gt;0,1,0)</f>
@@ -33564,94 +33227,79 @@
         <f>IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
       </c>
       <c r="J23" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J10),"",'ONR 3'!J10)</f>
-      </c>
-      <c r="K25" s="247" t="str">
-        <f t="shared" si="50">IF(ISBLANK('ONR 3'!K12),"",'ONR 3'!K12)</f>
-      </c>
-      <c r="L25" s="247" t="b">
-        <f t="shared" si="51">IF(ISBLANK('ONR 3'!L12),"",'ONR 3'!L12)</f>
-        <v>0</v>
-      </c>
-      <c r="M25" s="247" t="b">
-        <f t="shared" si="52">IF(ISBLANK('ONR 3'!M12),"",'ONR 3'!M12)</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="247" t="b">
-        <f t="shared" si="53">IF(ISBLANK('ONR 3'!N12),"",'ONR 3'!N12)</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="247" t="b">
-        <f t="shared" si="54">IF(ISBLANK('ONR 3'!O12),"",'ONR 3'!O12)</f>
-        <v>0</v>
-      </c>
-      <c r="P25" s="247" t="b">
-        <f t="shared" si="55">IF(ISBLANK('ONR 3'!P12),"",'ONR 3'!P12)</f>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="247" t="b">
-        <f t="shared" si="56">IF(ISBLANK('ONR 3'!Q12),"",'ONR 3'!Q12)</f>
-        <v>0</v>
-      </c>
-      <c r="R25" s="247" t="b">
-        <f t="shared" si="57">IF(ISBLANK('ONR 3'!R12),"",'ONR 3'!R12)</f>
-        <v>0</v>
-      </c>
-      <c r="S25" s="248" t="str">
-        <f t="shared" si="58">IF(ISBLANK('ONR 3'!S12),"",'ONR 3'!S12)</f>
-      </c>
-      <c r="T25" s="249" t="str">
-        <f t="shared" si="59">IF(ISBLANK('ONR 3'!T12),"",'ONR 3'!T12)</f>
-      </c>
-      <c r="U25" s="250" t="str">
-        <f t="shared" si="60">IF(ISBLANK('ONR 3'!U12),"",'ONR 3'!U12)</f>
-      </c>
-      <c r="V25" s="252" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G12),"",'ONR 3'!G12)</f>
-      </c>
-      <c r="W25" s="252" t="str">
-        <f>IF(ISBLANK('ONR 3'!V12),"",'ONR 3'!V12)</f>
+        <f>IF(ISBLANK('ONR 3'!J10),"",'ONR 3'!J10)</f>
+      </c>
+      <c r="K23" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K10),"",'ONR 3'!K10)</f>
+      </c>
+      <c r="L23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L10),"",'ONR 3'!L10)</f>
+      </c>
+      <c r="M23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M10),"",'ONR 3'!M10)</f>
+      </c>
+      <c r="N23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N10),"",'ONR 3'!N10)</f>
+      </c>
+      <c r="O23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O10),"",'ONR 3'!O10)</f>
+      </c>
+      <c r="P23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P10),"",'ONR 3'!P10)</f>
+      </c>
+      <c r="Q23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q10),"",'ONR 3'!Q10)</f>
+      </c>
+      <c r="R23" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R10),"",'ONR 3'!R10)</f>
+      </c>
+      <c r="S23" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S10),"",'ONR 3'!S10)</f>
+      </c>
+      <c r="T23" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T10),"",'ONR 3'!T10)</f>
+      </c>
+      <c r="U23" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U10),"",'ONR 3'!U10)</f>
+      </c>
+      <c r="V23" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!G10),"",'ONR 3'!G10)</f>
+      </c>
+      <c r="W23" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!V10),"",'ONR 3'!V10)</f>
       </c>
       <c r="X23" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W10),"",'ONR 3'!W10)</f>
       </c>
       <c r="Y23" s="253" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
+        <f>IF(ISBLANK('ONR 3'!I10),"",'ONR 3'!I10)</f>
       </c>
       <c r="Z23" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D10),"",'ONR 3'!D10)</f>
+        <f>IF(ISBLANK('ONR 3'!D10),"",'ONR 3'!D10)</f>
       </c>
       <c r="AE23" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T23),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T23),0,1)</f>
       </c>
       <c r="AF23" s="206" t="n">
-        <f t="shared" si="65">IF(L23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L23=TRUE,1,0)</f>
       </c>
       <c r="AG23" s="206" t="n">
-        <f t="shared" si="65">IF(M23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M23=TRUE,1,0)</f>
       </c>
       <c r="AH23" s="206" t="n">
-        <f t="shared" si="65">IF(N23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N23=TRUE,1,0)</f>
       </c>
       <c r="AI23" s="206" t="n">
-        <f t="shared" si="65">IF(O23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O23=TRUE,1,0)</f>
       </c>
       <c r="AJ23" s="206" t="n">
-        <f t="shared" si="65">IF(P23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P23=TRUE,1,0)</f>
       </c>
       <c r="AK23" s="206" t="n">
-        <f t="shared" si="65">IF(Q23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q23=TRUE,1,0)</f>
       </c>
       <c r="AL23" s="206" t="n">
-        <f t="shared" si="65">IF(R23=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R23=TRUE,1,0)</f>
       </c>
       <c r="AM23" t="n">
         <f>IF(LEN(TRIM(W23))&gt;0,1,0)</f>
@@ -33687,94 +33335,79 @@
         <f>IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
       </c>
       <c r="J24" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J11),"",'ONR 3'!J11)</f>
-      </c>
-      <c r="K26" s="247" t="str">
-        <f t="shared" si="50"/>
-      </c>
-      <c r="L26" s="247" t="b">
-        <f t="shared" si="51"/>
-        <v>0</v>
-      </c>
-      <c r="M26" s="247" t="b">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="N26" s="247" t="b">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="O26" s="247" t="b">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="P26" s="247" t="b">
-        <f t="shared" si="55"/>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="247" t="b">
-        <f t="shared" si="56"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="247" t="b">
-        <f t="shared" si="57"/>
-        <v>0</v>
-      </c>
-      <c r="S26" s="248" t="str">
-        <f t="shared" si="58"/>
-      </c>
-      <c r="T26" s="249" t="str">
-        <f t="shared" si="59"/>
-      </c>
-      <c r="U26" s="250" t="str">
-        <f t="shared" si="60"/>
-      </c>
-      <c r="V26" s="252" t="str">
-        <f t="shared" si="61"/>
-      </c>
-      <c r="W26" s="145" t="str">
-        <f>IF(ISBLANK('ONR 3'!V13),"",'ONR 3'!V13)</f>
+        <f>IF(ISBLANK('ONR 3'!J11),"",'ONR 3'!J11)</f>
+      </c>
+      <c r="K24" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K11),"",'ONR 3'!K11)</f>
+      </c>
+      <c r="L24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L11),"",'ONR 3'!L11)</f>
+      </c>
+      <c r="M24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M11),"",'ONR 3'!M11)</f>
+      </c>
+      <c r="N24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N11),"",'ONR 3'!N11)</f>
+      </c>
+      <c r="O24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O11),"",'ONR 3'!O11)</f>
+      </c>
+      <c r="P24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P11),"",'ONR 3'!P11)</f>
+      </c>
+      <c r="Q24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q11),"",'ONR 3'!Q11)</f>
+      </c>
+      <c r="R24" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R11),"",'ONR 3'!R11)</f>
+      </c>
+      <c r="S24" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S11),"",'ONR 3'!S11)</f>
+      </c>
+      <c r="T24" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T11),"",'ONR 3'!T11)</f>
+      </c>
+      <c r="U24" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U11),"",'ONR 3'!U11)</f>
+      </c>
+      <c r="V24" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!G11),"",'ONR 3'!G11)</f>
+      </c>
+      <c r="W24" s="235" t="str">
+        <f>IF(ISBLANK('ONR 3'!V11),"",'ONR 3'!V11)</f>
       </c>
       <c r="X24" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W11),"",'ONR 3'!W11)</f>
       </c>
       <c r="Y24" s="253" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
+        <f>IF(ISBLANK('ONR 3'!I11),"",'ONR 3'!I11)</f>
       </c>
       <c r="Z24" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D11),"",'ONR 3'!D11)</f>
+        <f>IF(ISBLANK('ONR 3'!D11),"",'ONR 3'!D11)</f>
       </c>
       <c r="AE24" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T24),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T24),0,1)</f>
       </c>
       <c r="AF24" s="206" t="n">
-        <f t="shared" si="65">IF(L24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L24=TRUE,1,0)</f>
       </c>
       <c r="AG24" s="206" t="n">
-        <f t="shared" si="65">IF(M24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M24=TRUE,1,0)</f>
       </c>
       <c r="AH24" s="206" t="n">
-        <f t="shared" si="65">IF(N24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N24=TRUE,1,0)</f>
       </c>
       <c r="AI24" s="206" t="n">
-        <f t="shared" si="65">IF(O24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O24=TRUE,1,0)</f>
       </c>
       <c r="AJ24" s="206" t="n">
-        <f t="shared" si="65">IF(P24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P24=TRUE,1,0)</f>
       </c>
       <c r="AK24" s="206" t="n">
-        <f t="shared" si="65">IF(Q24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q24=TRUE,1,0)</f>
       </c>
       <c r="AL24" s="206" t="n">
-        <f t="shared" si="65">IF(R24=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R24=TRUE,1,0)</f>
       </c>
       <c r="AM24" t="n">
         <f>IF(LEN(TRIM(W24))&gt;0,1,0)</f>
@@ -33810,87 +33443,79 @@
         <f>IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
       </c>
       <c r="J25" s="246" t="str">
-        <f t="shared" si="49">IF(ISBLANK('ONR 3'!J12),"",'ONR 3'!J12)</f>
-      </c>
-      <c r="K28" s="247">
-        <f t="shared" si="50"/>
-      </c>
-      <c r="L28" s="247">
-        <f t="shared" si="51"/>
-      </c>
-      <c r="M28" s="247">
-        <f t="shared" si="52"/>
-      </c>
-      <c r="N28" s="247">
-        <f t="shared" si="53"/>
-      </c>
-      <c r="O28" s="247">
-        <f t="shared" si="54"/>
-      </c>
-      <c r="P28" s="247">
-        <f t="shared" si="55"/>
-      </c>
-      <c r="Q28" s="247">
-        <f t="shared" si="56"/>
-      </c>
-      <c r="R28" s="247">
-        <f t="shared" si="57"/>
-      </c>
-      <c r="S28" s="248">
-        <f t="shared" si="58"/>
-      </c>
-      <c r="T28" s="249">
-        <f t="shared" si="59"/>
-      </c>
-      <c r="U28" s="250">
-        <f t="shared" si="60"/>
-      </c>
-      <c r="V28" s="241">
-        <f t="shared" si="61"/>
-      </c>
-      <c r="W28" s="148">
-        <f>'ONR 3'!V12</f>
+        <f>IF(ISBLANK('ONR 3'!J12),"",'ONR 3'!J12)</f>
+      </c>
+      <c r="K25" s="247" t="str">
+        <f>IF(ISBLANK('ONR 3'!K12),"",'ONR 3'!K12)</f>
+      </c>
+      <c r="L25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!L12),"",'ONR 3'!L12)</f>
+      </c>
+      <c r="M25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!M12),"",'ONR 3'!M12)</f>
+      </c>
+      <c r="N25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!N12),"",'ONR 3'!N12)</f>
+      </c>
+      <c r="O25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!O12),"",'ONR 3'!O12)</f>
+      </c>
+      <c r="P25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!P12),"",'ONR 3'!P12)</f>
+      </c>
+      <c r="Q25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!Q12),"",'ONR 3'!Q12)</f>
+      </c>
+      <c r="R25" s="247" t="b">
+        <f>IF(ISBLANK('ONR 3'!R12),"",'ONR 3'!R12)</f>
+      </c>
+      <c r="S25" s="248" t="str">
+        <f>IF(ISBLANK('ONR 3'!S12),"",'ONR 3'!S12)</f>
+      </c>
+      <c r="T25" s="249" t="str">
+        <f>IF(ISBLANK('ONR 3'!T12),"",'ONR 3'!T12)</f>
+      </c>
+      <c r="U25" s="250" t="str">
+        <f>IF(ISBLANK('ONR 3'!U12),"",'ONR 3'!U12)</f>
+      </c>
+      <c r="V25" s="252" t="str">
+        <f>IF(ISBLANK('ONR 3'!G12),"",'ONR 3'!G12)</f>
+      </c>
+      <c r="W25" s="252" t="str">
+        <f>IF(ISBLANK('ONR 3'!V12),"",'ONR 3'!V12)</f>
       </c>
       <c r="X25" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W12),"",'ONR 3'!W12)</f>
       </c>
       <c r="Y25" s="254" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
+        <f>IF(ISBLANK('ONR 3'!I12),"",'ONR 3'!I12)</f>
       </c>
       <c r="Z25" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D12),"",'ONR 3'!D12)</f>
+        <f>IF(ISBLANK('ONR 3'!D12),"",'ONR 3'!D12)</f>
       </c>
       <c r="AE25" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T25),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T25),0,1)</f>
       </c>
       <c r="AF25" s="206" t="n">
-        <f t="shared" si="65">IF(L25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L25=TRUE,1,0)</f>
       </c>
       <c r="AG25" s="206" t="n">
-        <f t="shared" si="65">IF(M25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M25=TRUE,1,0)</f>
       </c>
       <c r="AH25" s="206" t="n">
-        <f t="shared" si="65">IF(N25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N25=TRUE,1,0)</f>
       </c>
       <c r="AI25" s="206" t="n">
-        <f t="shared" si="65">IF(O25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O25=TRUE,1,0)</f>
       </c>
       <c r="AJ25" s="206" t="n">
-        <f t="shared" si="65">IF(P25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P25=TRUE,1,0)</f>
       </c>
       <c r="AK25" s="206" t="n">
-        <f t="shared" si="65">IF(Q25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q25=TRUE,1,0)</f>
       </c>
       <c r="AL25" s="206" t="n">
-        <f t="shared" si="65">IF(R25=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R25=TRUE,1,0)</f>
       </c>
       <c r="AM25" t="n">
         <f>IF(LEN(TRIM(W25))&gt;0,1,0)</f>
@@ -33926,94 +33551,79 @@
         <f>IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
       </c>
       <c r="J26" s="246" t="str">
-        <f t="shared" ref="J26" si="66">IF(ISBLANK('ONR 3'!J13),"",'ONR 3'!J13)</f>
+        <f>IF(ISBLANK('ONR 3'!J13),"",'ONR 3'!J13)</f>
       </c>
       <c r="K26" s="247" t="str">
-        <f t="shared" ref="K26" si="67">IF(ISBLANK('ONR 3'!K13),"",'ONR 3'!K13)</f>
+        <f>IF(ISBLANK('ONR 3'!K13),"",'ONR 3'!K13)</f>
       </c>
       <c r="L26" s="247" t="b">
-        <f t="shared" ref="L26" si="68">IF(ISBLANK('ONR 3'!L13),"",'ONR 3'!L13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!L13),"",'ONR 3'!L13)</f>
       </c>
       <c r="M26" s="247" t="b">
-        <f t="shared" ref="M26" si="69">IF(ISBLANK('ONR 3'!M13),"",'ONR 3'!M13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!M13),"",'ONR 3'!M13)</f>
       </c>
       <c r="N26" s="247" t="b">
-        <f t="shared" ref="N26" si="70">IF(ISBLANK('ONR 3'!N13),"",'ONR 3'!N13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!N13),"",'ONR 3'!N13)</f>
       </c>
       <c r="O26" s="247" t="b">
-        <f t="shared" ref="O26" si="71">IF(ISBLANK('ONR 3'!O13),"",'ONR 3'!O13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!O13),"",'ONR 3'!O13)</f>
       </c>
       <c r="P26" s="247" t="b">
-        <f t="shared" ref="P26" si="72">IF(ISBLANK('ONR 3'!P13),"",'ONR 3'!P13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!P13),"",'ONR 3'!P13)</f>
       </c>
       <c r="Q26" s="247" t="b">
-        <f t="shared" ref="Q26" si="73">IF(ISBLANK('ONR 3'!Q13),"",'ONR 3'!Q13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!Q13),"",'ONR 3'!Q13)</f>
       </c>
       <c r="R26" s="247" t="b">
-        <f t="shared" ref="R26" si="74">IF(ISBLANK('ONR 3'!R13),"",'ONR 3'!R13)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 3'!R13),"",'ONR 3'!R13)</f>
       </c>
       <c r="S26" s="248" t="str">
-        <f t="shared" ref="S26" si="75">IF(ISBLANK('ONR 3'!S13),"",'ONR 3'!S13)</f>
+        <f>IF(ISBLANK('ONR 3'!S13),"",'ONR 3'!S13)</f>
       </c>
       <c r="T26" s="249" t="str">
-        <f t="shared" ref="T26" si="76">IF(ISBLANK('ONR 3'!T13),"",'ONR 3'!T13)</f>
+        <f>IF(ISBLANK('ONR 3'!T13),"",'ONR 3'!T13)</f>
       </c>
       <c r="U26" s="250" t="str">
-        <f t="shared" ref="U26" si="77">IF(ISBLANK('ONR 3'!U13),"",'ONR 3'!U13)</f>
+        <f>IF(ISBLANK('ONR 3'!U13),"",'ONR 3'!U13)</f>
       </c>
       <c r="V26" s="255" t="str">
-        <f t="shared" si="61">IF(ISBLANK('ONR 3'!G13),"",'ONR 3'!G13)</f>
-      </c>
-      <c r="W29" s="215" t="str">
-        <f>'ONR 3'!V13</f>
+        <f>IF(ISBLANK('ONR 3'!G13),"",'ONR 3'!G13)</f>
+      </c>
+      <c r="W26" s="145" t="str">
+        <f>IF(ISBLANK('ONR 3'!V13),"",'ONR 3'!V13)</f>
       </c>
       <c r="X26" s="183" t="str">
         <f>IF(ISBLANK('ONR 3'!W13),"",'ONR 3'!W13)</f>
       </c>
       <c r="Y26" s="251" t="str">
-        <f t="shared" si="62">IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
+        <f>IF(ISBLANK('ONR 3'!I13),"",'ONR 3'!I13)</f>
       </c>
       <c r="Z26" s="251" t="str">
-        <f t="shared" si="63">IF(ISBLANK('ONR 3'!D13),"",'ONR 3'!D13)</f>
+        <f>IF(ISBLANK('ONR 3'!D13),"",'ONR 3'!D13)</f>
       </c>
       <c r="AE26" s="206" t="n">
-        <f t="shared" si="64">IF(ISNUMBER(T26),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T26),0,1)</f>
       </c>
       <c r="AF26" s="206" t="n">
-        <f t="shared" si="65">IF(L26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L26=TRUE,1,0)</f>
       </c>
       <c r="AG26" s="206" t="n">
-        <f t="shared" si="65">IF(M26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M26=TRUE,1,0)</f>
       </c>
       <c r="AH26" s="206" t="n">
-        <f t="shared" si="65">IF(N26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N26=TRUE,1,0)</f>
       </c>
       <c r="AI26" s="206" t="n">
-        <f t="shared" si="65">IF(O26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O26=TRUE,1,0)</f>
       </c>
       <c r="AJ26" s="206" t="n">
-        <f t="shared" si="65">IF(P26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P26=TRUE,1,0)</f>
       </c>
       <c r="AK26" s="206" t="n">
-        <f t="shared" si="65">IF(Q26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q26=TRUE,1,0)</f>
       </c>
       <c r="AL26" s="206" t="n">
-        <f t="shared" si="65">IF(R26=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R26=TRUE,1,0)</f>
       </c>
       <c r="AM26" t="n">
         <f>IF(LEN(TRIM(W26))&gt;0,1,0)</f>
@@ -34251,7 +33861,7 @@
         <f>IF(ISBLANK('ONR 4'!J7),"",'ONR 4'!J7)</f>
       </c>
       <c r="K29" s="227" t="str">
-        <f t="shared" ref="K29:K30" si="79">IF(ISBLANK('ONR 4'!K7),"",'ONR 4'!K7)</f>
+        <f>IF(ISBLANK('ONR 4'!K7),"",'ONR 4'!K7)</f>
       </c>
       <c r="L29" s="227" t="b">
         <f>IF(ISBLANK('ONR 4'!L7),"",'ONR 4'!L7)</f>
@@ -34282,13 +33892,13 @@
         <v>0</v>
       </c>
       <c r="S29" s="228" t="str">
-        <f t="shared" ref="S29:S30" si="80">IF(ISBLANK('ONR 4'!S7),"",'ONR 4'!S7)</f>
+        <f>IF(ISBLANK('ONR 4'!S7),"",'ONR 4'!S7)</f>
       </c>
       <c r="T29" s="226" t="str">
-        <f t="shared" ref="T29" si="81">IF(ISBLANK('ONR 4'!T7),"",'ONR 4'!T7)</f>
+        <f>IF(ISBLANK('ONR 4'!T7),"",'ONR 4'!T7)</f>
       </c>
       <c r="U29" s="242" t="str">
-        <f t="shared" ref="U29" si="82">IF(ISBLANK('ONR 4'!U7),"",'ONR 4'!U7)</f>
+        <f>IF(ISBLANK('ONR 4'!U7),"",'ONR 4'!U7)</f>
       </c>
       <c r="V29" s="229" t="str">
         <f>IF(ISBLANK('ONR 4'!G7),"",'ONR 4'!G7)</f>
@@ -34310,32 +33920,25 @@
         <v>1</v>
       </c>
       <c r="AF29" s="206" t="n">
-        <f t="shared" ref="AF29:AL32" si="83">IF(L29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L29=TRUE,1,0)</f>
       </c>
       <c r="AG29" s="206" t="n">
-        <f t="shared" si="83">IF(M29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M29=TRUE,1,0)</f>
       </c>
       <c r="AH29" s="206" t="n">
-        <f t="shared" si="83">IF(N29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N29=TRUE,1,0)</f>
       </c>
       <c r="AI29" s="206" t="n">
-        <f t="shared" si="83">IF(O29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O29=TRUE,1,0)</f>
       </c>
       <c r="AJ29" s="206" t="n">
-        <f t="shared" si="83">IF(P29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P29=TRUE,1,0)</f>
       </c>
       <c r="AK29" s="206" t="n">
-        <f t="shared" si="83">IF(Q29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q29=TRUE,1,0)</f>
       </c>
       <c r="AL29" s="206" t="n">
-        <f t="shared" si="83">IF(R29=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R29=TRUE,1,0)</f>
       </c>
       <c r="AM29" t="n">
         <f>IF(LEN(TRIM(W29))&gt;0,1,0)</f>
@@ -34371,59 +33974,41 @@
         <f>IF(ISBLANK('ONR 4'!I8),"",'ONR 4'!I8)</f>
       </c>
       <c r="J30" s="219" t="str">
-        <f t="shared" ref="J30:J38" si="84">IF(ISBLANK('ONR 4'!J8),"",'ONR 4'!J8)</f>
+        <f>IF(ISBLANK('ONR 4'!J8),"",'ONR 4'!J8)</f>
       </c>
       <c r="K30" s="233" t="str">
-        <f t="shared" si="79">IF(ISBLANK('ONR 4'!K8),"",'ONR 4'!K8)</f>
-      </c>
-      <c r="L33" s="233">
-        <f t="shared" ref="L33" si="85">OR(K30=31)</f>
+        <f>IF(ISBLANK('ONR 4'!K8),"",'ONR 4'!K8)</f>
       </c>
       <c r="L30" t="b" s="227">
         <f>IF(ISBLANK('ONR 4'!L8),"",'ONR 4'!L8)</f>
         <v>0</v>
       </c>
       <c r="M30" s="233" t="b">
-        <f t="shared" ref="M30" si="86">IF(ISBLANK('ONR 4'!M8),"",'ONR 4'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!M8),"",'ONR 4'!M8)</f>
       </c>
       <c r="N30" s="233" t="b">
-        <f t="shared" ref="N30" si="87">IF(ISBLANK('ONR 4'!N8),"",'ONR 4'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!N8),"",'ONR 4'!N8)</f>
       </c>
       <c r="O30" s="233" t="b">
-        <f t="shared" ref="O30" si="88">IF(ISBLANK('ONR 4'!O8),"",'ONR 4'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!O8),"",'ONR 4'!O8)</f>
       </c>
       <c r="P30" s="233" t="b">
-        <f t="shared" ref="P30" si="89">IF(ISBLANK('ONR 4'!P8),"",'ONR 4'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!P8),"",'ONR 4'!P8)</f>
       </c>
       <c r="Q30" s="233" t="b">
-        <f t="shared" ref="Q30" si="90">IF(ISBLANK('ONR 4'!Q8),"",'ONR 4'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!Q8),"",'ONR 4'!Q8)</f>
       </c>
       <c r="R30" s="233" t="b">
-        <f t="shared" ref="R30" si="91">IF(ISBLANK('ONR 4'!R8),"",'ONR 4'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!R8),"",'ONR 4'!R8)</f>
       </c>
       <c r="S30" s="234" t="str">
-        <f t="shared" si="80">IF(ISBLANK('ONR 4'!S8),"",'ONR 4'!S8)</f>
-      </c>
-      <c r="T33" s="232">
-        <f t="shared" si="81"/>
+        <f>IF(ISBLANK('ONR 4'!S8),"",'ONR 4'!S8)</f>
       </c>
       <c r="T30" t="str" s="226">
         <f>IF(ISBLANK('ONR 4'!T8),"",'ONR 4'!T8)</f>
       </c>
-      <c r="U33" s="243">
-        <f t="shared" si="82"/>
-      </c>
       <c r="U30" t="str" s="242">
         <f>IF(ISBLANK('ONR 4'!U8),"",'ONR 4'!U8)</f>
-      </c>
-      <c r="V33" s="235">
-        <f>G30</f>
       </c>
       <c r="V30" t="str" s="229">
         <f>IF(ISBLANK('ONR 4'!G8),"",'ONR 4'!G8)</f>
@@ -34445,32 +34030,25 @@
         <v>1</v>
       </c>
       <c r="AF30" s="206" t="n">
-        <f t="shared" si="83">IF(L30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L30=TRUE,1,0)</f>
       </c>
       <c r="AG30" s="206" t="n">
-        <f t="shared" si="83">IF(M30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M30=TRUE,1,0)</f>
       </c>
       <c r="AH30" s="206" t="n">
-        <f t="shared" si="83">IF(N30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N30=TRUE,1,0)</f>
       </c>
       <c r="AI30" s="206" t="n">
-        <f t="shared" si="83">IF(O30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O30=TRUE,1,0)</f>
       </c>
       <c r="AJ30" s="206" t="n">
-        <f t="shared" si="83">IF(P30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P30=TRUE,1,0)</f>
       </c>
       <c r="AK30" s="206" t="n">
-        <f t="shared" si="83">IF(Q30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q30=TRUE,1,0)</f>
       </c>
       <c r="AL30" s="206" t="n">
-        <f t="shared" si="83">IF(R30=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R30=TRUE,1,0)</f>
       </c>
       <c r="AM30" t="n">
         <f>IF(LEN(TRIM(W30))&gt;0,1,0)</f>
@@ -34506,47 +34084,40 @@
         <f>IF(ISBLANK('ONR 4'!I9),"",'ONR 4'!I9)</f>
       </c>
       <c r="J31" s="219" t="str">
-        <f t="shared" ref="J31:J32" si="92">IF(ISBLANK('ONR 4'!J9),"",'ONR 4'!J9)</f>
+        <f>IF(ISBLANK('ONR 4'!J9),"",'ONR 4'!J9)</f>
       </c>
       <c r="K31" s="233" t="str">
-        <f t="shared" ref="K31:K35" si="93">IF(ISBLANK('ONR 4'!K9),"",'ONR 4'!K9)</f>
+        <f>IF(ISBLANK('ONR 4'!K9),"",'ONR 4'!K9)</f>
       </c>
       <c r="L31" s="233" t="b">
-        <f t="shared" ref="L31:L35" si="94">IF(ISBLANK('ONR 4'!L9),"",'ONR 4'!L9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!L9),"",'ONR 4'!L9)</f>
       </c>
       <c r="M31" s="233" t="b">
-        <f t="shared" ref="M31" si="95">IF(ISBLANK('ONR 4'!M9),"",'ONR 4'!M9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!M9),"",'ONR 4'!M9)</f>
       </c>
       <c r="N31" s="233" t="b">
-        <f t="shared" ref="N31" si="96">IF(ISBLANK('ONR 4'!N9),"",'ONR 4'!N9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!N9),"",'ONR 4'!N9)</f>
       </c>
       <c r="O31" s="233" t="b">
-        <f t="shared" ref="O31" si="97">IF(ISBLANK('ONR 4'!O9),"",'ONR 4'!O9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!O9),"",'ONR 4'!O9)</f>
       </c>
       <c r="P31" s="233" t="b">
-        <f t="shared" ref="P31" si="98">IF(ISBLANK('ONR 4'!P9),"",'ONR 4'!P9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!P9),"",'ONR 4'!P9)</f>
       </c>
       <c r="Q31" s="233" t="b">
-        <f t="shared" ref="Q31" si="99">IF(ISBLANK('ONR 4'!Q9),"",'ONR 4'!Q9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!Q9),"",'ONR 4'!Q9)</f>
       </c>
       <c r="R31" s="233" t="b">
-        <f t="shared" ref="R31" si="100">IF(ISBLANK('ONR 4'!R9),"",'ONR 4'!R9)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 4'!R9),"",'ONR 4'!R9)</f>
       </c>
       <c r="S31" s="234" t="str">
-        <f t="shared" ref="S31" si="101">IF(ISBLANK('ONR 4'!S9),"",'ONR 4'!S9)</f>
+        <f>IF(ISBLANK('ONR 4'!S9),"",'ONR 4'!S9)</f>
       </c>
       <c r="T31" s="232" t="str">
-        <f t="shared" ref="T31:T35" si="102">IF(ISBLANK('ONR 4'!T9),"",'ONR 4'!T9)</f>
+        <f>IF(ISBLANK('ONR 4'!T9),"",'ONR 4'!T9)</f>
       </c>
       <c r="U31" s="243" t="str">
-        <f t="shared" ref="U31:U35" si="103">IF(ISBLANK('ONR 4'!U9),"",'ONR 4'!U9)</f>
+        <f>IF(ISBLANK('ONR 4'!U9),"",'ONR 4'!U9)</f>
       </c>
       <c r="V31" s="235" t="str">
         <f>IF(ISBLANK('ONR 4'!G9),"",'ONR 4'!G9)</f>
@@ -34568,32 +34139,25 @@
         <v>1</v>
       </c>
       <c r="AF31" s="206" t="n">
-        <f t="shared" si="83">IF(L31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L31=TRUE,1,0)</f>
       </c>
       <c r="AG31" s="206" t="n">
-        <f t="shared" si="83">IF(M31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M31=TRUE,1,0)</f>
       </c>
       <c r="AH31" s="206" t="n">
-        <f t="shared" si="83">IF(N31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N31=TRUE,1,0)</f>
       </c>
       <c r="AI31" s="206" t="n">
-        <f t="shared" si="83">IF(O31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O31=TRUE,1,0)</f>
       </c>
       <c r="AJ31" s="206" t="n">
-        <f t="shared" si="83">IF(P31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P31=TRUE,1,0)</f>
       </c>
       <c r="AK31" s="206" t="n">
-        <f t="shared" si="83">IF(Q31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q31=TRUE,1,0)</f>
       </c>
       <c r="AL31" s="206" t="n">
-        <f t="shared" si="83">IF(R31=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R31=TRUE,1,0)</f>
       </c>
       <c r="AM31" t="n">
         <f>IF(LEN(TRIM(W31))&gt;0,1,0)</f>
@@ -34629,91 +34193,47 @@
         <f>IF(ISBLANK('ONR 4'!I10),"",'ONR 4'!I10)</f>
       </c>
       <c r="J32" s="219" t="n">
-        <f t="shared" si="92">IF(ISBLANK('ONR 4'!J10),"",'ONR 4'!J10)</f>
-        <v>0</v>
-      </c>
-      <c r="K35" s="233" t="str">
-        <f t="shared" si="93">IF(ISBLANK('ONR 5'!K8),"",'ONR 5'!K8)</f>
+        <f>IF(ISBLANK('ONR 4'!J10),"",'ONR 4'!J10)</f>
       </c>
       <c r="K32" t="str" s="233">
         <f>IF(ISBLANK('ONR 4'!K10),"",'ONR 4'!K10)</f>
-      </c>
-      <c r="L35" s="233" t="b">
-        <f t="shared" si="94">IF(ISBLANK('ONR 5'!L8),"",'ONR 5'!L8)</f>
-        <v>0</v>
       </c>
       <c r="L32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!L10),"",'ONR 4'!L10)</f>
         <v>0</v>
       </c>
-      <c r="M35" s="233" t="b">
-        <f t="shared" si="95"/>
-        <v>0</v>
-      </c>
       <c r="M32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!M10),"",'ONR 4'!M10)</f>
         <v>0</v>
       </c>
-      <c r="N35" s="233" t="b">
-        <f t="shared" si="96"/>
-        <v>0</v>
-      </c>
       <c r="N32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!N10),"",'ONR 4'!N10)</f>
         <v>0</v>
       </c>
-      <c r="O35" s="233" t="b">
-        <f t="shared" si="97"/>
-        <v>0</v>
-      </c>
       <c r="O32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!O10),"",'ONR 4'!O10)</f>
         <v>0</v>
       </c>
-      <c r="P35" s="233" t="b">
-        <f t="shared" si="98"/>
-        <v>0</v>
-      </c>
       <c r="P32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!P10),"",'ONR 4'!P10)</f>
         <v>0</v>
       </c>
-      <c r="Q35" s="233" t="b">
-        <f t="shared" si="99"/>
-        <v>0</v>
-      </c>
       <c r="Q32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!Q10),"",'ONR 4'!Q10)</f>
         <v>0</v>
       </c>
-      <c r="R35" s="233" t="b">
-        <f t="shared" si="100"/>
-        <v>0</v>
-      </c>
       <c r="R32" t="b" s="233">
         <f>IF(ISBLANK('ONR 4'!R10),"",'ONR 4'!R10)</f>
         <v>0</v>
       </c>
-      <c r="S35" s="234" t="str">
-        <f t="shared" si="101"/>
-      </c>
       <c r="S32" t="str" s="234">
         <f>IF(ISBLANK('ONR 4'!S10),"",'ONR 4'!S10)</f>
       </c>
-      <c r="T35" s="232" t="str">
-        <f t="shared" si="102">IF(ISBLANK('ONR 5'!T8),"",'ONR 5'!T8)</f>
-      </c>
       <c r="T32" t="str" s="232">
         <f>IF(ISBLANK('ONR 4'!T10),"",'ONR 4'!T10)</f>
       </c>
-      <c r="U35" s="243" t="str">
-        <f t="shared" si="103">IF(ISBLANK('ONR 5'!U8),"",'ONR 5'!U8)</f>
-      </c>
       <c r="U32" t="str" s="243">
         <f>IF(ISBLANK('ONR 4'!U10),"",'ONR 4'!U10)</f>
-      </c>
-      <c r="V35" s="235" t="str">
-        <f>IF(ISBLANK('ONR 5'!G8),"",'ONR 5'!G8)</f>
       </c>
       <c r="V32" t="str" s="235">
         <f>IF(ISBLANK('ONR 4'!G10),"",'ONR 4'!G10)</f>
@@ -34735,32 +34255,25 @@
         <v>1</v>
       </c>
       <c r="AF32" s="206" t="n">
-        <f t="shared" si="83">IF(L32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L32=TRUE,1,0)</f>
       </c>
       <c r="AG32" s="206" t="n">
-        <f t="shared" si="83">IF(M32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M32=TRUE,1,0)</f>
       </c>
       <c r="AH32" s="206" t="n">
-        <f t="shared" si="83">IF(N32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N32=TRUE,1,0)</f>
       </c>
       <c r="AI32" s="206" t="n">
-        <f t="shared" si="83">IF(O32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O32=TRUE,1,0)</f>
       </c>
       <c r="AJ32" s="206" t="n">
-        <f t="shared" si="83">IF(P32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P32=TRUE,1,0)</f>
       </c>
       <c r="AK32" s="206" t="n">
-        <f t="shared" si="83">IF(Q32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q32=TRUE,1,0)</f>
       </c>
       <c r="AL32" s="206" t="n">
-        <f t="shared" si="83">IF(R32=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R32=TRUE,1,0)</f>
       </c>
       <c r="AM32" t="n">
         <f>IF(LEN(TRIM(W32))&gt;0,1,0)</f>
@@ -34871,10 +34384,7 @@
         <f>IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
       </c>
       <c r="J34" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J7),"",'ONR 5'!J7)</f>
-      </c>
-      <c r="K37" s="227" t="str">
-        <f t="shared" ref="K37:K38" si="105">E34*10+F34</f>
+        <f>IF(ISBLANK('ONR 5'!J7),"",'ONR 5'!J7)</f>
       </c>
       <c r="K34" t="str" s="362">
         <f>IF(ISBLANK('ONR 5'!K7),"",'ONR 5'!K7)</f>
@@ -34908,16 +34418,16 @@
         <v>0</v>
       </c>
       <c r="S34" s="228" t="str">
-        <f t="shared" ref="S34:S38" si="106">IF(ISBLANK('ONR 5'!S7),"",'ONR 5'!S7)</f>
+        <f>IF(ISBLANK('ONR 5'!S7),"",'ONR 5'!S7)</f>
       </c>
       <c r="T34" s="226" t="str">
-        <f t="shared" ref="T34:T38" si="107">IF(ISBLANK('ONR 5'!T7),"",'ONR 5'!T7)</f>
+        <f>IF(ISBLANK('ONR 5'!T7),"",'ONR 5'!T7)</f>
       </c>
       <c r="U34" s="242" t="str">
-        <f t="shared" ref="U34:U38" si="108">IF(ISBLANK('ONR 5'!U7),"",'ONR 5'!U7)</f>
+        <f>IF(ISBLANK('ONR 5'!U7),"",'ONR 5'!U7)</f>
       </c>
       <c r="V34" s="229" t="str">
-        <f t="shared" ref="V34:V38" si="109">IF(ISBLANK('ONR 5'!G7),"",'ONR 5'!G7)</f>
+        <f>IF(ISBLANK('ONR 5'!G7),"",'ONR 5'!G7)</f>
       </c>
       <c r="W34" s="203" t="str">
         <f>IF(ISBLANK('ONR 5'!V7),"",'ONR 5'!V7)</f>
@@ -34926,42 +34436,34 @@
         <f>IF(ISBLANK('ONR 5'!W7),"",'ONR 5'!W7)</f>
       </c>
       <c r="Y34" s="257" t="str">
-        <f t="shared" ref="Y34:Y38" si="110">IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
+        <f>IF(ISBLANK('ONR 5'!I7),"",'ONR 5'!I7)</f>
       </c>
       <c r="Z34" s="256" t="str">
         <f>IF(ISBLANK('ONR 5'!D7),"",'ONR 5'!D7)</f>
       </c>
       <c r="AE34" s="206" t="n">
-        <f t="shared" ref="AE34:AE38" si="111">IF(ISNUMBER(T34),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T34),0,1)</f>
       </c>
       <c r="AF34" s="206" t="n">
-        <f t="shared" ref="AF34:AF38" si="112">IF(L34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L34=TRUE,1,0)</f>
       </c>
       <c r="AG34" s="206" t="n">
-        <f t="shared" ref="AG34:AG38" si="113">IF(M34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M34=TRUE,1,0)</f>
       </c>
       <c r="AH34" s="206" t="n">
-        <f t="shared" ref="AH34:AH38" si="114">IF(N34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N34=TRUE,1,0)</f>
       </c>
       <c r="AI34" s="206" t="n">
-        <f t="shared" ref="AI34:AI38" si="115">IF(O34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O34=TRUE,1,0)</f>
       </c>
       <c r="AJ34" s="206" t="n">
-        <f t="shared" ref="AJ34:AJ38" si="116">IF(P34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P34=TRUE,1,0)</f>
       </c>
       <c r="AK34" s="206" t="n">
-        <f t="shared" ref="AK34:AK38" si="117">IF(Q34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q34=TRUE,1,0)</f>
       </c>
       <c r="AL34" s="206" t="n">
-        <f t="shared" ref="AL34:AL38" si="118">IF(R34=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R34=TRUE,1,0)</f>
       </c>
       <c r="AM34" t="n">
         <f>IF(LEN(TRIM(W34))&gt;0,1,0)</f>
@@ -34997,53 +34499,43 @@
         <f>IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
       </c>
       <c r="J35" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J8),"",'ONR 5'!J8)</f>
-      </c>
-      <c r="K38" s="233" t="str">
-        <f t="shared" si="105"/>
-      </c>
-      <c r="L38" s="233" t="b">
-        <f t="shared" ref="L38:L38" si="119">OR(K35=31)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!J8),"",'ONR 5'!J8)</f>
+      </c>
+      <c r="K35" s="233" t="str">
+        <f>IF(ISBLANK('ONR 5'!K8),"",'ONR 5'!K8)</f>
+      </c>
+      <c r="L35" s="233" t="b">
+        <f>IF(ISBLANK('ONR 5'!L8),"",'ONR 5'!L8)</f>
       </c>
       <c r="M35" s="233" t="b">
-        <f t="shared" ref="M35:M38" si="120">IF(ISBLANK('ONR 5'!M8),"",'ONR 5'!M8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M8),"",'ONR 5'!M8)</f>
       </c>
       <c r="N35" s="233" t="b">
-        <f t="shared" ref="N35:N38" si="121">IF(ISBLANK('ONR 5'!N8),"",'ONR 5'!N8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N8),"",'ONR 5'!N8)</f>
       </c>
       <c r="O35" s="233" t="b">
-        <f t="shared" ref="O35:O38" si="122">IF(ISBLANK('ONR 5'!O8),"",'ONR 5'!O8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O8),"",'ONR 5'!O8)</f>
       </c>
       <c r="P35" s="233" t="b">
-        <f t="shared" ref="P35:P38" si="123">IF(ISBLANK('ONR 5'!P8),"",'ONR 5'!P8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P8),"",'ONR 5'!P8)</f>
       </c>
       <c r="Q35" s="233" t="b">
-        <f t="shared" ref="Q35:Q38" si="124">IF(ISBLANK('ONR 5'!Q8),"",'ONR 5'!Q8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q8),"",'ONR 5'!Q8)</f>
       </c>
       <c r="R35" s="233" t="b">
-        <f t="shared" ref="R35:R38" si="125">IF(ISBLANK('ONR 5'!R8),"",'ONR 5'!R8)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R8),"",'ONR 5'!R8)</f>
       </c>
       <c r="S35" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S8),"",'ONR 5'!S8)</f>
-      </c>
-      <c r="T38" s="232" t="str">
-        <f t="shared" si="107"/>
-      </c>
-      <c r="U38" s="243" t="str">
-        <f t="shared" si="108"/>
-      </c>
-      <c r="V38" s="235" t="str">
-        <f t="shared" si="109"/>
-      </c>
-      <c r="W38" s="142" t="str">
-        <f>'ONR 5'!V8</f>
+        <f>IF(ISBLANK('ONR 5'!S8),"",'ONR 5'!S8)</f>
+      </c>
+      <c r="T35" s="232" t="str">
+        <f>IF(ISBLANK('ONR 5'!T8),"",'ONR 5'!T8)</f>
+      </c>
+      <c r="U35" s="243" t="str">
+        <f>IF(ISBLANK('ONR 5'!U8),"",'ONR 5'!U8)</f>
+      </c>
+      <c r="V35" s="235" t="str">
+        <f>IF(ISBLANK('ONR 5'!G8),"",'ONR 5'!G8)</f>
       </c>
       <c r="W35" t="str" s="203">
         <f>IF(ISBLANK('ONR 5'!V8),"",'ONR 5'!V8)</f>
@@ -35052,45 +34544,34 @@
         <f>IF(ISBLANK('ONR 5'!W8),"",'ONR 5'!W8)</f>
       </c>
       <c r="Y35" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
-      </c>
-      <c r="Z38" s="256" t="str">
-        <f t="shared" ref="Z38:Z38" si="126">D35</f>
+        <f>IF(ISBLANK('ONR 5'!I8),"",'ONR 5'!I8)</f>
       </c>
       <c r="Z35" t="str" s="256">
         <f>IF(ISBLANK('ONR 5'!D8),"",'ONR 5'!D8)</f>
       </c>
       <c r="AE35" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T35),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T35),0,1)</f>
       </c>
       <c r="AF35" s="206" t="n">
-        <f t="shared" si="112">IF(L35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L35=TRUE,1,0)</f>
       </c>
       <c r="AG35" s="206" t="n">
-        <f t="shared" si="113">IF(M35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M35=TRUE,1,0)</f>
       </c>
       <c r="AH35" s="206" t="n">
-        <f t="shared" si="114">IF(N35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N35=TRUE,1,0)</f>
       </c>
       <c r="AI35" s="206" t="n">
-        <f t="shared" si="115">IF(O35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O35=TRUE,1,0)</f>
       </c>
       <c r="AJ35" s="206" t="n">
-        <f t="shared" si="116">IF(P35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P35=TRUE,1,0)</f>
       </c>
       <c r="AK35" s="206" t="n">
-        <f t="shared" si="117">IF(Q35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q35=TRUE,1,0)</f>
       </c>
       <c r="AL35" s="206" t="n">
-        <f t="shared" si="118">IF(R35=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R35=TRUE,1,0)</f>
       </c>
       <c r="AM35" t="n">
         <f>IF(LEN(TRIM(W35))&gt;0,1,0)</f>
@@ -35126,97 +34607,51 @@
         <f>IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
       </c>
       <c r="J36" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J9),"",'ONR 5'!J9)</f>
-      </c>
-      <c r="K39" s="233" t="str">
-        <f t="shared" si="105"/>
+        <f>IF(ISBLANK('ONR 5'!J9),"",'ONR 5'!J9)</f>
       </c>
       <c r="K36" t="str" s="233">
         <f>IF(ISBLANK('ONR 5'!K9),"",'ONR 5'!K9)</f>
-      </c>
-      <c r="L39" s="233" t="b">
-        <f t="shared" si="119"/>
-        <v>0</v>
       </c>
       <c r="L36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!L9),"",'ONR 5'!L9)</f>
         <v>0</v>
       </c>
-      <c r="M39" s="233" t="b">
-        <f t="shared" si="120"/>
-        <v>0</v>
-      </c>
       <c r="M36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!M9),"",'ONR 5'!M9)</f>
         <v>0</v>
       </c>
-      <c r="N39" s="233" t="b">
-        <f t="shared" si="121"/>
-        <v>0</v>
-      </c>
       <c r="N36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!N9),"",'ONR 5'!N9)</f>
         <v>0</v>
       </c>
-      <c r="O39" s="233" t="b">
-        <f t="shared" si="122"/>
-        <v>0</v>
-      </c>
       <c r="O36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!O9),"",'ONR 5'!O9)</f>
         <v>0</v>
       </c>
-      <c r="P39" s="233" t="b">
-        <f t="shared" si="123"/>
-        <v>0</v>
-      </c>
       <c r="P36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!P9),"",'ONR 5'!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q39" s="233" t="b">
-        <f t="shared" si="124"/>
-        <v>0</v>
-      </c>
       <c r="Q36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!Q9),"",'ONR 5'!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R39" s="233" t="b">
-        <f t="shared" si="125"/>
-        <v>0</v>
-      </c>
       <c r="R36" t="b" s="233">
         <f>IF(ISBLANK('ONR 5'!R9),"",'ONR 5'!R9)</f>
         <v>0</v>
       </c>
-      <c r="S39" s="234" t="str">
-        <f t="shared" si="106"/>
-      </c>
       <c r="S36" t="str" s="234">
         <f>IF(ISBLANK('ONR 5'!S9),"",'ONR 5'!S9)</f>
       </c>
-      <c r="T39" s="232" t="str">
-        <f t="shared" si="107"/>
-      </c>
       <c r="T36" t="str" s="232">
         <f>IF(ISBLANK('ONR 5'!T9),"",'ONR 5'!T9)</f>
       </c>
-      <c r="U39" s="243" t="str">
-        <f t="shared" si="108"/>
-      </c>
       <c r="U36" t="str" s="243">
         <f>IF(ISBLANK('ONR 5'!U9),"",'ONR 5'!U9)</f>
       </c>
-      <c r="V39" s="235" t="str">
-        <f t="shared" si="109"/>
-      </c>
       <c r="V36" t="str" s="235">
         <f>IF(ISBLANK('ONR 5'!G9),"",'ONR 5'!G9)</f>
       </c>
-      <c r="W39" s="142" t="str">
-        <f>'ONR 5'!V9</f>
-      </c>
       <c r="W36" t="str" s="142">
         <f>IF(ISBLANK('ONR 5'!V9),"",'ONR 5'!V9)</f>
       </c>
@@ -35224,42 +34659,34 @@
         <f>IF(ISBLANK('ONR 5'!W9),"",'ONR 5'!W9)</f>
       </c>
       <c r="Y36" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
+        <f>IF(ISBLANK('ONR 5'!I9),"",'ONR 5'!I9)</f>
       </c>
       <c r="Z36" s="256" t="str">
-        <f t="shared" si="126">IF(ISBLANK('ONR 5'!D9),"",'ONR 5'!D9)</f>
+        <f>IF(ISBLANK('ONR 5'!D9),"",'ONR 5'!D9)</f>
       </c>
       <c r="AE36" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T36),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T36),0,1)</f>
       </c>
       <c r="AF36" s="206" t="n">
-        <f t="shared" si="112">IF(L36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L36=TRUE,1,0)</f>
       </c>
       <c r="AG36" s="206" t="n">
-        <f t="shared" si="113">IF(M36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M36=TRUE,1,0)</f>
       </c>
       <c r="AH36" s="206" t="n">
-        <f t="shared" si="114">IF(N36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N36=TRUE,1,0)</f>
       </c>
       <c r="AI36" s="206" t="n">
-        <f t="shared" si="115">IF(O36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O36=TRUE,1,0)</f>
       </c>
       <c r="AJ36" s="206" t="n">
-        <f t="shared" si="116">IF(P36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P36=TRUE,1,0)</f>
       </c>
       <c r="AK36" s="206" t="n">
-        <f t="shared" si="117">IF(Q36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q36=TRUE,1,0)</f>
       </c>
       <c r="AL36" s="206" t="n">
-        <f t="shared" si="118">IF(R36=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R36=TRUE,1,0)</f>
       </c>
       <c r="AM36" t="n">
         <f>IF(LEN(TRIM(W36))&gt;0,1,0)</f>
@@ -35295,50 +34722,43 @@
         <f>IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
       </c>
       <c r="J37" s="220" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J10),"",'ONR 5'!J10)</f>
+        <f>IF(ISBLANK('ONR 5'!J10),"",'ONR 5'!J10)</f>
       </c>
       <c r="K37" s="233" t="str">
-        <f t="shared" ref="K37:K38" si="105">IF(ISBLANK('ONR 5'!K10),"",'ONR 5'!K10)</f>
+        <f>IF(ISBLANK('ONR 5'!K10),"",'ONR 5'!K10)</f>
       </c>
       <c r="L37" s="233" t="b">
-        <f t="shared" si="119">IF(ISBLANK('ONR 5'!L10),"",'ONR 5'!L10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L10),"",'ONR 5'!L10)</f>
       </c>
       <c r="M37" s="233" t="b">
-        <f t="shared" si="120">IF(ISBLANK('ONR 5'!M10),"",'ONR 5'!M10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M10),"",'ONR 5'!M10)</f>
       </c>
       <c r="N37" s="233" t="b">
-        <f t="shared" si="121">IF(ISBLANK('ONR 5'!N10),"",'ONR 5'!N10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N10),"",'ONR 5'!N10)</f>
       </c>
       <c r="O37" s="233" t="b">
-        <f t="shared" si="122">IF(ISBLANK('ONR 5'!O10),"",'ONR 5'!O10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O10),"",'ONR 5'!O10)</f>
       </c>
       <c r="P37" s="233" t="b">
-        <f t="shared" si="123">IF(ISBLANK('ONR 5'!P10),"",'ONR 5'!P10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P10),"",'ONR 5'!P10)</f>
       </c>
       <c r="Q37" s="233" t="b">
-        <f t="shared" si="124">IF(ISBLANK('ONR 5'!Q10),"",'ONR 5'!Q10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q10),"",'ONR 5'!Q10)</f>
       </c>
       <c r="R37" s="233" t="b">
-        <f t="shared" si="125">IF(ISBLANK('ONR 5'!R10),"",'ONR 5'!R10)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R10),"",'ONR 5'!R10)</f>
       </c>
       <c r="S37" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S10),"",'ONR 5'!S10)</f>
+        <f>IF(ISBLANK('ONR 5'!S10),"",'ONR 5'!S10)</f>
       </c>
       <c r="T37" s="232" t="str">
-        <f t="shared" si="107">IF(ISBLANK('ONR 5'!T10),"",'ONR 5'!T10)</f>
+        <f>IF(ISBLANK('ONR 5'!T10),"",'ONR 5'!T10)</f>
       </c>
       <c r="U37" s="243" t="str">
-        <f t="shared" si="108">IF(ISBLANK('ONR 5'!U10),"",'ONR 5'!U10)</f>
+        <f>IF(ISBLANK('ONR 5'!U10),"",'ONR 5'!U10)</f>
       </c>
       <c r="V37" s="235" t="str">
-        <f t="shared" si="109">IF(ISBLANK('ONR 5'!G10),"",'ONR 5'!G10)</f>
+        <f>IF(ISBLANK('ONR 5'!G10),"",'ONR 5'!G10)</f>
       </c>
       <c r="W37" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V10),"",'ONR 5'!V10)</f>
@@ -35347,42 +34767,34 @@
         <f>IF(ISBLANK('ONR 5'!W10),"",'ONR 5'!W10)</f>
       </c>
       <c r="Y37" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
+        <f>IF(ISBLANK('ONR 5'!I10),"",'ONR 5'!I10)</f>
       </c>
       <c r="Z37" s="256" t="str">
-        <f t="shared" si="126">IF(ISBLANK('ONR 5'!D10),"",'ONR 5'!D10)</f>
+        <f>IF(ISBLANK('ONR 5'!D10),"",'ONR 5'!D10)</f>
       </c>
       <c r="AE37" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T37),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T37),0,1)</f>
       </c>
       <c r="AF37" s="206" t="n">
-        <f t="shared" si="112">IF(L37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L37=TRUE,1,0)</f>
       </c>
       <c r="AG37" s="206" t="n">
-        <f t="shared" si="113">IF(M37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M37=TRUE,1,0)</f>
       </c>
       <c r="AH37" s="206" t="n">
-        <f t="shared" si="114">IF(N37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N37=TRUE,1,0)</f>
       </c>
       <c r="AI37" s="206" t="n">
-        <f t="shared" si="115">IF(O37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O37=TRUE,1,0)</f>
       </c>
       <c r="AJ37" s="206" t="n">
-        <f t="shared" si="116">IF(P37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P37=TRUE,1,0)</f>
       </c>
       <c r="AK37" s="206" t="n">
-        <f t="shared" si="117">IF(Q37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q37=TRUE,1,0)</f>
       </c>
       <c r="AL37" s="206" t="n">
-        <f t="shared" si="118">IF(R37=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R37=TRUE,1,0)</f>
       </c>
       <c r="AM37" t="n">
         <f>IF(LEN(TRIM(W37))&gt;0,1,0)</f>
@@ -35418,50 +34830,43 @@
         <f>IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
       </c>
       <c r="J38" s="219" t="str">
-        <f t="shared" si="84">IF(ISBLANK('ONR 5'!J11),"",'ONR 5'!J11)</f>
+        <f>IF(ISBLANK('ONR 5'!J11),"",'ONR 5'!J11)</f>
       </c>
       <c r="K38" s="233" t="str">
-        <f t="shared" si="105">IF(ISBLANK('ONR 5'!K11),"",'ONR 5'!K11)</f>
+        <f>IF(ISBLANK('ONR 5'!K11),"",'ONR 5'!K11)</f>
       </c>
       <c r="L38" s="233" t="b">
-        <f t="shared" ref="L37:L38" si="119">IF(ISBLANK('ONR 5'!L11),"",'ONR 5'!L11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L11),"",'ONR 5'!L11)</f>
       </c>
       <c r="M38" s="233" t="b">
-        <f t="shared" si="120">IF(ISBLANK('ONR 5'!M11),"",'ONR 5'!M11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M11),"",'ONR 5'!M11)</f>
       </c>
       <c r="N38" s="233" t="b">
-        <f t="shared" si="121">IF(ISBLANK('ONR 5'!N11),"",'ONR 5'!N11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N11),"",'ONR 5'!N11)</f>
       </c>
       <c r="O38" s="233" t="b">
-        <f t="shared" si="122">IF(ISBLANK('ONR 5'!O11),"",'ONR 5'!O11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O11),"",'ONR 5'!O11)</f>
       </c>
       <c r="P38" s="233" t="b">
-        <f t="shared" si="123">IF(ISBLANK('ONR 5'!P11),"",'ONR 5'!P11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P11),"",'ONR 5'!P11)</f>
       </c>
       <c r="Q38" s="233" t="b">
-        <f t="shared" si="124">IF(ISBLANK('ONR 5'!Q11),"",'ONR 5'!Q11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q11),"",'ONR 5'!Q11)</f>
       </c>
       <c r="R38" s="233" t="b">
-        <f t="shared" si="125">IF(ISBLANK('ONR 5'!R11),"",'ONR 5'!R11)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R11),"",'ONR 5'!R11)</f>
       </c>
       <c r="S38" s="234" t="str">
-        <f t="shared" si="106">IF(ISBLANK('ONR 5'!S11),"",'ONR 5'!S11)</f>
+        <f>IF(ISBLANK('ONR 5'!S11),"",'ONR 5'!S11)</f>
       </c>
       <c r="T38" s="232" t="str">
-        <f t="shared" si="107">IF(ISBLANK('ONR 5'!T11),"",'ONR 5'!T11)</f>
+        <f>IF(ISBLANK('ONR 5'!T11),"",'ONR 5'!T11)</f>
       </c>
       <c r="U38" s="243" t="str">
-        <f t="shared" si="108">IF(ISBLANK('ONR 5'!U11),"",'ONR 5'!U11)</f>
+        <f>IF(ISBLANK('ONR 5'!U11),"",'ONR 5'!U11)</f>
       </c>
       <c r="V38" s="235" t="str">
-        <f t="shared" si="109">IF(ISBLANK('ONR 5'!G11),"",'ONR 5'!G11)</f>
+        <f>IF(ISBLANK('ONR 5'!G11),"",'ONR 5'!G11)</f>
       </c>
       <c r="W38" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V11),"",'ONR 5'!V11)</f>
@@ -35470,42 +34875,34 @@
         <f>IF(ISBLANK('ONR 5'!W11),"",'ONR 5'!W11)</f>
       </c>
       <c r="Y38" s="258" t="str">
-        <f t="shared" si="110">IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
+        <f>IF(ISBLANK('ONR 5'!I11),"",'ONR 5'!I11)</f>
       </c>
       <c r="Z38" s="236" t="str">
-        <f t="shared" ref="Z36:Z38" si="126">IF(ISBLANK('ONR 5'!D11),"",'ONR 5'!D11)</f>
+        <f>IF(ISBLANK('ONR 5'!D11),"",'ONR 5'!D11)</f>
       </c>
       <c r="AE38" s="206" t="n">
-        <f t="shared" si="111">IF(ISNUMBER(T38),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T38),0,1)</f>
       </c>
       <c r="AF38" s="206" t="n">
-        <f t="shared" si="112">IF(L38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L38=TRUE,1,0)</f>
       </c>
       <c r="AG38" s="206" t="n">
-        <f t="shared" si="113">IF(M38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M38=TRUE,1,0)</f>
       </c>
       <c r="AH38" s="206" t="n">
-        <f t="shared" si="114">IF(N38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N38=TRUE,1,0)</f>
       </c>
       <c r="AI38" s="206" t="n">
-        <f t="shared" si="115">IF(O38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O38=TRUE,1,0)</f>
       </c>
       <c r="AJ38" s="206" t="n">
-        <f t="shared" si="116">IF(P38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P38=TRUE,1,0)</f>
       </c>
       <c r="AK38" s="206" t="n">
-        <f t="shared" si="117">IF(Q38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q38=TRUE,1,0)</f>
       </c>
       <c r="AL38" s="206" t="n">
-        <f t="shared" si="118">IF(R38=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R38=TRUE,1,0)</f>
       </c>
       <c r="AM38" t="n">
         <f>IF(LEN(TRIM(W38))&gt;0,1,0)</f>
@@ -35540,50 +34937,43 @@
         <f>IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
       </c>
       <c r="J39" s="219" t="str">
-        <f t="shared" ref="J39" si="127">IF(ISBLANK('ONR 5'!J12),"",'ONR 5'!J12)</f>
+        <f>IF(ISBLANK('ONR 5'!J12),"",'ONR 5'!J12)</f>
       </c>
       <c r="K39" s="233" t="str">
-        <f t="shared" ref="K39" si="128">IF(ISBLANK('ONR 5'!K12),"",'ONR 5'!K12)</f>
+        <f>IF(ISBLANK('ONR 5'!K12),"",'ONR 5'!K12)</f>
       </c>
       <c r="L39" s="233" t="b">
-        <f t="shared" ref="L39" si="129">IF(ISBLANK('ONR 5'!L12),"",'ONR 5'!L12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!L12),"",'ONR 5'!L12)</f>
       </c>
       <c r="M39" s="233" t="b">
-        <f t="shared" ref="M39" si="130">IF(ISBLANK('ONR 5'!M12),"",'ONR 5'!M12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!M12),"",'ONR 5'!M12)</f>
       </c>
       <c r="N39" s="233" t="b">
-        <f t="shared" ref="N39" si="131">IF(ISBLANK('ONR 5'!N12),"",'ONR 5'!N12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!N12),"",'ONR 5'!N12)</f>
       </c>
       <c r="O39" s="233" t="b">
-        <f t="shared" ref="O39" si="132">IF(ISBLANK('ONR 5'!O12),"",'ONR 5'!O12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!O12),"",'ONR 5'!O12)</f>
       </c>
       <c r="P39" s="233" t="b">
-        <f t="shared" ref="P39" si="133">IF(ISBLANK('ONR 5'!P12),"",'ONR 5'!P12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!P12),"",'ONR 5'!P12)</f>
       </c>
       <c r="Q39" s="233" t="b">
-        <f t="shared" ref="Q39" si="134">IF(ISBLANK('ONR 5'!Q12),"",'ONR 5'!Q12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!Q12),"",'ONR 5'!Q12)</f>
       </c>
       <c r="R39" s="233" t="b">
-        <f t="shared" ref="R39" si="135">IF(ISBLANK('ONR 5'!R12),"",'ONR 5'!R12)</f>
-        <v>0</v>
+        <f>IF(ISBLANK('ONR 5'!R12),"",'ONR 5'!R12)</f>
       </c>
       <c r="S39" s="234" t="str">
-        <f t="shared" ref="S39" si="136">IF(ISBLANK('ONR 5'!S12),"",'ONR 5'!S12)</f>
+        <f>IF(ISBLANK('ONR 5'!S12),"",'ONR 5'!S12)</f>
       </c>
       <c r="T39" s="232" t="str">
-        <f t="shared" ref="T39" si="137">IF(ISBLANK('ONR 5'!T12),"",'ONR 5'!T12)</f>
+        <f>IF(ISBLANK('ONR 5'!T12),"",'ONR 5'!T12)</f>
       </c>
       <c r="U39" s="243" t="str">
-        <f t="shared" ref="U39" si="138">IF(ISBLANK('ONR 5'!U12),"",'ONR 5'!U12)</f>
+        <f>IF(ISBLANK('ONR 5'!U12),"",'ONR 5'!U12)</f>
       </c>
       <c r="V39" s="235" t="str">
-        <f t="shared" ref="V39" si="139">IF(ISBLANK('ONR 5'!G12),"",'ONR 5'!G12)</f>
+        <f>IF(ISBLANK('ONR 5'!G12),"",'ONR 5'!G12)</f>
       </c>
       <c r="W39" s="142" t="str">
         <f>IF(ISBLANK('ONR 5'!V12),"",'ONR 5'!V12)</f>
@@ -35592,42 +34982,34 @@
         <f>IF(ISBLANK('ONR 5'!W12),"",'ONR 5'!W12)</f>
       </c>
       <c r="Y39" s="258" t="str">
-        <f t="shared" ref="Y39" si="140">IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
+        <f>IF(ISBLANK('ONR 5'!I12),"",'ONR 5'!I12)</f>
       </c>
       <c r="Z39" s="236" t="str">
-        <f t="shared" ref="Z39" si="141">IF(ISBLANK('ONR 5'!D12),"",'ONR 5'!D12)</f>
+        <f>IF(ISBLANK('ONR 5'!D12),"",'ONR 5'!D12)</f>
       </c>
       <c r="AE39" s="206" t="n">
-        <f t="shared" ref="AE39" si="142">IF(ISNUMBER(T39),0,1)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(T39),0,1)</f>
       </c>
       <c r="AF39" s="206" t="n">
-        <f t="shared" ref="AF39" si="143">IF(L39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(L39=TRUE,1,0)</f>
       </c>
       <c r="AG39" s="206" t="n">
-        <f t="shared" ref="AG39" si="144">IF(M39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(M39=TRUE,1,0)</f>
       </c>
       <c r="AH39" s="206" t="n">
-        <f t="shared" ref="AH39" si="145">IF(N39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(N39=TRUE,1,0)</f>
       </c>
       <c r="AI39" s="206" t="n">
-        <f t="shared" ref="AI39" si="146">IF(O39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(O39=TRUE,1,0)</f>
       </c>
       <c r="AJ39" s="206" t="n">
-        <f t="shared" ref="AJ39" si="147">IF(P39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(P39=TRUE,1,0)</f>
       </c>
       <c r="AK39" s="206" t="n">
-        <f t="shared" ref="AK39" si="148">IF(Q39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(Q39=TRUE,1,0)</f>
       </c>
       <c r="AL39" s="206" t="n">
-        <f t="shared" ref="AL39" si="149">IF(R39=TRUE,1,0)</f>
-        <v>0</v>
+        <f>IF(R39=TRUE,1,0)</f>
       </c>
       <c r="AM39" t="n">
         <f>IF(LEN(TRIM(W39))&gt;0,1,0)</f>

</xml_diff>